<commit_message>
Update project configuration and enhance user management features
</commit_message>
<xml_diff>
--- a/src/assets/excel/report.xlsx
+++ b/src/assets/excel/report.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20409"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF20948-6138-497C-A548-2CD302D51A1E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEEADF01-824D-4BCA-942C-660C87189E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4890" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="4" r:id="rId1"/>
@@ -122,9 +122,6 @@
     <t>Requestor</t>
   </si>
   <si>
-    <t>PE</t>
-  </si>
-  <si>
     <t>AE</t>
   </si>
   <si>
@@ -146,27 +143,7 @@
     <t>TE</t>
   </si>
   <si>
-    <t>Mr.Rho S.
-Ms.Sirinthip K.</t>
-  </si>
-  <si>
-    <t>Ms. Pronpimon J.</t>
-  </si>
-  <si>
     <t>Mr.Chadin K.</t>
-  </si>
-  <si>
-    <t>Ms.Sirintip P.</t>
-  </si>
-  <si>
-    <t>Mrs. Rujirek R.</t>
-  </si>
-  <si>
-    <t>Ms.Jarussri W.</t>
-  </si>
-  <si>
-    <t>Mrs. Wanna H,
-Mr.Kinugasa H.</t>
   </si>
   <si>
     <t>Mr.Somchat T.</t>
@@ -348,6 +325,31 @@
   </si>
   <si>
     <t xml:space="preserve"> -</t>
+  </si>
+  <si>
+    <t>IMP</t>
+  </si>
+  <si>
+    <t>Ms.Pronpimon J.</t>
+  </si>
+  <si>
+    <t>Ms.Vasana S.
+Ms.Kesinee T.
+Ms.Sirintip K.</t>
+  </si>
+  <si>
+    <t>Ms.Pornpailin K.</t>
+  </si>
+  <si>
+    <t>Ms.Tipakorn S.</t>
+  </si>
+  <si>
+    <t>Ms.Somruetai T.</t>
+  </si>
+  <si>
+    <t>Ms.Khachinrat D.
+Ms.Sumitra S.
+Mr.Watcharapan P.</t>
   </si>
 </sst>
 </file>
@@ -1593,6 +1595,132 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="16" fontId="23" fillId="2" borderId="23" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1610,212 +1738,251 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="11" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="11" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1840,171 +2007,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="11" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="11" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2109,9 +2111,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2149,7 +2151,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2255,7 +2257,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2397,7 +2399,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2439,9 +2441,9 @@
       <c r="AB1" s="89"/>
     </row>
     <row r="2" spans="1:28" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="148"/>
-      <c r="B2" s="149"/>
-      <c r="C2" s="149"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="151"/>
+      <c r="C2" s="151"/>
       <c r="D2" s="91"/>
       <c r="E2" s="91"/>
       <c r="F2" s="91"/>
@@ -2450,12 +2452,12 @@
       <c r="I2" s="91"/>
       <c r="J2" s="91"/>
       <c r="K2" s="91"/>
-      <c r="L2" s="149"/>
-      <c r="M2" s="149"/>
-      <c r="N2" s="149"/>
-      <c r="O2" s="149"/>
-      <c r="P2" s="149"/>
-      <c r="Q2" s="149"/>
+      <c r="L2" s="151"/>
+      <c r="M2" s="151"/>
+      <c r="N2" s="151"/>
+      <c r="O2" s="151"/>
+      <c r="P2" s="151"/>
+      <c r="Q2" s="151"/>
       <c r="R2" s="90"/>
       <c r="S2" s="90"/>
       <c r="T2" s="90"/>
@@ -2469,9 +2471,9 @@
       <c r="AB2" s="92"/>
     </row>
     <row r="3" spans="1:28" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="150"/>
-      <c r="B3" s="151"/>
-      <c r="C3" s="151"/>
+      <c r="A3" s="153"/>
+      <c r="B3" s="154"/>
+      <c r="C3" s="154"/>
       <c r="D3" s="93"/>
       <c r="E3" s="93"/>
       <c r="F3" s="94"/>
@@ -2480,12 +2482,12 @@
       <c r="I3" s="94"/>
       <c r="J3" s="94"/>
       <c r="K3" s="94"/>
-      <c r="L3" s="153"/>
-      <c r="M3" s="153"/>
-      <c r="N3" s="153"/>
-      <c r="O3" s="153"/>
-      <c r="P3" s="153"/>
-      <c r="Q3" s="153"/>
+      <c r="L3" s="157"/>
+      <c r="M3" s="157"/>
+      <c r="N3" s="157"/>
+      <c r="O3" s="157"/>
+      <c r="P3" s="157"/>
+      <c r="Q3" s="157"/>
       <c r="R3" s="95"/>
       <c r="S3" s="95"/>
       <c r="T3" s="95"/>
@@ -2495,93 +2497,93 @@
       <c r="AB3" s="96"/>
     </row>
     <row r="4" spans="1:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="150"/>
-      <c r="B4" s="151"/>
-      <c r="C4" s="151"/>
+      <c r="A4" s="153"/>
+      <c r="B4" s="154"/>
+      <c r="C4" s="154"/>
       <c r="E4" s="97"/>
-      <c r="F4" s="149" t="s">
+      <c r="F4" s="151" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="149"/>
-      <c r="H4" s="149"/>
-      <c r="I4" s="149"/>
-      <c r="J4" s="149"/>
-      <c r="K4" s="149"/>
-      <c r="L4" s="149"/>
-      <c r="M4" s="149"/>
-      <c r="N4" s="149"/>
-      <c r="O4" s="149"/>
-      <c r="P4" s="149"/>
-      <c r="Q4" s="149"/>
-      <c r="R4" s="149"/>
-      <c r="S4" s="149"/>
-      <c r="T4" s="149"/>
-      <c r="U4" s="149"/>
-      <c r="V4" s="149"/>
-      <c r="W4" s="149"/>
+      <c r="G4" s="151"/>
+      <c r="H4" s="151"/>
+      <c r="I4" s="151"/>
+      <c r="J4" s="151"/>
+      <c r="K4" s="151"/>
+      <c r="L4" s="151"/>
+      <c r="M4" s="151"/>
+      <c r="N4" s="151"/>
+      <c r="O4" s="151"/>
+      <c r="P4" s="151"/>
+      <c r="Q4" s="151"/>
+      <c r="R4" s="151"/>
+      <c r="S4" s="151"/>
+      <c r="T4" s="151"/>
+      <c r="U4" s="151"/>
+      <c r="V4" s="151"/>
+      <c r="W4" s="151"/>
       <c r="AB4" s="96"/>
     </row>
     <row r="5" spans="1:28" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="152"/>
-      <c r="B5" s="153"/>
-      <c r="C5" s="153"/>
-      <c r="D5" s="154"/>
-      <c r="E5" s="154"/>
-      <c r="F5" s="154"/>
-      <c r="G5" s="154"/>
-      <c r="H5" s="154"/>
-      <c r="I5" s="154"/>
-      <c r="J5" s="154"/>
-      <c r="K5" s="154"/>
-      <c r="L5" s="154"/>
-      <c r="M5" s="154"/>
-      <c r="N5" s="154"/>
-      <c r="O5" s="154"/>
-      <c r="P5" s="154"/>
-      <c r="Q5" s="154"/>
-      <c r="R5" s="154"/>
-      <c r="S5" s="154"/>
-      <c r="T5" s="154"/>
-      <c r="U5" s="154"/>
-      <c r="V5" s="154"/>
-      <c r="W5" s="154"/>
-      <c r="X5" s="154"/>
-      <c r="Y5" s="154"/>
-      <c r="Z5" s="154"/>
-      <c r="AA5" s="154"/>
-      <c r="AB5" s="155"/>
+      <c r="A5" s="156"/>
+      <c r="B5" s="157"/>
+      <c r="C5" s="157"/>
+      <c r="D5" s="206"/>
+      <c r="E5" s="206"/>
+      <c r="F5" s="206"/>
+      <c r="G5" s="206"/>
+      <c r="H5" s="206"/>
+      <c r="I5" s="206"/>
+      <c r="J5" s="206"/>
+      <c r="K5" s="206"/>
+      <c r="L5" s="206"/>
+      <c r="M5" s="206"/>
+      <c r="N5" s="206"/>
+      <c r="O5" s="206"/>
+      <c r="P5" s="206"/>
+      <c r="Q5" s="206"/>
+      <c r="R5" s="206"/>
+      <c r="S5" s="206"/>
+      <c r="T5" s="206"/>
+      <c r="U5" s="206"/>
+      <c r="V5" s="206"/>
+      <c r="W5" s="206"/>
+      <c r="X5" s="206"/>
+      <c r="Y5" s="206"/>
+      <c r="Z5" s="206"/>
+      <c r="AA5" s="206"/>
+      <c r="AB5" s="207"/>
     </row>
     <row r="6" spans="1:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="156" t="s">
+      <c r="A6" s="208" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="157"/>
-      <c r="C6" s="157"/>
-      <c r="D6" s="157"/>
-      <c r="E6" s="157"/>
-      <c r="F6" s="157"/>
-      <c r="G6" s="158"/>
-      <c r="H6" s="157"/>
-      <c r="I6" s="157"/>
-      <c r="J6" s="157"/>
-      <c r="K6" s="157"/>
-      <c r="L6" s="157"/>
-      <c r="M6" s="157"/>
-      <c r="N6" s="157"/>
-      <c r="O6" s="157"/>
-      <c r="P6" s="157"/>
-      <c r="Q6" s="157"/>
-      <c r="R6" s="157"/>
-      <c r="S6" s="157"/>
-      <c r="T6" s="157"/>
-      <c r="U6" s="157"/>
-      <c r="V6" s="157"/>
-      <c r="W6" s="157"/>
-      <c r="X6" s="157"/>
-      <c r="Y6" s="157"/>
-      <c r="Z6" s="157"/>
-      <c r="AA6" s="157"/>
-      <c r="AB6" s="159"/>
+      <c r="B6" s="209"/>
+      <c r="C6" s="209"/>
+      <c r="D6" s="209"/>
+      <c r="E6" s="209"/>
+      <c r="F6" s="209"/>
+      <c r="G6" s="210"/>
+      <c r="H6" s="209"/>
+      <c r="I6" s="209"/>
+      <c r="J6" s="209"/>
+      <c r="K6" s="209"/>
+      <c r="L6" s="209"/>
+      <c r="M6" s="209"/>
+      <c r="N6" s="209"/>
+      <c r="O6" s="209"/>
+      <c r="P6" s="209"/>
+      <c r="Q6" s="209"/>
+      <c r="R6" s="209"/>
+      <c r="S6" s="209"/>
+      <c r="T6" s="209"/>
+      <c r="U6" s="209"/>
+      <c r="V6" s="209"/>
+      <c r="W6" s="209"/>
+      <c r="X6" s="209"/>
+      <c r="Y6" s="209"/>
+      <c r="Z6" s="209"/>
+      <c r="AA6" s="209"/>
+      <c r="AB6" s="211"/>
     </row>
     <row r="7" spans="1:28" ht="6.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="99"/>
@@ -3241,97 +3243,97 @@
     </row>
     <row r="33" spans="1:28" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="105"/>
-      <c r="B33" s="164" t="s">
+      <c r="B33" s="187" t="s">
         <v>17</v>
       </c>
-      <c r="C33" s="165"/>
-      <c r="D33" s="170" t="s">
+      <c r="C33" s="188"/>
+      <c r="D33" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="E33" s="171"/>
-      <c r="F33" s="171"/>
-      <c r="G33" s="171"/>
-      <c r="H33" s="171"/>
-      <c r="I33" s="171"/>
-      <c r="J33" s="171"/>
-      <c r="K33" s="172"/>
-      <c r="L33" s="170" t="s">
+      <c r="E33" s="194"/>
+      <c r="F33" s="194"/>
+      <c r="G33" s="194"/>
+      <c r="H33" s="194"/>
+      <c r="I33" s="194"/>
+      <c r="J33" s="194"/>
+      <c r="K33" s="195"/>
+      <c r="L33" s="193" t="s">
         <v>19</v>
       </c>
-      <c r="M33" s="171"/>
-      <c r="N33" s="172"/>
-      <c r="O33" s="160" t="s">
+      <c r="M33" s="194"/>
+      <c r="N33" s="195"/>
+      <c r="O33" s="202" t="s">
         <v>20</v>
       </c>
-      <c r="P33" s="161"/>
-      <c r="Q33" s="161"/>
-      <c r="R33" s="161"/>
-      <c r="S33" s="161"/>
-      <c r="T33" s="161"/>
-      <c r="U33" s="161"/>
-      <c r="V33" s="162"/>
-      <c r="W33" s="163" t="s">
+      <c r="P33" s="203"/>
+      <c r="Q33" s="203"/>
+      <c r="R33" s="203"/>
+      <c r="S33" s="203"/>
+      <c r="T33" s="203"/>
+      <c r="U33" s="203"/>
+      <c r="V33" s="204"/>
+      <c r="W33" s="205" t="s">
         <v>21</v>
       </c>
-      <c r="X33" s="163"/>
-      <c r="Y33" s="163"/>
-      <c r="Z33" s="163"/>
+      <c r="X33" s="205"/>
+      <c r="Y33" s="205"/>
+      <c r="Z33" s="205"/>
       <c r="AA33" s="106"/>
       <c r="AB33" s="96"/>
     </row>
     <row r="34" spans="1:28" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="105"/>
-      <c r="B34" s="166"/>
-      <c r="C34" s="167"/>
-      <c r="D34" s="173"/>
-      <c r="E34" s="174"/>
-      <c r="F34" s="174"/>
-      <c r="G34" s="174"/>
-      <c r="H34" s="174"/>
-      <c r="I34" s="174"/>
-      <c r="J34" s="174"/>
-      <c r="K34" s="175"/>
-      <c r="L34" s="173"/>
-      <c r="M34" s="174"/>
-      <c r="N34" s="175"/>
-      <c r="O34" s="160" t="s">
+      <c r="B34" s="189"/>
+      <c r="C34" s="190"/>
+      <c r="D34" s="196"/>
+      <c r="E34" s="197"/>
+      <c r="F34" s="197"/>
+      <c r="G34" s="197"/>
+      <c r="H34" s="197"/>
+      <c r="I34" s="197"/>
+      <c r="J34" s="197"/>
+      <c r="K34" s="198"/>
+      <c r="L34" s="196"/>
+      <c r="M34" s="197"/>
+      <c r="N34" s="198"/>
+      <c r="O34" s="202" t="s">
         <v>22</v>
       </c>
-      <c r="P34" s="162"/>
-      <c r="Q34" s="160" t="s">
+      <c r="P34" s="204"/>
+      <c r="Q34" s="202" t="s">
         <v>23</v>
       </c>
-      <c r="R34" s="162"/>
-      <c r="S34" s="160" t="s">
+      <c r="R34" s="204"/>
+      <c r="S34" s="202" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="162"/>
-      <c r="U34" s="160" t="s">
+      <c r="T34" s="204"/>
+      <c r="U34" s="202" t="s">
         <v>25</v>
       </c>
-      <c r="V34" s="162"/>
-      <c r="W34" s="163"/>
-      <c r="X34" s="163"/>
-      <c r="Y34" s="163"/>
-      <c r="Z34" s="163"/>
+      <c r="V34" s="204"/>
+      <c r="W34" s="205"/>
+      <c r="X34" s="205"/>
+      <c r="Y34" s="205"/>
+      <c r="Z34" s="205"/>
       <c r="AA34" s="106"/>
       <c r="AB34" s="96"/>
     </row>
     <row r="35" spans="1:28" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="105"/>
-      <c r="B35" s="168"/>
-      <c r="C35" s="169"/>
-      <c r="D35" s="176"/>
-      <c r="E35" s="177"/>
-      <c r="F35" s="177"/>
-      <c r="G35" s="177"/>
-      <c r="H35" s="177"/>
-      <c r="I35" s="177"/>
-      <c r="J35" s="177"/>
-      <c r="K35" s="178"/>
-      <c r="L35" s="176"/>
-      <c r="M35" s="177"/>
-      <c r="N35" s="178"/>
+      <c r="B35" s="191"/>
+      <c r="C35" s="192"/>
+      <c r="D35" s="199"/>
+      <c r="E35" s="200"/>
+      <c r="F35" s="200"/>
+      <c r="G35" s="200"/>
+      <c r="H35" s="200"/>
+      <c r="I35" s="200"/>
+      <c r="J35" s="200"/>
+      <c r="K35" s="201"/>
+      <c r="L35" s="199"/>
+      <c r="M35" s="200"/>
+      <c r="N35" s="201"/>
       <c r="O35" s="137" t="s">
         <v>26</v>
       </c>
@@ -3356,34 +3358,34 @@
       <c r="V35" s="139" t="s">
         <v>27</v>
       </c>
-      <c r="W35" s="163"/>
-      <c r="X35" s="163"/>
-      <c r="Y35" s="163"/>
-      <c r="Z35" s="163"/>
+      <c r="W35" s="205"/>
+      <c r="X35" s="205"/>
+      <c r="Y35" s="205"/>
+      <c r="Z35" s="205"/>
       <c r="AA35" s="106"/>
       <c r="AB35" s="96"/>
     </row>
     <row r="36" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="105"/>
-      <c r="B36" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C36" s="141"/>
-      <c r="D36" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E36" s="143"/>
-      <c r="F36" s="143"/>
-      <c r="G36" s="143"/>
-      <c r="H36" s="143"/>
-      <c r="I36" s="143"/>
-      <c r="J36" s="143"/>
-      <c r="K36" s="144"/>
-      <c r="L36" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M36" s="143"/>
-      <c r="N36" s="144"/>
+      <c r="B36" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" s="183"/>
+      <c r="D36" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E36" s="185"/>
+      <c r="F36" s="185"/>
+      <c r="G36" s="185"/>
+      <c r="H36" s="185"/>
+      <c r="I36" s="185"/>
+      <c r="J36" s="185"/>
+      <c r="K36" s="186"/>
+      <c r="L36" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M36" s="185"/>
+      <c r="N36" s="186"/>
       <c r="O36" s="136">
         <v>1</v>
       </c>
@@ -3408,36 +3410,36 @@
       <c r="V36" s="136">
         <v>8</v>
       </c>
-      <c r="W36" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X36" s="146"/>
-      <c r="Y36" s="146"/>
-      <c r="Z36" s="147"/>
+      <c r="W36" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X36" s="180"/>
+      <c r="Y36" s="180"/>
+      <c r="Z36" s="181"/>
       <c r="AA36" s="88"/>
       <c r="AB36" s="96"/>
     </row>
     <row r="37" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="105"/>
-      <c r="B37" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C37" s="141"/>
-      <c r="D37" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E37" s="143"/>
-      <c r="F37" s="143"/>
-      <c r="G37" s="143"/>
-      <c r="H37" s="143"/>
-      <c r="I37" s="143"/>
-      <c r="J37" s="143"/>
-      <c r="K37" s="144"/>
-      <c r="L37" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M37" s="143"/>
-      <c r="N37" s="144"/>
+      <c r="B37" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C37" s="183"/>
+      <c r="D37" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E37" s="185"/>
+      <c r="F37" s="185"/>
+      <c r="G37" s="185"/>
+      <c r="H37" s="185"/>
+      <c r="I37" s="185"/>
+      <c r="J37" s="185"/>
+      <c r="K37" s="186"/>
+      <c r="L37" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M37" s="185"/>
+      <c r="N37" s="186"/>
       <c r="O37" s="136">
         <v>1</v>
       </c>
@@ -3462,36 +3464,36 @@
       <c r="V37" s="136">
         <v>8</v>
       </c>
-      <c r="W37" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X37" s="146"/>
-      <c r="Y37" s="146"/>
-      <c r="Z37" s="147"/>
+      <c r="W37" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X37" s="180"/>
+      <c r="Y37" s="180"/>
+      <c r="Z37" s="181"/>
       <c r="AA37" s="88"/>
       <c r="AB37" s="96"/>
     </row>
     <row r="38" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="105"/>
-      <c r="B38" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C38" s="141"/>
-      <c r="D38" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E38" s="143"/>
-      <c r="F38" s="143"/>
-      <c r="G38" s="143"/>
-      <c r="H38" s="143"/>
-      <c r="I38" s="143"/>
-      <c r="J38" s="143"/>
-      <c r="K38" s="144"/>
-      <c r="L38" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M38" s="143"/>
-      <c r="N38" s="144"/>
+      <c r="B38" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C38" s="183"/>
+      <c r="D38" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38" s="185"/>
+      <c r="F38" s="185"/>
+      <c r="G38" s="185"/>
+      <c r="H38" s="185"/>
+      <c r="I38" s="185"/>
+      <c r="J38" s="185"/>
+      <c r="K38" s="186"/>
+      <c r="L38" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M38" s="185"/>
+      <c r="N38" s="186"/>
       <c r="O38" s="136">
         <v>1</v>
       </c>
@@ -3516,35 +3518,35 @@
       <c r="V38" s="136">
         <v>8</v>
       </c>
-      <c r="W38" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X38" s="146"/>
-      <c r="Y38" s="146"/>
-      <c r="Z38" s="147"/>
+      <c r="W38" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X38" s="180"/>
+      <c r="Y38" s="180"/>
+      <c r="Z38" s="181"/>
       <c r="AA38" s="88"/>
       <c r="AB38" s="96"/>
     </row>
     <row r="39" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C39" s="141"/>
-      <c r="D39" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E39" s="143"/>
-      <c r="F39" s="143"/>
-      <c r="G39" s="143"/>
-      <c r="H39" s="143"/>
-      <c r="I39" s="143"/>
-      <c r="J39" s="143"/>
-      <c r="K39" s="144"/>
-      <c r="L39" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M39" s="143"/>
-      <c r="N39" s="144"/>
+      <c r="B39" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C39" s="183"/>
+      <c r="D39" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E39" s="185"/>
+      <c r="F39" s="185"/>
+      <c r="G39" s="185"/>
+      <c r="H39" s="185"/>
+      <c r="I39" s="185"/>
+      <c r="J39" s="185"/>
+      <c r="K39" s="186"/>
+      <c r="L39" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M39" s="185"/>
+      <c r="N39" s="186"/>
       <c r="O39" s="136">
         <v>1</v>
       </c>
@@ -3569,33 +3571,33 @@
       <c r="V39" s="136">
         <v>8</v>
       </c>
-      <c r="W39" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X39" s="146"/>
-      <c r="Y39" s="146"/>
-      <c r="Z39" s="147"/>
+      <c r="W39" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X39" s="180"/>
+      <c r="Y39" s="180"/>
+      <c r="Z39" s="181"/>
     </row>
     <row r="40" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C40" s="141"/>
-      <c r="D40" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E40" s="143"/>
-      <c r="F40" s="143"/>
-      <c r="G40" s="143"/>
-      <c r="H40" s="143"/>
-      <c r="I40" s="143"/>
-      <c r="J40" s="143"/>
-      <c r="K40" s="144"/>
-      <c r="L40" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M40" s="143"/>
-      <c r="N40" s="144"/>
+      <c r="B40" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C40" s="183"/>
+      <c r="D40" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E40" s="185"/>
+      <c r="F40" s="185"/>
+      <c r="G40" s="185"/>
+      <c r="H40" s="185"/>
+      <c r="I40" s="185"/>
+      <c r="J40" s="185"/>
+      <c r="K40" s="186"/>
+      <c r="L40" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M40" s="185"/>
+      <c r="N40" s="186"/>
       <c r="O40" s="136">
         <v>1</v>
       </c>
@@ -3620,33 +3622,33 @@
       <c r="V40" s="136">
         <v>8</v>
       </c>
-      <c r="W40" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X40" s="146"/>
-      <c r="Y40" s="146"/>
-      <c r="Z40" s="147"/>
+      <c r="W40" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X40" s="180"/>
+      <c r="Y40" s="180"/>
+      <c r="Z40" s="181"/>
     </row>
     <row r="41" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C41" s="141"/>
-      <c r="D41" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E41" s="143"/>
-      <c r="F41" s="143"/>
-      <c r="G41" s="143"/>
-      <c r="H41" s="143"/>
-      <c r="I41" s="143"/>
-      <c r="J41" s="143"/>
-      <c r="K41" s="144"/>
-      <c r="L41" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M41" s="143"/>
-      <c r="N41" s="144"/>
+      <c r="B41" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C41" s="183"/>
+      <c r="D41" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41" s="185"/>
+      <c r="F41" s="185"/>
+      <c r="G41" s="185"/>
+      <c r="H41" s="185"/>
+      <c r="I41" s="185"/>
+      <c r="J41" s="185"/>
+      <c r="K41" s="186"/>
+      <c r="L41" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M41" s="185"/>
+      <c r="N41" s="186"/>
       <c r="O41" s="136">
         <v>1</v>
       </c>
@@ -3671,33 +3673,33 @@
       <c r="V41" s="136">
         <v>8</v>
       </c>
-      <c r="W41" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X41" s="146"/>
-      <c r="Y41" s="146"/>
-      <c r="Z41" s="147"/>
+      <c r="W41" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X41" s="180"/>
+      <c r="Y41" s="180"/>
+      <c r="Z41" s="181"/>
     </row>
     <row r="42" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C42" s="141"/>
-      <c r="D42" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E42" s="143"/>
-      <c r="F42" s="143"/>
-      <c r="G42" s="143"/>
-      <c r="H42" s="143"/>
-      <c r="I42" s="143"/>
-      <c r="J42" s="143"/>
-      <c r="K42" s="144"/>
-      <c r="L42" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M42" s="143"/>
-      <c r="N42" s="144"/>
+      <c r="B42" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C42" s="183"/>
+      <c r="D42" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E42" s="185"/>
+      <c r="F42" s="185"/>
+      <c r="G42" s="185"/>
+      <c r="H42" s="185"/>
+      <c r="I42" s="185"/>
+      <c r="J42" s="185"/>
+      <c r="K42" s="186"/>
+      <c r="L42" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M42" s="185"/>
+      <c r="N42" s="186"/>
       <c r="O42" s="136">
         <v>1</v>
       </c>
@@ -3722,33 +3724,33 @@
       <c r="V42" s="136">
         <v>8</v>
       </c>
-      <c r="W42" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X42" s="146"/>
-      <c r="Y42" s="146"/>
-      <c r="Z42" s="147"/>
+      <c r="W42" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X42" s="180"/>
+      <c r="Y42" s="180"/>
+      <c r="Z42" s="181"/>
     </row>
     <row r="43" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C43" s="141"/>
-      <c r="D43" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E43" s="143"/>
-      <c r="F43" s="143"/>
-      <c r="G43" s="143"/>
-      <c r="H43" s="143"/>
-      <c r="I43" s="143"/>
-      <c r="J43" s="143"/>
-      <c r="K43" s="144"/>
-      <c r="L43" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M43" s="143"/>
-      <c r="N43" s="144"/>
+      <c r="B43" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C43" s="183"/>
+      <c r="D43" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E43" s="185"/>
+      <c r="F43" s="185"/>
+      <c r="G43" s="185"/>
+      <c r="H43" s="185"/>
+      <c r="I43" s="185"/>
+      <c r="J43" s="185"/>
+      <c r="K43" s="186"/>
+      <c r="L43" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M43" s="185"/>
+      <c r="N43" s="186"/>
       <c r="O43" s="136">
         <v>1</v>
       </c>
@@ -3773,33 +3775,33 @@
       <c r="V43" s="136">
         <v>8</v>
       </c>
-      <c r="W43" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X43" s="146"/>
-      <c r="Y43" s="146"/>
-      <c r="Z43" s="147"/>
+      <c r="W43" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X43" s="180"/>
+      <c r="Y43" s="180"/>
+      <c r="Z43" s="181"/>
     </row>
     <row r="44" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C44" s="141"/>
-      <c r="D44" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E44" s="143"/>
-      <c r="F44" s="143"/>
-      <c r="G44" s="143"/>
-      <c r="H44" s="143"/>
-      <c r="I44" s="143"/>
-      <c r="J44" s="143"/>
-      <c r="K44" s="144"/>
-      <c r="L44" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M44" s="143"/>
-      <c r="N44" s="144"/>
+      <c r="B44" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C44" s="183"/>
+      <c r="D44" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E44" s="185"/>
+      <c r="F44" s="185"/>
+      <c r="G44" s="185"/>
+      <c r="H44" s="185"/>
+      <c r="I44" s="185"/>
+      <c r="J44" s="185"/>
+      <c r="K44" s="186"/>
+      <c r="L44" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M44" s="185"/>
+      <c r="N44" s="186"/>
       <c r="O44" s="136">
         <v>1</v>
       </c>
@@ -3824,33 +3826,33 @@
       <c r="V44" s="136">
         <v>8</v>
       </c>
-      <c r="W44" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X44" s="146"/>
-      <c r="Y44" s="146"/>
-      <c r="Z44" s="147"/>
+      <c r="W44" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X44" s="180"/>
+      <c r="Y44" s="180"/>
+      <c r="Z44" s="181"/>
     </row>
     <row r="45" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="140" t="s">
-        <v>99</v>
-      </c>
-      <c r="C45" s="141"/>
-      <c r="D45" s="142" t="s">
-        <v>100</v>
-      </c>
-      <c r="E45" s="143"/>
-      <c r="F45" s="143"/>
-      <c r="G45" s="143"/>
-      <c r="H45" s="143"/>
-      <c r="I45" s="143"/>
-      <c r="J45" s="143"/>
-      <c r="K45" s="144"/>
-      <c r="L45" s="142" t="s">
-        <v>101</v>
-      </c>
-      <c r="M45" s="143"/>
-      <c r="N45" s="144"/>
+      <c r="B45" s="182" t="s">
+        <v>92</v>
+      </c>
+      <c r="C45" s="183"/>
+      <c r="D45" s="184" t="s">
+        <v>93</v>
+      </c>
+      <c r="E45" s="185"/>
+      <c r="F45" s="185"/>
+      <c r="G45" s="185"/>
+      <c r="H45" s="185"/>
+      <c r="I45" s="185"/>
+      <c r="J45" s="185"/>
+      <c r="K45" s="186"/>
+      <c r="L45" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="M45" s="185"/>
+      <c r="N45" s="186"/>
       <c r="O45" s="136">
         <v>1</v>
       </c>
@@ -3875,12 +3877,12 @@
       <c r="V45" s="136">
         <v>8</v>
       </c>
-      <c r="W45" s="145" t="s">
-        <v>102</v>
-      </c>
-      <c r="X45" s="146"/>
-      <c r="Y45" s="146"/>
-      <c r="Z45" s="147"/>
+      <c r="W45" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="X45" s="180"/>
+      <c r="Y45" s="180"/>
+      <c r="Z45" s="181"/>
     </row>
     <row r="46" spans="1:28" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="105"/>
@@ -4071,34 +4073,34 @@
       <c r="AB51" s="125"/>
     </row>
     <row r="52" spans="1:32" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="150"/>
-      <c r="B52" s="151"/>
-      <c r="C52" s="151"/>
-      <c r="D52" s="151"/>
-      <c r="E52" s="151"/>
-      <c r="F52" s="151"/>
-      <c r="G52" s="151"/>
-      <c r="H52" s="151"/>
-      <c r="I52" s="151"/>
-      <c r="J52" s="151"/>
-      <c r="K52" s="151"/>
-      <c r="L52" s="151"/>
-      <c r="M52" s="151"/>
-      <c r="N52" s="151"/>
-      <c r="O52" s="151"/>
-      <c r="P52" s="151"/>
-      <c r="Q52" s="151"/>
+      <c r="A52" s="153"/>
+      <c r="B52" s="154"/>
+      <c r="C52" s="154"/>
+      <c r="D52" s="154"/>
+      <c r="E52" s="154"/>
+      <c r="F52" s="154"/>
+      <c r="G52" s="154"/>
+      <c r="H52" s="154"/>
+      <c r="I52" s="154"/>
+      <c r="J52" s="154"/>
+      <c r="K52" s="154"/>
+      <c r="L52" s="154"/>
+      <c r="M52" s="154"/>
+      <c r="N52" s="154"/>
+      <c r="O52" s="154"/>
+      <c r="P52" s="154"/>
+      <c r="Q52" s="154"/>
       <c r="R52" s="88"/>
       <c r="S52" s="88"/>
       <c r="T52" s="88"/>
-      <c r="U52" s="151"/>
-      <c r="V52" s="151"/>
-      <c r="W52" s="151"/>
+      <c r="U52" s="154"/>
+      <c r="V52" s="154"/>
+      <c r="W52" s="154"/>
       <c r="X52" s="88"/>
-      <c r="Y52" s="151"/>
-      <c r="Z52" s="151"/>
-      <c r="AA52" s="151"/>
-      <c r="AB52" s="179"/>
+      <c r="Y52" s="154"/>
+      <c r="Z52" s="154"/>
+      <c r="AA52" s="154"/>
+      <c r="AB52" s="155"/>
     </row>
     <row r="53" spans="1:32" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="105"/>
@@ -4145,162 +4147,162 @@
       <c r="AB54" s="96"/>
     </row>
     <row r="55" spans="1:32" s="119" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="180" t="s">
+      <c r="A55" s="149" t="s">
         <v>31</v>
       </c>
-      <c r="B55" s="180"/>
-      <c r="C55" s="180"/>
-      <c r="D55" s="181" t="s">
+      <c r="B55" s="149"/>
+      <c r="C55" s="149"/>
+      <c r="D55" s="175" t="s">
+        <v>96</v>
+      </c>
+      <c r="E55" s="176"/>
+      <c r="F55" s="176"/>
+      <c r="G55" s="177"/>
+      <c r="H55" s="178" t="s">
         <v>32</v>
       </c>
-      <c r="E55" s="182"/>
-      <c r="F55" s="182"/>
-      <c r="G55" s="183"/>
-      <c r="H55" s="184" t="s">
+      <c r="I55" s="178"/>
+      <c r="J55" s="178"/>
+      <c r="K55" s="175" t="s">
         <v>33</v>
       </c>
-      <c r="I55" s="184"/>
-      <c r="J55" s="184"/>
-      <c r="K55" s="181" t="s">
+      <c r="L55" s="176"/>
+      <c r="M55" s="177"/>
+      <c r="N55" s="178" t="s">
         <v>34</v>
       </c>
-      <c r="L55" s="182"/>
-      <c r="M55" s="183"/>
-      <c r="N55" s="184" t="s">
+      <c r="O55" s="178"/>
+      <c r="P55" s="178"/>
+      <c r="Q55" s="178" t="s">
         <v>35</v>
       </c>
-      <c r="O55" s="184"/>
-      <c r="P55" s="184"/>
-      <c r="Q55" s="184" t="s">
+      <c r="R55" s="178"/>
+      <c r="S55" s="178"/>
+      <c r="T55" s="175" t="s">
         <v>36</v>
       </c>
-      <c r="R55" s="184"/>
-      <c r="S55" s="184"/>
-      <c r="T55" s="181" t="s">
+      <c r="U55" s="176"/>
+      <c r="V55" s="177"/>
+      <c r="W55" s="175" t="s">
         <v>37</v>
       </c>
-      <c r="U55" s="182"/>
-      <c r="V55" s="183"/>
-      <c r="W55" s="181" t="s">
+      <c r="X55" s="176"/>
+      <c r="Y55" s="177"/>
+      <c r="Z55" s="175" t="s">
         <v>38</v>
       </c>
-      <c r="X55" s="182"/>
-      <c r="Y55" s="183"/>
-      <c r="Z55" s="181" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA55" s="182"/>
-      <c r="AB55" s="183"/>
+      <c r="AA55" s="176"/>
+      <c r="AB55" s="177"/>
       <c r="AC55" s="87"/>
       <c r="AF55" s="128"/>
     </row>
     <row r="56" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="185"/>
-      <c r="B56" s="186"/>
-      <c r="C56" s="187"/>
-      <c r="D56" s="194" t="s">
+      <c r="A56" s="166"/>
+      <c r="B56" s="167"/>
+      <c r="C56" s="168"/>
+      <c r="D56" s="140" t="s">
+        <v>98</v>
+      </c>
+      <c r="E56" s="141"/>
+      <c r="F56" s="141"/>
+      <c r="G56" s="142"/>
+      <c r="H56" s="140" t="s">
+        <v>97</v>
+      </c>
+      <c r="I56" s="141"/>
+      <c r="J56" s="142"/>
+      <c r="K56" s="150" t="s">
+        <v>39</v>
+      </c>
+      <c r="L56" s="151"/>
+      <c r="M56" s="152"/>
+      <c r="N56" s="150" t="s">
+        <v>99</v>
+      </c>
+      <c r="O56" s="151"/>
+      <c r="P56" s="152"/>
+      <c r="Q56" s="150" t="s">
+        <v>100</v>
+      </c>
+      <c r="R56" s="151"/>
+      <c r="S56" s="152"/>
+      <c r="T56" s="150" t="s">
+        <v>101</v>
+      </c>
+      <c r="U56" s="151"/>
+      <c r="V56" s="152"/>
+      <c r="W56" s="140" t="s">
+        <v>102</v>
+      </c>
+      <c r="X56" s="141"/>
+      <c r="Y56" s="142"/>
+      <c r="Z56" s="150" t="s">
         <v>40</v>
       </c>
-      <c r="E56" s="195"/>
-      <c r="F56" s="195"/>
-      <c r="G56" s="196"/>
-      <c r="H56" s="194" t="s">
-        <v>41</v>
-      </c>
-      <c r="I56" s="195"/>
-      <c r="J56" s="196"/>
-      <c r="K56" s="148" t="s">
-        <v>42</v>
-      </c>
-      <c r="L56" s="149"/>
-      <c r="M56" s="203"/>
-      <c r="N56" s="148" t="s">
-        <v>43</v>
-      </c>
-      <c r="O56" s="149"/>
-      <c r="P56" s="203"/>
-      <c r="Q56" s="148" t="s">
-        <v>44</v>
-      </c>
-      <c r="R56" s="149"/>
-      <c r="S56" s="203"/>
-      <c r="T56" s="148" t="s">
-        <v>45</v>
-      </c>
-      <c r="U56" s="149"/>
-      <c r="V56" s="203"/>
-      <c r="W56" s="194" t="s">
-        <v>46</v>
-      </c>
-      <c r="X56" s="195"/>
-      <c r="Y56" s="196"/>
-      <c r="Z56" s="148" t="s">
-        <v>47</v>
-      </c>
-      <c r="AA56" s="149"/>
-      <c r="AB56" s="203"/>
+      <c r="AA56" s="151"/>
+      <c r="AB56" s="152"/>
       <c r="AF56" s="128"/>
     </row>
     <row r="57" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="188"/>
-      <c r="B57" s="189"/>
-      <c r="C57" s="190"/>
-      <c r="D57" s="197"/>
-      <c r="E57" s="198"/>
-      <c r="F57" s="198"/>
-      <c r="G57" s="199"/>
-      <c r="H57" s="197"/>
-      <c r="I57" s="198"/>
-      <c r="J57" s="199"/>
-      <c r="K57" s="150"/>
-      <c r="L57" s="151"/>
-      <c r="M57" s="179"/>
-      <c r="N57" s="150"/>
-      <c r="O57" s="151"/>
-      <c r="P57" s="179"/>
-      <c r="Q57" s="150"/>
-      <c r="R57" s="151"/>
-      <c r="S57" s="179"/>
-      <c r="T57" s="150"/>
-      <c r="U57" s="151"/>
-      <c r="V57" s="179"/>
-      <c r="W57" s="197"/>
-      <c r="X57" s="198"/>
-      <c r="Y57" s="199"/>
-      <c r="Z57" s="150"/>
-      <c r="AA57" s="151"/>
-      <c r="AB57" s="179"/>
+      <c r="A57" s="169"/>
+      <c r="B57" s="170"/>
+      <c r="C57" s="171"/>
+      <c r="D57" s="143"/>
+      <c r="E57" s="144"/>
+      <c r="F57" s="144"/>
+      <c r="G57" s="145"/>
+      <c r="H57" s="143"/>
+      <c r="I57" s="144"/>
+      <c r="J57" s="145"/>
+      <c r="K57" s="153"/>
+      <c r="L57" s="154"/>
+      <c r="M57" s="155"/>
+      <c r="N57" s="153"/>
+      <c r="O57" s="154"/>
+      <c r="P57" s="155"/>
+      <c r="Q57" s="153"/>
+      <c r="R57" s="154"/>
+      <c r="S57" s="155"/>
+      <c r="T57" s="153"/>
+      <c r="U57" s="154"/>
+      <c r="V57" s="155"/>
+      <c r="W57" s="143"/>
+      <c r="X57" s="144"/>
+      <c r="Y57" s="145"/>
+      <c r="Z57" s="153"/>
+      <c r="AA57" s="154"/>
+      <c r="AB57" s="155"/>
       <c r="AF57" s="128"/>
     </row>
     <row r="58" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="191"/>
-      <c r="B58" s="192"/>
-      <c r="C58" s="193"/>
-      <c r="D58" s="200"/>
-      <c r="E58" s="201"/>
-      <c r="F58" s="201"/>
-      <c r="G58" s="202"/>
-      <c r="H58" s="200"/>
-      <c r="I58" s="201"/>
-      <c r="J58" s="202"/>
-      <c r="K58" s="152"/>
-      <c r="L58" s="153"/>
-      <c r="M58" s="204"/>
-      <c r="N58" s="152"/>
-      <c r="O58" s="153"/>
-      <c r="P58" s="204"/>
-      <c r="Q58" s="152"/>
-      <c r="R58" s="153"/>
-      <c r="S58" s="204"/>
-      <c r="T58" s="152"/>
-      <c r="U58" s="153"/>
-      <c r="V58" s="204"/>
-      <c r="W58" s="200"/>
-      <c r="X58" s="201"/>
-      <c r="Y58" s="202"/>
-      <c r="Z58" s="152"/>
-      <c r="AA58" s="153"/>
-      <c r="AB58" s="204"/>
+      <c r="A58" s="172"/>
+      <c r="B58" s="173"/>
+      <c r="C58" s="174"/>
+      <c r="D58" s="146"/>
+      <c r="E58" s="147"/>
+      <c r="F58" s="147"/>
+      <c r="G58" s="148"/>
+      <c r="H58" s="146"/>
+      <c r="I58" s="147"/>
+      <c r="J58" s="148"/>
+      <c r="K58" s="156"/>
+      <c r="L58" s="157"/>
+      <c r="M58" s="158"/>
+      <c r="N58" s="156"/>
+      <c r="O58" s="157"/>
+      <c r="P58" s="158"/>
+      <c r="Q58" s="156"/>
+      <c r="R58" s="157"/>
+      <c r="S58" s="158"/>
+      <c r="T58" s="156"/>
+      <c r="U58" s="157"/>
+      <c r="V58" s="158"/>
+      <c r="W58" s="146"/>
+      <c r="X58" s="147"/>
+      <c r="Y58" s="148"/>
+      <c r="Z58" s="156"/>
+      <c r="AA58" s="157"/>
+      <c r="AB58" s="158"/>
       <c r="AF58" s="128"/>
     </row>
     <row r="59" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4312,7 +4314,7 @@
         <v>3</v>
       </c>
       <c r="D59" s="131" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E59" s="130"/>
       <c r="F59" s="132"/>
@@ -4342,15 +4344,15 @@
     </row>
     <row r="60" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="129" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B60" s="130"/>
       <c r="C60" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="D60" s="205"/>
-      <c r="E60" s="205"/>
-      <c r="F60" s="205"/>
+      <c r="D60" s="165"/>
+      <c r="E60" s="165"/>
+      <c r="F60" s="165"/>
       <c r="G60" s="130"/>
       <c r="H60" s="130"/>
       <c r="I60" s="130"/>
@@ -4391,203 +4393,203 @@
       <c r="AF61" s="128"/>
     </row>
     <row r="62" spans="1:32" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="206" t="s">
-        <v>50</v>
-      </c>
-      <c r="B62" s="207"/>
-      <c r="C62" s="207"/>
-      <c r="D62" s="207"/>
-      <c r="E62" s="207"/>
-      <c r="F62" s="207"/>
-      <c r="G62" s="207"/>
-      <c r="H62" s="207"/>
-      <c r="I62" s="207"/>
-      <c r="J62" s="207"/>
-      <c r="K62" s="207"/>
-      <c r="L62" s="207"/>
-      <c r="M62" s="207"/>
-      <c r="N62" s="207"/>
-      <c r="O62" s="207"/>
-      <c r="P62" s="207"/>
-      <c r="Q62" s="207"/>
-      <c r="R62" s="207"/>
-      <c r="S62" s="207"/>
-      <c r="T62" s="207"/>
-      <c r="U62" s="207"/>
-      <c r="V62" s="207"/>
-      <c r="W62" s="207"/>
-      <c r="X62" s="207"/>
-      <c r="Y62" s="207"/>
-      <c r="Z62" s="207"/>
-      <c r="AA62" s="207"/>
-      <c r="AB62" s="208"/>
+      <c r="A62" s="159" t="s">
+        <v>43</v>
+      </c>
+      <c r="B62" s="160"/>
+      <c r="C62" s="160"/>
+      <c r="D62" s="160"/>
+      <c r="E62" s="160"/>
+      <c r="F62" s="160"/>
+      <c r="G62" s="160"/>
+      <c r="H62" s="160"/>
+      <c r="I62" s="160"/>
+      <c r="J62" s="160"/>
+      <c r="K62" s="160"/>
+      <c r="L62" s="160"/>
+      <c r="M62" s="160"/>
+      <c r="N62" s="160"/>
+      <c r="O62" s="160"/>
+      <c r="P62" s="160"/>
+      <c r="Q62" s="160"/>
+      <c r="R62" s="160"/>
+      <c r="S62" s="160"/>
+      <c r="T62" s="160"/>
+      <c r="U62" s="160"/>
+      <c r="V62" s="160"/>
+      <c r="W62" s="160"/>
+      <c r="X62" s="160"/>
+      <c r="Y62" s="160"/>
+      <c r="Z62" s="160"/>
+      <c r="AA62" s="160"/>
+      <c r="AB62" s="161"/>
       <c r="AF62" s="128" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="63" spans="1:32" s="119" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="209" t="s">
-        <v>52</v>
-      </c>
-      <c r="B63" s="210"/>
-      <c r="C63" s="210"/>
-      <c r="D63" s="210"/>
-      <c r="E63" s="211"/>
-      <c r="F63" s="209" t="s">
-        <v>53</v>
-      </c>
-      <c r="G63" s="210"/>
-      <c r="H63" s="210"/>
-      <c r="I63" s="210"/>
-      <c r="J63" s="210"/>
-      <c r="K63" s="211"/>
-      <c r="L63" s="209" t="s">
-        <v>54</v>
-      </c>
-      <c r="M63" s="210"/>
-      <c r="N63" s="210"/>
-      <c r="O63" s="210"/>
-      <c r="P63" s="211"/>
-      <c r="Q63" s="148" t="s">
-        <v>55</v>
-      </c>
-      <c r="R63" s="149"/>
-      <c r="S63" s="149"/>
-      <c r="T63" s="149"/>
-      <c r="U63" s="203"/>
-      <c r="V63" s="209" t="s">
-        <v>56</v>
-      </c>
-      <c r="W63" s="210"/>
-      <c r="X63" s="210"/>
-      <c r="Y63" s="210"/>
-      <c r="Z63" s="210"/>
-      <c r="AA63" s="210"/>
-      <c r="AB63" s="211"/>
+      <c r="A63" s="162" t="s">
+        <v>45</v>
+      </c>
+      <c r="B63" s="163"/>
+      <c r="C63" s="163"/>
+      <c r="D63" s="163"/>
+      <c r="E63" s="164"/>
+      <c r="F63" s="162" t="s">
+        <v>46</v>
+      </c>
+      <c r="G63" s="163"/>
+      <c r="H63" s="163"/>
+      <c r="I63" s="163"/>
+      <c r="J63" s="163"/>
+      <c r="K63" s="164"/>
+      <c r="L63" s="162" t="s">
+        <v>47</v>
+      </c>
+      <c r="M63" s="163"/>
+      <c r="N63" s="163"/>
+      <c r="O63" s="163"/>
+      <c r="P63" s="164"/>
+      <c r="Q63" s="150" t="s">
+        <v>48</v>
+      </c>
+      <c r="R63" s="151"/>
+      <c r="S63" s="151"/>
+      <c r="T63" s="151"/>
+      <c r="U63" s="152"/>
+      <c r="V63" s="162" t="s">
+        <v>49</v>
+      </c>
+      <c r="W63" s="163"/>
+      <c r="X63" s="163"/>
+      <c r="Y63" s="163"/>
+      <c r="Z63" s="163"/>
+      <c r="AA63" s="163"/>
+      <c r="AB63" s="164"/>
       <c r="AF63" s="128"/>
     </row>
     <row r="64" spans="1:32" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="194"/>
-      <c r="B64" s="195"/>
-      <c r="C64" s="195"/>
-      <c r="D64" s="195"/>
-      <c r="E64" s="196"/>
-      <c r="F64" s="194"/>
-      <c r="G64" s="195"/>
-      <c r="H64" s="195"/>
-      <c r="I64" s="195"/>
-      <c r="J64" s="195"/>
-      <c r="K64" s="196"/>
-      <c r="L64" s="195"/>
-      <c r="M64" s="195"/>
-      <c r="N64" s="195"/>
-      <c r="O64" s="195"/>
-      <c r="P64" s="196"/>
-      <c r="Q64" s="180"/>
-      <c r="R64" s="180"/>
-      <c r="S64" s="180"/>
-      <c r="T64" s="180"/>
-      <c r="U64" s="180"/>
-      <c r="V64" s="148"/>
-      <c r="W64" s="149"/>
-      <c r="X64" s="149"/>
-      <c r="Y64" s="149"/>
-      <c r="Z64" s="149"/>
-      <c r="AA64" s="149"/>
-      <c r="AB64" s="203"/>
+      <c r="A64" s="140"/>
+      <c r="B64" s="141"/>
+      <c r="C64" s="141"/>
+      <c r="D64" s="141"/>
+      <c r="E64" s="142"/>
+      <c r="F64" s="140"/>
+      <c r="G64" s="141"/>
+      <c r="H64" s="141"/>
+      <c r="I64" s="141"/>
+      <c r="J64" s="141"/>
+      <c r="K64" s="142"/>
+      <c r="L64" s="141"/>
+      <c r="M64" s="141"/>
+      <c r="N64" s="141"/>
+      <c r="O64" s="141"/>
+      <c r="P64" s="142"/>
+      <c r="Q64" s="149"/>
+      <c r="R64" s="149"/>
+      <c r="S64" s="149"/>
+      <c r="T64" s="149"/>
+      <c r="U64" s="149"/>
+      <c r="V64" s="150"/>
+      <c r="W64" s="151"/>
+      <c r="X64" s="151"/>
+      <c r="Y64" s="151"/>
+      <c r="Z64" s="151"/>
+      <c r="AA64" s="151"/>
+      <c r="AB64" s="152"/>
       <c r="AF64" s="128"/>
     </row>
     <row r="65" spans="1:32" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="197"/>
-      <c r="B65" s="198"/>
-      <c r="C65" s="198"/>
-      <c r="D65" s="198"/>
-      <c r="E65" s="199"/>
-      <c r="F65" s="197"/>
-      <c r="G65" s="198"/>
-      <c r="H65" s="198"/>
-      <c r="I65" s="198"/>
-      <c r="J65" s="198"/>
-      <c r="K65" s="199"/>
-      <c r="L65" s="198"/>
-      <c r="M65" s="198"/>
-      <c r="N65" s="198"/>
-      <c r="O65" s="198"/>
-      <c r="P65" s="199"/>
-      <c r="Q65" s="180"/>
-      <c r="R65" s="180"/>
-      <c r="S65" s="180"/>
-      <c r="T65" s="180"/>
-      <c r="U65" s="180"/>
-      <c r="V65" s="150"/>
-      <c r="W65" s="151"/>
-      <c r="X65" s="151"/>
-      <c r="Y65" s="151"/>
-      <c r="Z65" s="151"/>
-      <c r="AA65" s="151"/>
-      <c r="AB65" s="179"/>
+      <c r="A65" s="143"/>
+      <c r="B65" s="144"/>
+      <c r="C65" s="144"/>
+      <c r="D65" s="144"/>
+      <c r="E65" s="145"/>
+      <c r="F65" s="143"/>
+      <c r="G65" s="144"/>
+      <c r="H65" s="144"/>
+      <c r="I65" s="144"/>
+      <c r="J65" s="144"/>
+      <c r="K65" s="145"/>
+      <c r="L65" s="144"/>
+      <c r="M65" s="144"/>
+      <c r="N65" s="144"/>
+      <c r="O65" s="144"/>
+      <c r="P65" s="145"/>
+      <c r="Q65" s="149"/>
+      <c r="R65" s="149"/>
+      <c r="S65" s="149"/>
+      <c r="T65" s="149"/>
+      <c r="U65" s="149"/>
+      <c r="V65" s="153"/>
+      <c r="W65" s="154"/>
+      <c r="X65" s="154"/>
+      <c r="Y65" s="154"/>
+      <c r="Z65" s="154"/>
+      <c r="AA65" s="154"/>
+      <c r="AB65" s="155"/>
       <c r="AF65" s="128"/>
     </row>
     <row r="66" spans="1:32" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="197"/>
-      <c r="B66" s="198"/>
-      <c r="C66" s="198"/>
-      <c r="D66" s="198"/>
-      <c r="E66" s="199"/>
-      <c r="F66" s="197"/>
-      <c r="G66" s="198"/>
-      <c r="H66" s="198"/>
-      <c r="I66" s="198"/>
-      <c r="J66" s="198"/>
-      <c r="K66" s="199"/>
-      <c r="L66" s="198"/>
-      <c r="M66" s="198"/>
-      <c r="N66" s="198"/>
-      <c r="O66" s="198"/>
-      <c r="P66" s="199"/>
-      <c r="Q66" s="180"/>
-      <c r="R66" s="180"/>
-      <c r="S66" s="180"/>
-      <c r="T66" s="180"/>
-      <c r="U66" s="180"/>
-      <c r="V66" s="150"/>
-      <c r="W66" s="151"/>
-      <c r="X66" s="151"/>
-      <c r="Y66" s="151"/>
-      <c r="Z66" s="151"/>
-      <c r="AA66" s="151"/>
-      <c r="AB66" s="179"/>
+      <c r="A66" s="143"/>
+      <c r="B66" s="144"/>
+      <c r="C66" s="144"/>
+      <c r="D66" s="144"/>
+      <c r="E66" s="145"/>
+      <c r="F66" s="143"/>
+      <c r="G66" s="144"/>
+      <c r="H66" s="144"/>
+      <c r="I66" s="144"/>
+      <c r="J66" s="144"/>
+      <c r="K66" s="145"/>
+      <c r="L66" s="144"/>
+      <c r="M66" s="144"/>
+      <c r="N66" s="144"/>
+      <c r="O66" s="144"/>
+      <c r="P66" s="145"/>
+      <c r="Q66" s="149"/>
+      <c r="R66" s="149"/>
+      <c r="S66" s="149"/>
+      <c r="T66" s="149"/>
+      <c r="U66" s="149"/>
+      <c r="V66" s="153"/>
+      <c r="W66" s="154"/>
+      <c r="X66" s="154"/>
+      <c r="Y66" s="154"/>
+      <c r="Z66" s="154"/>
+      <c r="AA66" s="154"/>
+      <c r="AB66" s="155"/>
       <c r="AF66" s="128"/>
     </row>
     <row r="67" spans="1:32" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="200"/>
-      <c r="B67" s="201"/>
-      <c r="C67" s="201"/>
-      <c r="D67" s="201"/>
-      <c r="E67" s="202"/>
-      <c r="F67" s="200"/>
-      <c r="G67" s="201"/>
-      <c r="H67" s="201"/>
-      <c r="I67" s="201"/>
-      <c r="J67" s="201"/>
-      <c r="K67" s="202"/>
-      <c r="L67" s="201"/>
-      <c r="M67" s="201"/>
-      <c r="N67" s="201"/>
-      <c r="O67" s="201"/>
-      <c r="P67" s="202"/>
-      <c r="Q67" s="180"/>
-      <c r="R67" s="180"/>
-      <c r="S67" s="180"/>
-      <c r="T67" s="180"/>
-      <c r="U67" s="180"/>
-      <c r="V67" s="152"/>
-      <c r="W67" s="153"/>
-      <c r="X67" s="153"/>
-      <c r="Y67" s="153"/>
-      <c r="Z67" s="153"/>
-      <c r="AA67" s="153"/>
-      <c r="AB67" s="204"/>
+      <c r="A67" s="146"/>
+      <c r="B67" s="147"/>
+      <c r="C67" s="147"/>
+      <c r="D67" s="147"/>
+      <c r="E67" s="148"/>
+      <c r="F67" s="146"/>
+      <c r="G67" s="147"/>
+      <c r="H67" s="147"/>
+      <c r="I67" s="147"/>
+      <c r="J67" s="147"/>
+      <c r="K67" s="148"/>
+      <c r="L67" s="147"/>
+      <c r="M67" s="147"/>
+      <c r="N67" s="147"/>
+      <c r="O67" s="147"/>
+      <c r="P67" s="148"/>
+      <c r="Q67" s="149"/>
+      <c r="R67" s="149"/>
+      <c r="S67" s="149"/>
+      <c r="T67" s="149"/>
+      <c r="U67" s="149"/>
+      <c r="V67" s="156"/>
+      <c r="W67" s="157"/>
+      <c r="X67" s="157"/>
+      <c r="Y67" s="157"/>
+      <c r="Z67" s="157"/>
+      <c r="AA67" s="157"/>
+      <c r="AB67" s="158"/>
       <c r="AF67" s="128"/>
     </row>
     <row r="68" spans="1:32" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4628,27 +4630,64 @@
     </row>
   </sheetData>
   <mergeCells count="95">
-    <mergeCell ref="A64:E67"/>
-    <mergeCell ref="F64:K67"/>
-    <mergeCell ref="L64:P67"/>
-    <mergeCell ref="Q64:U67"/>
-    <mergeCell ref="V64:AB67"/>
-    <mergeCell ref="A62:AB62"/>
-    <mergeCell ref="A63:E63"/>
-    <mergeCell ref="F63:K63"/>
-    <mergeCell ref="L63:P63"/>
-    <mergeCell ref="Q63:U63"/>
-    <mergeCell ref="V63:AB63"/>
-    <mergeCell ref="Q56:S58"/>
-    <mergeCell ref="T56:V58"/>
-    <mergeCell ref="W56:Y58"/>
-    <mergeCell ref="Z56:AB58"/>
-    <mergeCell ref="D60:F60"/>
-    <mergeCell ref="A56:C58"/>
-    <mergeCell ref="D56:G58"/>
-    <mergeCell ref="H56:J58"/>
-    <mergeCell ref="K56:M58"/>
-    <mergeCell ref="N56:P58"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="D45:K45"/>
+    <mergeCell ref="L45:N45"/>
+    <mergeCell ref="W45:Z45"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="D43:K43"/>
+    <mergeCell ref="L43:N43"/>
+    <mergeCell ref="W43:Z43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="D44:K44"/>
+    <mergeCell ref="L44:N44"/>
+    <mergeCell ref="W44:Z44"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D41:K41"/>
+    <mergeCell ref="L41:N41"/>
+    <mergeCell ref="W41:Z41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D42:K42"/>
+    <mergeCell ref="L42:N42"/>
+    <mergeCell ref="W42:Z42"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D39:K39"/>
+    <mergeCell ref="L39:N39"/>
+    <mergeCell ref="W39:Z39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="D40:K40"/>
+    <mergeCell ref="L40:N40"/>
+    <mergeCell ref="W40:Z40"/>
+    <mergeCell ref="A2:C5"/>
+    <mergeCell ref="L2:Q3"/>
+    <mergeCell ref="F4:W4"/>
+    <mergeCell ref="D5:AB5"/>
+    <mergeCell ref="A6:AB6"/>
+    <mergeCell ref="O33:V33"/>
+    <mergeCell ref="W33:Z35"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="U34:V34"/>
+    <mergeCell ref="B33:C35"/>
+    <mergeCell ref="D33:K35"/>
+    <mergeCell ref="L33:N35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="D36:K36"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D37:K37"/>
+    <mergeCell ref="L37:N37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D38:K38"/>
+    <mergeCell ref="L38:N38"/>
+    <mergeCell ref="M52:O52"/>
+    <mergeCell ref="P52:Q52"/>
+    <mergeCell ref="U52:W52"/>
+    <mergeCell ref="Y52:Z52"/>
+    <mergeCell ref="W36:Z36"/>
+    <mergeCell ref="W37:Z37"/>
+    <mergeCell ref="W38:Z38"/>
     <mergeCell ref="AA52:AB52"/>
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="D55:G55"/>
@@ -4665,64 +4704,27 @@
     <mergeCell ref="G52:H52"/>
     <mergeCell ref="I52:J52"/>
     <mergeCell ref="K52:L52"/>
-    <mergeCell ref="M52:O52"/>
-    <mergeCell ref="P52:Q52"/>
-    <mergeCell ref="U52:W52"/>
-    <mergeCell ref="Y52:Z52"/>
-    <mergeCell ref="W36:Z36"/>
-    <mergeCell ref="W37:Z37"/>
-    <mergeCell ref="W38:Z38"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="D37:K37"/>
-    <mergeCell ref="L37:N37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:K38"/>
-    <mergeCell ref="L38:N38"/>
-    <mergeCell ref="B33:C35"/>
-    <mergeCell ref="D33:K35"/>
-    <mergeCell ref="L33:N35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="D36:K36"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="O33:V33"/>
-    <mergeCell ref="W33:Z35"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:R34"/>
-    <mergeCell ref="S34:T34"/>
-    <mergeCell ref="U34:V34"/>
-    <mergeCell ref="A2:C5"/>
-    <mergeCell ref="L2:Q3"/>
-    <mergeCell ref="F4:W4"/>
-    <mergeCell ref="D5:AB5"/>
-    <mergeCell ref="A6:AB6"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D39:K39"/>
-    <mergeCell ref="L39:N39"/>
-    <mergeCell ref="W39:Z39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D40:K40"/>
-    <mergeCell ref="L40:N40"/>
-    <mergeCell ref="W40:Z40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="D41:K41"/>
-    <mergeCell ref="L41:N41"/>
-    <mergeCell ref="W41:Z41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="D42:K42"/>
-    <mergeCell ref="L42:N42"/>
-    <mergeCell ref="W42:Z42"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="D45:K45"/>
-    <mergeCell ref="L45:N45"/>
-    <mergeCell ref="W45:Z45"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="D43:K43"/>
-    <mergeCell ref="L43:N43"/>
-    <mergeCell ref="W43:Z43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="D44:K44"/>
-    <mergeCell ref="L44:N44"/>
-    <mergeCell ref="W44:Z44"/>
+    <mergeCell ref="A56:C58"/>
+    <mergeCell ref="D56:G58"/>
+    <mergeCell ref="H56:J58"/>
+    <mergeCell ref="K56:M58"/>
+    <mergeCell ref="N56:P58"/>
+    <mergeCell ref="Q56:S58"/>
+    <mergeCell ref="T56:V58"/>
+    <mergeCell ref="W56:Y58"/>
+    <mergeCell ref="Z56:AB58"/>
+    <mergeCell ref="D60:F60"/>
+    <mergeCell ref="A62:AB62"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="F63:K63"/>
+    <mergeCell ref="L63:P63"/>
+    <mergeCell ref="Q63:U63"/>
+    <mergeCell ref="V63:AB63"/>
+    <mergeCell ref="A64:E67"/>
+    <mergeCell ref="F64:K67"/>
+    <mergeCell ref="L64:P67"/>
+    <mergeCell ref="Q64:U67"/>
+    <mergeCell ref="V64:AB67"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="24" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -4749,48 +4751,48 @@
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
-      <c r="L1" s="212"/>
-      <c r="M1" s="212"/>
-      <c r="N1" s="212"/>
-      <c r="O1" s="212"/>
-      <c r="P1" s="212"/>
-      <c r="Q1" s="212"/>
-      <c r="R1" s="212"/>
+      <c r="L1" s="267"/>
+      <c r="M1" s="267"/>
+      <c r="N1" s="267"/>
+      <c r="O1" s="267"/>
+      <c r="P1" s="267"/>
+      <c r="Q1" s="267"/>
+      <c r="R1" s="267"/>
     </row>
     <row r="2" spans="1:21" s="4" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="213" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2" s="214"/>
-      <c r="C2" s="214"/>
-      <c r="D2" s="214"/>
-      <c r="E2" s="214"/>
-      <c r="F2" s="214"/>
-      <c r="G2" s="214"/>
-      <c r="H2" s="214"/>
-      <c r="I2" s="214"/>
-      <c r="J2" s="214"/>
-      <c r="K2" s="214"/>
-      <c r="L2" s="214"/>
-      <c r="M2" s="214"/>
-      <c r="N2" s="214"/>
-      <c r="O2" s="214"/>
+      <c r="A2" s="268" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="269"/>
+      <c r="C2" s="269"/>
+      <c r="D2" s="269"/>
+      <c r="E2" s="269"/>
+      <c r="F2" s="269"/>
+      <c r="G2" s="269"/>
+      <c r="H2" s="269"/>
+      <c r="I2" s="269"/>
+      <c r="J2" s="269"/>
+      <c r="K2" s="269"/>
+      <c r="L2" s="269"/>
+      <c r="M2" s="269"/>
+      <c r="N2" s="269"/>
+      <c r="O2" s="269"/>
       <c r="P2" s="5" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="Q2" s="6"/>
       <c r="R2" s="7"/>
     </row>
     <row r="3" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="216" t="s">
-        <v>60</v>
+      <c r="A3" s="271" t="s">
+        <v>53</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C3" s="10"/>
       <c r="D3" s="10"/>
@@ -4798,10 +4800,10 @@
       <c r="F3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="215"/>
-      <c r="H3" s="215"/>
-      <c r="I3" s="215"/>
-      <c r="J3" s="215"/>
+      <c r="G3" s="270"/>
+      <c r="H3" s="270"/>
+      <c r="I3" s="270"/>
+      <c r="J3" s="270"/>
       <c r="K3" s="13"/>
       <c r="R3" s="14"/>
       <c r="S3" s="15"/>
@@ -4809,9 +4811,9 @@
       <c r="U3" s="15"/>
     </row>
     <row r="4" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="217"/>
+      <c r="A4" s="272"/>
       <c r="B4" s="16" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C4" s="17"/>
       <c r="D4" s="17"/>
@@ -4819,10 +4821,10 @@
       <c r="F4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="215"/>
-      <c r="H4" s="215"/>
-      <c r="I4" s="215"/>
-      <c r="J4" s="215"/>
+      <c r="G4" s="270"/>
+      <c r="H4" s="270"/>
+      <c r="I4" s="270"/>
+      <c r="J4" s="270"/>
       <c r="K4" s="18"/>
       <c r="R4" s="14"/>
       <c r="S4" s="15"/>
@@ -4830,9 +4832,9 @@
       <c r="U4" s="15"/>
     </row>
     <row r="5" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="217"/>
+      <c r="A5" s="272"/>
       <c r="B5" s="16" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
@@ -4840,10 +4842,10 @@
       <c r="F5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="215"/>
-      <c r="H5" s="215"/>
-      <c r="I5" s="215"/>
-      <c r="J5" s="215"/>
+      <c r="G5" s="270"/>
+      <c r="H5" s="270"/>
+      <c r="I5" s="270"/>
+      <c r="J5" s="270"/>
       <c r="K5" s="18"/>
       <c r="R5" s="14"/>
       <c r="S5" s="15"/>
@@ -4851,9 +4853,9 @@
       <c r="U5" s="15"/>
     </row>
     <row r="6" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="217"/>
+      <c r="A6" s="272"/>
       <c r="B6" s="16" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C6" s="19"/>
       <c r="D6" s="19"/>
@@ -4861,10 +4863,10 @@
       <c r="F6" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="219"/>
-      <c r="H6" s="219"/>
-      <c r="I6" s="219"/>
-      <c r="J6" s="219"/>
+      <c r="G6" s="274"/>
+      <c r="H6" s="274"/>
+      <c r="I6" s="274"/>
+      <c r="J6" s="274"/>
       <c r="K6" s="20"/>
       <c r="R6" s="14"/>
       <c r="S6" s="15"/>
@@ -4872,9 +4874,9 @@
       <c r="U6" s="15"/>
     </row>
     <row r="7" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="217"/>
+      <c r="A7" s="272"/>
       <c r="B7" s="21" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C7" s="19"/>
       <c r="D7" s="19"/>
@@ -4882,10 +4884,10 @@
       <c r="F7" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="219"/>
-      <c r="H7" s="219"/>
-      <c r="I7" s="219"/>
-      <c r="J7" s="219"/>
+      <c r="G7" s="274"/>
+      <c r="H7" s="274"/>
+      <c r="I7" s="274"/>
+      <c r="J7" s="274"/>
       <c r="K7" s="20"/>
       <c r="R7" s="14"/>
       <c r="S7" s="15"/>
@@ -4893,9 +4895,9 @@
       <c r="U7" s="15"/>
     </row>
     <row r="8" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="217"/>
+      <c r="A8" s="272"/>
       <c r="B8" s="16" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
@@ -4903,10 +4905,10 @@
       <c r="F8" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G8" s="215"/>
-      <c r="H8" s="215"/>
-      <c r="I8" s="215"/>
-      <c r="J8" s="215"/>
+      <c r="G8" s="270"/>
+      <c r="H8" s="270"/>
+      <c r="I8" s="270"/>
+      <c r="J8" s="270"/>
       <c r="K8" s="20"/>
       <c r="R8" s="14"/>
       <c r="S8" s="15"/>
@@ -4914,9 +4916,9 @@
       <c r="U8" s="15"/>
     </row>
     <row r="9" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="217"/>
+      <c r="A9" s="272"/>
       <c r="B9" s="16" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
@@ -4924,10 +4926,10 @@
       <c r="F9" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G9" s="215"/>
-      <c r="H9" s="215"/>
-      <c r="I9" s="215"/>
-      <c r="J9" s="215"/>
+      <c r="G9" s="270"/>
+      <c r="H9" s="270"/>
+      <c r="I9" s="270"/>
+      <c r="J9" s="270"/>
       <c r="K9" s="18"/>
       <c r="R9" s="14"/>
       <c r="S9" s="15"/>
@@ -4935,9 +4937,9 @@
       <c r="U9" s="15"/>
     </row>
     <row r="10" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="217"/>
+      <c r="A10" s="272"/>
       <c r="B10" s="16" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
@@ -4945,10 +4947,10 @@
       <c r="F10" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G10" s="215"/>
-      <c r="H10" s="215"/>
-      <c r="I10" s="215"/>
-      <c r="J10" s="215"/>
+      <c r="G10" s="270"/>
+      <c r="H10" s="270"/>
+      <c r="I10" s="270"/>
+      <c r="J10" s="270"/>
       <c r="K10" s="18"/>
       <c r="R10" s="14"/>
       <c r="S10" s="15"/>
@@ -4956,9 +4958,9 @@
       <c r="U10" s="15"/>
     </row>
     <row r="11" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="217"/>
+      <c r="A11" s="272"/>
       <c r="B11" s="22" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
@@ -4966,10 +4968,10 @@
       <c r="F11" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="215"/>
-      <c r="H11" s="215"/>
-      <c r="I11" s="215"/>
-      <c r="J11" s="215"/>
+      <c r="G11" s="270"/>
+      <c r="H11" s="270"/>
+      <c r="I11" s="270"/>
+      <c r="J11" s="270"/>
       <c r="K11" s="18"/>
       <c r="L11" s="18"/>
       <c r="M11" s="18"/>
@@ -4983,9 +4985,9 @@
       <c r="U11" s="15"/>
     </row>
     <row r="12" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="217"/>
+      <c r="A12" s="272"/>
       <c r="B12" s="22" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C12" s="23"/>
       <c r="D12" s="23"/>
@@ -4993,10 +4995,10 @@
       <c r="F12" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G12" s="215"/>
-      <c r="H12" s="215"/>
-      <c r="I12" s="215"/>
-      <c r="J12" s="215"/>
+      <c r="G12" s="270"/>
+      <c r="H12" s="270"/>
+      <c r="I12" s="270"/>
+      <c r="J12" s="270"/>
       <c r="K12" s="18"/>
       <c r="L12" s="24"/>
       <c r="M12" s="24"/>
@@ -5007,9 +5009,9 @@
       <c r="R12" s="25"/>
     </row>
     <row r="13" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="217"/>
+      <c r="A13" s="272"/>
       <c r="B13" s="26" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C13" s="23"/>
       <c r="D13" s="23"/>
@@ -5017,10 +5019,10 @@
       <c r="F13" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G13" s="219"/>
-      <c r="H13" s="219"/>
-      <c r="I13" s="219"/>
-      <c r="J13" s="219"/>
+      <c r="G13" s="274"/>
+      <c r="H13" s="274"/>
+      <c r="I13" s="274"/>
+      <c r="J13" s="274"/>
       <c r="K13" s="24"/>
       <c r="L13" s="18"/>
       <c r="M13" s="24"/>
@@ -5031,9 +5033,9 @@
       <c r="R13" s="25"/>
     </row>
     <row r="14" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="217"/>
+      <c r="A14" s="272"/>
       <c r="B14" s="22" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C14" s="23"/>
       <c r="D14" s="23"/>
@@ -5041,10 +5043,10 @@
       <c r="F14" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G14" s="219"/>
-      <c r="H14" s="219"/>
-      <c r="I14" s="219"/>
-      <c r="J14" s="219"/>
+      <c r="G14" s="274"/>
+      <c r="H14" s="274"/>
+      <c r="I14" s="274"/>
+      <c r="J14" s="274"/>
       <c r="K14" s="24"/>
       <c r="L14" s="18"/>
       <c r="M14" s="24"/>
@@ -5055,9 +5057,9 @@
       <c r="R14" s="25"/>
     </row>
     <row r="15" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="217"/>
+      <c r="A15" s="272"/>
       <c r="B15" s="22" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C15" s="23"/>
       <c r="D15" s="23"/>
@@ -5065,10 +5067,10 @@
       <c r="F15" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G15" s="215"/>
-      <c r="H15" s="215"/>
-      <c r="I15" s="215"/>
-      <c r="J15" s="215"/>
+      <c r="G15" s="270"/>
+      <c r="H15" s="270"/>
+      <c r="I15" s="270"/>
+      <c r="J15" s="270"/>
       <c r="K15" s="24"/>
       <c r="L15" s="18"/>
       <c r="M15" s="24"/>
@@ -5079,9 +5081,9 @@
       <c r="R15" s="25"/>
     </row>
     <row r="16" spans="1:21" s="8" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="217"/>
+      <c r="A16" s="272"/>
       <c r="B16" s="22" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="23"/>
@@ -5089,10 +5091,10 @@
       <c r="F16" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G16" s="215"/>
-      <c r="H16" s="215"/>
-      <c r="I16" s="215"/>
-      <c r="J16" s="215"/>
+      <c r="G16" s="270"/>
+      <c r="H16" s="270"/>
+      <c r="I16" s="270"/>
+      <c r="J16" s="270"/>
       <c r="K16" s="24"/>
       <c r="L16" s="18"/>
       <c r="M16" s="24"/>
@@ -5103,7 +5105,7 @@
       <c r="R16" s="25"/>
     </row>
     <row r="17" spans="1:23" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="217"/>
+      <c r="A17" s="272"/>
       <c r="B17" s="22"/>
       <c r="C17" s="28"/>
       <c r="D17" s="28"/>
@@ -5123,7 +5125,7 @@
       <c r="R17" s="25"/>
     </row>
     <row r="18" spans="1:23" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="217"/>
+      <c r="A18" s="272"/>
       <c r="B18" s="22"/>
       <c r="C18" s="28"/>
       <c r="D18" s="28"/>
@@ -5143,7 +5145,7 @@
       <c r="R18" s="25"/>
     </row>
     <row r="19" spans="1:23" s="8" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="217"/>
+      <c r="A19" s="272"/>
       <c r="B19" s="22"/>
       <c r="C19" s="24"/>
       <c r="D19" s="24"/>
@@ -5163,9 +5165,9 @@
       <c r="R19" s="25"/>
     </row>
     <row r="20" spans="1:23" s="8" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="217"/>
+      <c r="A20" s="272"/>
       <c r="B20" s="33" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C20" s="34"/>
       <c r="D20" s="34"/>
@@ -5185,23 +5187,23 @@
       <c r="R20" s="36"/>
     </row>
     <row r="21" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="217"/>
+      <c r="A21" s="272"/>
       <c r="B21" s="38"/>
-      <c r="C21" s="220"/>
-      <c r="D21" s="220"/>
-      <c r="E21" s="220"/>
-      <c r="F21" s="220"/>
-      <c r="G21" s="220"/>
-      <c r="H21" s="220"/>
-      <c r="I21" s="220"/>
-      <c r="J21" s="220"/>
-      <c r="K21" s="220"/>
-      <c r="L21" s="220"/>
-      <c r="M21" s="220"/>
-      <c r="N21" s="220"/>
-      <c r="O21" s="220"/>
-      <c r="P21" s="220"/>
-      <c r="Q21" s="220"/>
+      <c r="C21" s="248"/>
+      <c r="D21" s="248"/>
+      <c r="E21" s="248"/>
+      <c r="F21" s="248"/>
+      <c r="G21" s="248"/>
+      <c r="H21" s="248"/>
+      <c r="I21" s="248"/>
+      <c r="J21" s="248"/>
+      <c r="K21" s="248"/>
+      <c r="L21" s="248"/>
+      <c r="M21" s="248"/>
+      <c r="N21" s="248"/>
+      <c r="O21" s="248"/>
+      <c r="P21" s="248"/>
+      <c r="Q21" s="248"/>
       <c r="R21" s="39"/>
       <c r="S21" s="40"/>
       <c r="T21" s="41"/>
@@ -5210,23 +5212,23 @@
       <c r="W21" s="41"/>
     </row>
     <row r="22" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="217"/>
+      <c r="A22" s="272"/>
       <c r="B22" s="38"/>
-      <c r="C22" s="220"/>
-      <c r="D22" s="220"/>
-      <c r="E22" s="220"/>
-      <c r="F22" s="220"/>
-      <c r="G22" s="220"/>
-      <c r="H22" s="220"/>
-      <c r="I22" s="220"/>
-      <c r="J22" s="220"/>
-      <c r="K22" s="220"/>
-      <c r="L22" s="220"/>
-      <c r="M22" s="220"/>
-      <c r="N22" s="220"/>
-      <c r="O22" s="220"/>
-      <c r="P22" s="220"/>
-      <c r="Q22" s="220"/>
+      <c r="C22" s="248"/>
+      <c r="D22" s="248"/>
+      <c r="E22" s="248"/>
+      <c r="F22" s="248"/>
+      <c r="G22" s="248"/>
+      <c r="H22" s="248"/>
+      <c r="I22" s="248"/>
+      <c r="J22" s="248"/>
+      <c r="K22" s="248"/>
+      <c r="L22" s="248"/>
+      <c r="M22" s="248"/>
+      <c r="N22" s="248"/>
+      <c r="O22" s="248"/>
+      <c r="P22" s="248"/>
+      <c r="Q22" s="248"/>
       <c r="R22" s="39"/>
       <c r="S22" s="40"/>
       <c r="T22" s="41"/>
@@ -5235,23 +5237,23 @@
       <c r="W22" s="41"/>
     </row>
     <row r="23" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="217"/>
+      <c r="A23" s="272"/>
       <c r="B23" s="38"/>
-      <c r="C23" s="220"/>
-      <c r="D23" s="220"/>
-      <c r="E23" s="220"/>
-      <c r="F23" s="220"/>
-      <c r="G23" s="220"/>
-      <c r="H23" s="220"/>
-      <c r="I23" s="220"/>
-      <c r="J23" s="220"/>
-      <c r="K23" s="220"/>
-      <c r="L23" s="220"/>
-      <c r="M23" s="220"/>
-      <c r="N23" s="220"/>
-      <c r="O23" s="220"/>
-      <c r="P23" s="220"/>
-      <c r="Q23" s="220"/>
+      <c r="C23" s="248"/>
+      <c r="D23" s="248"/>
+      <c r="E23" s="248"/>
+      <c r="F23" s="248"/>
+      <c r="G23" s="248"/>
+      <c r="H23" s="248"/>
+      <c r="I23" s="248"/>
+      <c r="J23" s="248"/>
+      <c r="K23" s="248"/>
+      <c r="L23" s="248"/>
+      <c r="M23" s="248"/>
+      <c r="N23" s="248"/>
+      <c r="O23" s="248"/>
+      <c r="P23" s="248"/>
+      <c r="Q23" s="248"/>
       <c r="R23" s="39"/>
       <c r="S23" s="40"/>
       <c r="T23" s="41"/>
@@ -5260,23 +5262,23 @@
       <c r="W23" s="41"/>
     </row>
     <row r="24" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="217"/>
+      <c r="A24" s="272"/>
       <c r="B24" s="38"/>
-      <c r="C24" s="220"/>
-      <c r="D24" s="220"/>
-      <c r="E24" s="220"/>
-      <c r="F24" s="220"/>
-      <c r="G24" s="220"/>
-      <c r="H24" s="220"/>
-      <c r="I24" s="220"/>
-      <c r="J24" s="220"/>
-      <c r="K24" s="220"/>
-      <c r="L24" s="220"/>
-      <c r="M24" s="220"/>
-      <c r="N24" s="220"/>
-      <c r="O24" s="220"/>
-      <c r="P24" s="220"/>
-      <c r="Q24" s="220"/>
+      <c r="C24" s="248"/>
+      <c r="D24" s="248"/>
+      <c r="E24" s="248"/>
+      <c r="F24" s="248"/>
+      <c r="G24" s="248"/>
+      <c r="H24" s="248"/>
+      <c r="I24" s="248"/>
+      <c r="J24" s="248"/>
+      <c r="K24" s="248"/>
+      <c r="L24" s="248"/>
+      <c r="M24" s="248"/>
+      <c r="N24" s="248"/>
+      <c r="O24" s="248"/>
+      <c r="P24" s="248"/>
+      <c r="Q24" s="248"/>
       <c r="R24" s="39"/>
       <c r="S24" s="40"/>
       <c r="T24" s="41"/>
@@ -5285,23 +5287,23 @@
       <c r="W24" s="41"/>
     </row>
     <row r="25" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="217"/>
+      <c r="A25" s="272"/>
       <c r="B25" s="38"/>
-      <c r="C25" s="220"/>
-      <c r="D25" s="220"/>
-      <c r="E25" s="220"/>
-      <c r="F25" s="220"/>
-      <c r="G25" s="220"/>
-      <c r="H25" s="220"/>
-      <c r="I25" s="220"/>
-      <c r="J25" s="220"/>
-      <c r="K25" s="220"/>
-      <c r="L25" s="220"/>
-      <c r="M25" s="220"/>
-      <c r="N25" s="220"/>
-      <c r="O25" s="220"/>
-      <c r="P25" s="220"/>
-      <c r="Q25" s="220"/>
+      <c r="C25" s="248"/>
+      <c r="D25" s="248"/>
+      <c r="E25" s="248"/>
+      <c r="F25" s="248"/>
+      <c r="G25" s="248"/>
+      <c r="H25" s="248"/>
+      <c r="I25" s="248"/>
+      <c r="J25" s="248"/>
+      <c r="K25" s="248"/>
+      <c r="L25" s="248"/>
+      <c r="M25" s="248"/>
+      <c r="N25" s="248"/>
+      <c r="O25" s="248"/>
+      <c r="P25" s="248"/>
+      <c r="Q25" s="248"/>
       <c r="R25" s="42"/>
       <c r="S25" s="40"/>
       <c r="T25" s="41"/>
@@ -5310,23 +5312,23 @@
       <c r="W25" s="41"/>
     </row>
     <row r="26" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="217"/>
+      <c r="A26" s="272"/>
       <c r="B26" s="38"/>
-      <c r="C26" s="220"/>
-      <c r="D26" s="220"/>
-      <c r="E26" s="220"/>
-      <c r="F26" s="220"/>
-      <c r="G26" s="220"/>
-      <c r="H26" s="220"/>
-      <c r="I26" s="220"/>
-      <c r="J26" s="220"/>
-      <c r="K26" s="220"/>
-      <c r="L26" s="220"/>
-      <c r="M26" s="220"/>
-      <c r="N26" s="220"/>
-      <c r="O26" s="220"/>
-      <c r="P26" s="220"/>
-      <c r="Q26" s="220"/>
+      <c r="C26" s="248"/>
+      <c r="D26" s="248"/>
+      <c r="E26" s="248"/>
+      <c r="F26" s="248"/>
+      <c r="G26" s="248"/>
+      <c r="H26" s="248"/>
+      <c r="I26" s="248"/>
+      <c r="J26" s="248"/>
+      <c r="K26" s="248"/>
+      <c r="L26" s="248"/>
+      <c r="M26" s="248"/>
+      <c r="N26" s="248"/>
+      <c r="O26" s="248"/>
+      <c r="P26" s="248"/>
+      <c r="Q26" s="248"/>
       <c r="R26" s="39"/>
       <c r="S26" s="40"/>
       <c r="T26" s="41"/>
@@ -5335,23 +5337,23 @@
       <c r="W26" s="41"/>
     </row>
     <row r="27" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="217"/>
+      <c r="A27" s="272"/>
       <c r="B27" s="38"/>
-      <c r="C27" s="220"/>
-      <c r="D27" s="220"/>
-      <c r="E27" s="220"/>
-      <c r="F27" s="220"/>
-      <c r="G27" s="220"/>
-      <c r="H27" s="220"/>
-      <c r="I27" s="220"/>
-      <c r="J27" s="220"/>
-      <c r="K27" s="220"/>
-      <c r="L27" s="220"/>
-      <c r="M27" s="220"/>
-      <c r="N27" s="220"/>
-      <c r="O27" s="220"/>
-      <c r="P27" s="220"/>
-      <c r="Q27" s="220"/>
+      <c r="C27" s="248"/>
+      <c r="D27" s="248"/>
+      <c r="E27" s="248"/>
+      <c r="F27" s="248"/>
+      <c r="G27" s="248"/>
+      <c r="H27" s="248"/>
+      <c r="I27" s="248"/>
+      <c r="J27" s="248"/>
+      <c r="K27" s="248"/>
+      <c r="L27" s="248"/>
+      <c r="M27" s="248"/>
+      <c r="N27" s="248"/>
+      <c r="O27" s="248"/>
+      <c r="P27" s="248"/>
+      <c r="Q27" s="248"/>
       <c r="R27" s="39"/>
       <c r="S27" s="40"/>
       <c r="T27" s="41"/>
@@ -5360,23 +5362,23 @@
       <c r="W27" s="41"/>
     </row>
     <row r="28" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="217"/>
+      <c r="A28" s="272"/>
       <c r="B28" s="38"/>
-      <c r="C28" s="220"/>
-      <c r="D28" s="220"/>
-      <c r="E28" s="220"/>
-      <c r="F28" s="220"/>
-      <c r="G28" s="220"/>
-      <c r="H28" s="220"/>
-      <c r="I28" s="220"/>
-      <c r="J28" s="220"/>
-      <c r="K28" s="220"/>
-      <c r="L28" s="220"/>
-      <c r="M28" s="220"/>
-      <c r="N28" s="220"/>
-      <c r="O28" s="220"/>
-      <c r="P28" s="220"/>
-      <c r="Q28" s="220"/>
+      <c r="C28" s="248"/>
+      <c r="D28" s="248"/>
+      <c r="E28" s="248"/>
+      <c r="F28" s="248"/>
+      <c r="G28" s="248"/>
+      <c r="H28" s="248"/>
+      <c r="I28" s="248"/>
+      <c r="J28" s="248"/>
+      <c r="K28" s="248"/>
+      <c r="L28" s="248"/>
+      <c r="M28" s="248"/>
+      <c r="N28" s="248"/>
+      <c r="O28" s="248"/>
+      <c r="P28" s="248"/>
+      <c r="Q28" s="248"/>
       <c r="R28" s="39"/>
       <c r="S28" s="40"/>
       <c r="T28" s="41"/>
@@ -5385,7 +5387,7 @@
       <c r="W28" s="41"/>
     </row>
     <row r="29" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="217"/>
+      <c r="A29" s="272"/>
       <c r="B29" s="38"/>
       <c r="C29" s="43"/>
       <c r="D29" s="43"/>
@@ -5410,7 +5412,7 @@
       <c r="W29" s="41"/>
     </row>
     <row r="30" spans="1:23" s="8" customFormat="1" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="217"/>
+      <c r="A30" s="272"/>
       <c r="B30" s="46"/>
       <c r="C30" s="47"/>
       <c r="D30" s="47"/>
@@ -5430,9 +5432,9 @@
       <c r="R30" s="50"/>
     </row>
     <row r="31" spans="1:23" s="8" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="217"/>
+      <c r="A31" s="272"/>
       <c r="B31" s="51" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C31" s="52"/>
       <c r="D31" s="52"/>
@@ -5452,107 +5454,107 @@
       <c r="R31" s="55"/>
     </row>
     <row r="32" spans="1:23" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="217"/>
+      <c r="A32" s="272"/>
       <c r="B32" s="57"/>
-      <c r="C32" s="220"/>
-      <c r="D32" s="220"/>
-      <c r="E32" s="220"/>
-      <c r="F32" s="220"/>
-      <c r="G32" s="220"/>
-      <c r="H32" s="220"/>
-      <c r="I32" s="220"/>
-      <c r="J32" s="220"/>
-      <c r="K32" s="220"/>
-      <c r="L32" s="220"/>
-      <c r="M32" s="220"/>
-      <c r="N32" s="220"/>
-      <c r="O32" s="220"/>
-      <c r="P32" s="220"/>
-      <c r="Q32" s="220"/>
+      <c r="C32" s="248"/>
+      <c r="D32" s="248"/>
+      <c r="E32" s="248"/>
+      <c r="F32" s="248"/>
+      <c r="G32" s="248"/>
+      <c r="H32" s="248"/>
+      <c r="I32" s="248"/>
+      <c r="J32" s="248"/>
+      <c r="K32" s="248"/>
+      <c r="L32" s="248"/>
+      <c r="M32" s="248"/>
+      <c r="N32" s="248"/>
+      <c r="O32" s="248"/>
+      <c r="P32" s="248"/>
+      <c r="Q32" s="248"/>
       <c r="R32" s="58"/>
     </row>
     <row r="33" spans="1:18" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="217"/>
+      <c r="A33" s="272"/>
       <c r="B33" s="57"/>
-      <c r="C33" s="220"/>
-      <c r="D33" s="220"/>
-      <c r="E33" s="220"/>
-      <c r="F33" s="220"/>
-      <c r="G33" s="220"/>
-      <c r="H33" s="220"/>
-      <c r="I33" s="220"/>
-      <c r="J33" s="220"/>
-      <c r="K33" s="220"/>
-      <c r="L33" s="220"/>
-      <c r="M33" s="220"/>
-      <c r="N33" s="220"/>
-      <c r="O33" s="220"/>
-      <c r="P33" s="220"/>
-      <c r="Q33" s="220"/>
+      <c r="C33" s="248"/>
+      <c r="D33" s="248"/>
+      <c r="E33" s="248"/>
+      <c r="F33" s="248"/>
+      <c r="G33" s="248"/>
+      <c r="H33" s="248"/>
+      <c r="I33" s="248"/>
+      <c r="J33" s="248"/>
+      <c r="K33" s="248"/>
+      <c r="L33" s="248"/>
+      <c r="M33" s="248"/>
+      <c r="N33" s="248"/>
+      <c r="O33" s="248"/>
+      <c r="P33" s="248"/>
+      <c r="Q33" s="248"/>
       <c r="R33" s="58"/>
     </row>
     <row r="34" spans="1:18" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="217"/>
+      <c r="A34" s="272"/>
       <c r="B34" s="57"/>
-      <c r="C34" s="220"/>
-      <c r="D34" s="220"/>
-      <c r="E34" s="220"/>
-      <c r="F34" s="220"/>
-      <c r="G34" s="220"/>
-      <c r="H34" s="220"/>
-      <c r="I34" s="220"/>
-      <c r="J34" s="220"/>
-      <c r="K34" s="220"/>
-      <c r="L34" s="220"/>
-      <c r="M34" s="220"/>
-      <c r="N34" s="220"/>
-      <c r="O34" s="220"/>
-      <c r="P34" s="220"/>
-      <c r="Q34" s="220"/>
+      <c r="C34" s="248"/>
+      <c r="D34" s="248"/>
+      <c r="E34" s="248"/>
+      <c r="F34" s="248"/>
+      <c r="G34" s="248"/>
+      <c r="H34" s="248"/>
+      <c r="I34" s="248"/>
+      <c r="J34" s="248"/>
+      <c r="K34" s="248"/>
+      <c r="L34" s="248"/>
+      <c r="M34" s="248"/>
+      <c r="N34" s="248"/>
+      <c r="O34" s="248"/>
+      <c r="P34" s="248"/>
+      <c r="Q34" s="248"/>
       <c r="R34" s="58"/>
     </row>
     <row r="35" spans="1:18" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="217"/>
+      <c r="A35" s="272"/>
       <c r="B35" s="57"/>
-      <c r="C35" s="220"/>
-      <c r="D35" s="220"/>
-      <c r="E35" s="220"/>
-      <c r="F35" s="220"/>
-      <c r="G35" s="220"/>
-      <c r="H35" s="220"/>
-      <c r="I35" s="220"/>
-      <c r="J35" s="220"/>
-      <c r="K35" s="220"/>
-      <c r="L35" s="220"/>
-      <c r="M35" s="220"/>
-      <c r="N35" s="220"/>
-      <c r="O35" s="220"/>
-      <c r="P35" s="220"/>
-      <c r="Q35" s="220"/>
+      <c r="C35" s="248"/>
+      <c r="D35" s="248"/>
+      <c r="E35" s="248"/>
+      <c r="F35" s="248"/>
+      <c r="G35" s="248"/>
+      <c r="H35" s="248"/>
+      <c r="I35" s="248"/>
+      <c r="J35" s="248"/>
+      <c r="K35" s="248"/>
+      <c r="L35" s="248"/>
+      <c r="M35" s="248"/>
+      <c r="N35" s="248"/>
+      <c r="O35" s="248"/>
+      <c r="P35" s="248"/>
+      <c r="Q35" s="248"/>
       <c r="R35" s="58"/>
     </row>
     <row r="36" spans="1:18" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="217"/>
+      <c r="A36" s="272"/>
       <c r="B36" s="57"/>
-      <c r="C36" s="220"/>
-      <c r="D36" s="220"/>
-      <c r="E36" s="220"/>
-      <c r="F36" s="220"/>
-      <c r="G36" s="220"/>
-      <c r="H36" s="220"/>
-      <c r="I36" s="220"/>
-      <c r="J36" s="220"/>
-      <c r="K36" s="220"/>
-      <c r="L36" s="220"/>
-      <c r="M36" s="220"/>
-      <c r="N36" s="220"/>
-      <c r="O36" s="220"/>
-      <c r="P36" s="220"/>
-      <c r="Q36" s="220"/>
+      <c r="C36" s="248"/>
+      <c r="D36" s="248"/>
+      <c r="E36" s="248"/>
+      <c r="F36" s="248"/>
+      <c r="G36" s="248"/>
+      <c r="H36" s="248"/>
+      <c r="I36" s="248"/>
+      <c r="J36" s="248"/>
+      <c r="K36" s="248"/>
+      <c r="L36" s="248"/>
+      <c r="M36" s="248"/>
+      <c r="N36" s="248"/>
+      <c r="O36" s="248"/>
+      <c r="P36" s="248"/>
+      <c r="Q36" s="248"/>
       <c r="R36" s="58"/>
     </row>
     <row r="37" spans="1:18" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="217"/>
+      <c r="A37" s="272"/>
       <c r="B37" s="59"/>
       <c r="C37" s="24"/>
       <c r="D37" s="24"/>
@@ -5572,337 +5574,337 @@
       <c r="R37" s="25"/>
     </row>
     <row r="38" spans="1:18" s="8" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="217"/>
-      <c r="B38" s="221" t="s">
+      <c r="A38" s="272"/>
+      <c r="B38" s="249" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" s="250"/>
+      <c r="D38" s="250"/>
+      <c r="E38" s="250"/>
+      <c r="F38" s="250"/>
+      <c r="G38" s="250"/>
+      <c r="H38" s="250"/>
+      <c r="I38" s="250"/>
+      <c r="J38" s="250"/>
+      <c r="K38" s="250"/>
+      <c r="L38" s="250"/>
+      <c r="M38" s="250"/>
+      <c r="N38" s="250"/>
+      <c r="O38" s="250"/>
+      <c r="P38" s="250"/>
+      <c r="Q38" s="250"/>
+      <c r="R38" s="251"/>
+    </row>
+    <row r="39" spans="1:18" s="61" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="272"/>
+      <c r="B39" s="261" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" s="252" t="s">
+        <v>72</v>
+      </c>
+      <c r="D39" s="253"/>
+      <c r="E39" s="254"/>
+      <c r="F39" s="252" t="s">
+        <v>73</v>
+      </c>
+      <c r="G39" s="254"/>
+      <c r="H39" s="258" t="s">
+        <v>74</v>
+      </c>
+      <c r="I39" s="259"/>
+      <c r="J39" s="259"/>
+      <c r="K39" s="260"/>
+      <c r="L39" s="252" t="s">
+        <v>75</v>
+      </c>
+      <c r="M39" s="253"/>
+      <c r="N39" s="254"/>
+      <c r="O39" s="252" t="s">
+        <v>76</v>
+      </c>
+      <c r="P39" s="254"/>
+      <c r="Q39" s="263" t="s">
         <v>77</v>
       </c>
-      <c r="C38" s="222"/>
-      <c r="D38" s="222"/>
-      <c r="E38" s="222"/>
-      <c r="F38" s="222"/>
-      <c r="G38" s="222"/>
-      <c r="H38" s="222"/>
-      <c r="I38" s="222"/>
-      <c r="J38" s="222"/>
-      <c r="K38" s="222"/>
-      <c r="L38" s="222"/>
-      <c r="M38" s="222"/>
-      <c r="N38" s="222"/>
-      <c r="O38" s="222"/>
-      <c r="P38" s="222"/>
-      <c r="Q38" s="222"/>
-      <c r="R38" s="223"/>
-    </row>
-    <row r="39" spans="1:18" s="61" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="217"/>
-      <c r="B39" s="233" t="s">
+      <c r="R39" s="265" t="s">
         <v>78</v>
       </c>
-      <c r="C39" s="224" t="s">
+    </row>
+    <row r="40" spans="1:18" s="61" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="272"/>
+      <c r="B40" s="262"/>
+      <c r="C40" s="255"/>
+      <c r="D40" s="256"/>
+      <c r="E40" s="257"/>
+      <c r="F40" s="255"/>
+      <c r="G40" s="257"/>
+      <c r="H40" s="258" t="s">
         <v>79</v>
       </c>
-      <c r="D39" s="225"/>
-      <c r="E39" s="226"/>
-      <c r="F39" s="224" t="s">
-        <v>80</v>
-      </c>
-      <c r="G39" s="226"/>
-      <c r="H39" s="230" t="s">
-        <v>81</v>
-      </c>
-      <c r="I39" s="231"/>
-      <c r="J39" s="231"/>
-      <c r="K39" s="232"/>
-      <c r="L39" s="224" t="s">
-        <v>82</v>
-      </c>
-      <c r="M39" s="225"/>
-      <c r="N39" s="226"/>
-      <c r="O39" s="224" t="s">
-        <v>83</v>
-      </c>
-      <c r="P39" s="226"/>
-      <c r="Q39" s="235" t="s">
-        <v>84</v>
-      </c>
-      <c r="R39" s="237" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="40" spans="1:18" s="61" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="217"/>
-      <c r="B40" s="234"/>
-      <c r="C40" s="227"/>
-      <c r="D40" s="228"/>
-      <c r="E40" s="229"/>
-      <c r="F40" s="227"/>
-      <c r="G40" s="229"/>
-      <c r="H40" s="230" t="s">
-        <v>86</v>
-      </c>
-      <c r="I40" s="231"/>
-      <c r="J40" s="231"/>
-      <c r="K40" s="232"/>
-      <c r="L40" s="227"/>
-      <c r="M40" s="228"/>
-      <c r="N40" s="229"/>
-      <c r="O40" s="227"/>
-      <c r="P40" s="229"/>
-      <c r="Q40" s="236"/>
-      <c r="R40" s="238"/>
+      <c r="I40" s="259"/>
+      <c r="J40" s="259"/>
+      <c r="K40" s="260"/>
+      <c r="L40" s="255"/>
+      <c r="M40" s="256"/>
+      <c r="N40" s="257"/>
+      <c r="O40" s="255"/>
+      <c r="P40" s="257"/>
+      <c r="Q40" s="264"/>
+      <c r="R40" s="266"/>
     </row>
     <row r="41" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="217"/>
+      <c r="A41" s="272"/>
       <c r="B41" s="62"/>
-      <c r="C41" s="239"/>
-      <c r="D41" s="239"/>
-      <c r="E41" s="239"/>
-      <c r="F41" s="240"/>
-      <c r="G41" s="240"/>
-      <c r="H41" s="241"/>
-      <c r="I41" s="242"/>
-      <c r="J41" s="242"/>
-      <c r="K41" s="243"/>
-      <c r="L41" s="250"/>
-      <c r="M41" s="250"/>
-      <c r="N41" s="250"/>
-      <c r="O41" s="251"/>
-      <c r="P41" s="252"/>
+      <c r="C41" s="223"/>
+      <c r="D41" s="223"/>
+      <c r="E41" s="223"/>
+      <c r="F41" s="238"/>
+      <c r="G41" s="238"/>
+      <c r="H41" s="239"/>
+      <c r="I41" s="240"/>
+      <c r="J41" s="240"/>
+      <c r="K41" s="241"/>
+      <c r="L41" s="237"/>
+      <c r="M41" s="237"/>
+      <c r="N41" s="237"/>
+      <c r="O41" s="234"/>
+      <c r="P41" s="235"/>
       <c r="Q41" s="64"/>
       <c r="R41" s="65"/>
     </row>
     <row r="42" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="217"/>
+      <c r="A42" s="272"/>
       <c r="B42" s="66"/>
-      <c r="C42" s="239"/>
-      <c r="D42" s="239"/>
-      <c r="E42" s="239"/>
-      <c r="F42" s="253"/>
-      <c r="G42" s="253"/>
-      <c r="H42" s="244"/>
-      <c r="I42" s="245"/>
-      <c r="J42" s="245"/>
-      <c r="K42" s="246"/>
-      <c r="L42" s="250"/>
-      <c r="M42" s="250"/>
-      <c r="N42" s="250"/>
-      <c r="O42" s="251"/>
-      <c r="P42" s="252"/>
+      <c r="C42" s="223"/>
+      <c r="D42" s="223"/>
+      <c r="E42" s="223"/>
+      <c r="F42" s="236"/>
+      <c r="G42" s="236"/>
+      <c r="H42" s="242"/>
+      <c r="I42" s="243"/>
+      <c r="J42" s="243"/>
+      <c r="K42" s="244"/>
+      <c r="L42" s="237"/>
+      <c r="M42" s="237"/>
+      <c r="N42" s="237"/>
+      <c r="O42" s="234"/>
+      <c r="P42" s="235"/>
       <c r="Q42" s="63"/>
       <c r="R42" s="67"/>
     </row>
     <row r="43" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="217"/>
+      <c r="A43" s="272"/>
       <c r="B43" s="66"/>
-      <c r="C43" s="239"/>
-      <c r="D43" s="239"/>
-      <c r="E43" s="239"/>
-      <c r="F43" s="253"/>
-      <c r="G43" s="253"/>
-      <c r="H43" s="244"/>
-      <c r="I43" s="245"/>
-      <c r="J43" s="245"/>
-      <c r="K43" s="246"/>
-      <c r="L43" s="250"/>
-      <c r="M43" s="250"/>
-      <c r="N43" s="250"/>
-      <c r="O43" s="251"/>
-      <c r="P43" s="252"/>
+      <c r="C43" s="223"/>
+      <c r="D43" s="223"/>
+      <c r="E43" s="223"/>
+      <c r="F43" s="236"/>
+      <c r="G43" s="236"/>
+      <c r="H43" s="242"/>
+      <c r="I43" s="243"/>
+      <c r="J43" s="243"/>
+      <c r="K43" s="244"/>
+      <c r="L43" s="237"/>
+      <c r="M43" s="237"/>
+      <c r="N43" s="237"/>
+      <c r="O43" s="234"/>
+      <c r="P43" s="235"/>
       <c r="Q43" s="63"/>
       <c r="R43" s="67"/>
     </row>
     <row r="44" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="217"/>
+      <c r="A44" s="272"/>
       <c r="B44" s="66"/>
-      <c r="C44" s="239"/>
-      <c r="D44" s="239"/>
-      <c r="E44" s="239"/>
-      <c r="F44" s="253"/>
-      <c r="G44" s="253"/>
-      <c r="H44" s="244"/>
-      <c r="I44" s="245"/>
-      <c r="J44" s="245"/>
-      <c r="K44" s="246"/>
-      <c r="L44" s="250"/>
-      <c r="M44" s="250"/>
-      <c r="N44" s="250"/>
-      <c r="O44" s="251"/>
-      <c r="P44" s="252"/>
+      <c r="C44" s="223"/>
+      <c r="D44" s="223"/>
+      <c r="E44" s="223"/>
+      <c r="F44" s="236"/>
+      <c r="G44" s="236"/>
+      <c r="H44" s="242"/>
+      <c r="I44" s="243"/>
+      <c r="J44" s="243"/>
+      <c r="K44" s="244"/>
+      <c r="L44" s="237"/>
+      <c r="M44" s="237"/>
+      <c r="N44" s="237"/>
+      <c r="O44" s="234"/>
+      <c r="P44" s="235"/>
       <c r="Q44" s="63"/>
       <c r="R44" s="67"/>
     </row>
     <row r="45" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="217"/>
+      <c r="A45" s="272"/>
       <c r="B45" s="66"/>
-      <c r="C45" s="239"/>
-      <c r="D45" s="239"/>
-      <c r="E45" s="239"/>
-      <c r="F45" s="253"/>
-      <c r="G45" s="253"/>
-      <c r="H45" s="244"/>
-      <c r="I45" s="245"/>
-      <c r="J45" s="245"/>
-      <c r="K45" s="246"/>
-      <c r="L45" s="250"/>
-      <c r="M45" s="250"/>
-      <c r="N45" s="250"/>
-      <c r="O45" s="251"/>
-      <c r="P45" s="252"/>
+      <c r="C45" s="223"/>
+      <c r="D45" s="223"/>
+      <c r="E45" s="223"/>
+      <c r="F45" s="236"/>
+      <c r="G45" s="236"/>
+      <c r="H45" s="242"/>
+      <c r="I45" s="243"/>
+      <c r="J45" s="243"/>
+      <c r="K45" s="244"/>
+      <c r="L45" s="237"/>
+      <c r="M45" s="237"/>
+      <c r="N45" s="237"/>
+      <c r="O45" s="234"/>
+      <c r="P45" s="235"/>
       <c r="Q45" s="63"/>
       <c r="R45" s="67"/>
     </row>
     <row r="46" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="217"/>
+      <c r="A46" s="272"/>
       <c r="B46" s="66"/>
-      <c r="C46" s="239"/>
-      <c r="D46" s="239"/>
-      <c r="E46" s="239"/>
-      <c r="F46" s="253"/>
-      <c r="G46" s="253"/>
-      <c r="H46" s="244"/>
-      <c r="I46" s="245"/>
-      <c r="J46" s="245"/>
-      <c r="K46" s="246"/>
-      <c r="L46" s="250"/>
-      <c r="M46" s="250"/>
-      <c r="N46" s="250"/>
-      <c r="O46" s="251"/>
-      <c r="P46" s="252"/>
+      <c r="C46" s="223"/>
+      <c r="D46" s="223"/>
+      <c r="E46" s="223"/>
+      <c r="F46" s="236"/>
+      <c r="G46" s="236"/>
+      <c r="H46" s="242"/>
+      <c r="I46" s="243"/>
+      <c r="J46" s="243"/>
+      <c r="K46" s="244"/>
+      <c r="L46" s="237"/>
+      <c r="M46" s="237"/>
+      <c r="N46" s="237"/>
+      <c r="O46" s="234"/>
+      <c r="P46" s="235"/>
       <c r="Q46" s="63"/>
       <c r="R46" s="67"/>
     </row>
     <row r="47" spans="1:18" s="61" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="217"/>
+      <c r="A47" s="272"/>
       <c r="B47" s="66"/>
-      <c r="C47" s="239"/>
-      <c r="D47" s="239"/>
-      <c r="E47" s="239"/>
-      <c r="F47" s="253"/>
-      <c r="G47" s="253"/>
-      <c r="H47" s="244"/>
-      <c r="I47" s="245"/>
-      <c r="J47" s="245"/>
-      <c r="K47" s="246"/>
-      <c r="L47" s="250"/>
-      <c r="M47" s="250"/>
-      <c r="N47" s="250"/>
-      <c r="O47" s="251"/>
-      <c r="P47" s="252"/>
+      <c r="C47" s="223"/>
+      <c r="D47" s="223"/>
+      <c r="E47" s="223"/>
+      <c r="F47" s="236"/>
+      <c r="G47" s="236"/>
+      <c r="H47" s="242"/>
+      <c r="I47" s="243"/>
+      <c r="J47" s="243"/>
+      <c r="K47" s="244"/>
+      <c r="L47" s="237"/>
+      <c r="M47" s="237"/>
+      <c r="N47" s="237"/>
+      <c r="O47" s="234"/>
+      <c r="P47" s="235"/>
       <c r="Q47" s="63"/>
       <c r="R47" s="67"/>
     </row>
     <row r="48" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="217"/>
+      <c r="A48" s="272"/>
       <c r="B48" s="68"/>
-      <c r="C48" s="239"/>
-      <c r="D48" s="239"/>
-      <c r="E48" s="239"/>
-      <c r="F48" s="254"/>
-      <c r="G48" s="254"/>
-      <c r="H48" s="244"/>
-      <c r="I48" s="245"/>
-      <c r="J48" s="245"/>
-      <c r="K48" s="246"/>
-      <c r="L48" s="255"/>
-      <c r="M48" s="255"/>
-      <c r="N48" s="255"/>
-      <c r="O48" s="251"/>
-      <c r="P48" s="252"/>
+      <c r="C48" s="223"/>
+      <c r="D48" s="223"/>
+      <c r="E48" s="223"/>
+      <c r="F48" s="232"/>
+      <c r="G48" s="232"/>
+      <c r="H48" s="242"/>
+      <c r="I48" s="243"/>
+      <c r="J48" s="243"/>
+      <c r="K48" s="244"/>
+      <c r="L48" s="233"/>
+      <c r="M48" s="233"/>
+      <c r="N48" s="233"/>
+      <c r="O48" s="234"/>
+      <c r="P48" s="235"/>
       <c r="Q48" s="69"/>
       <c r="R48" s="70"/>
     </row>
     <row r="49" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="217"/>
+      <c r="A49" s="272"/>
       <c r="B49" s="68"/>
-      <c r="C49" s="239"/>
-      <c r="D49" s="239"/>
-      <c r="E49" s="239"/>
-      <c r="F49" s="254"/>
-      <c r="G49" s="254"/>
-      <c r="H49" s="244"/>
-      <c r="I49" s="245"/>
-      <c r="J49" s="245"/>
-      <c r="K49" s="246"/>
-      <c r="L49" s="255"/>
-      <c r="M49" s="255"/>
-      <c r="N49" s="255"/>
-      <c r="O49" s="251"/>
-      <c r="P49" s="252"/>
+      <c r="C49" s="223"/>
+      <c r="D49" s="223"/>
+      <c r="E49" s="223"/>
+      <c r="F49" s="232"/>
+      <c r="G49" s="232"/>
+      <c r="H49" s="242"/>
+      <c r="I49" s="243"/>
+      <c r="J49" s="243"/>
+      <c r="K49" s="244"/>
+      <c r="L49" s="233"/>
+      <c r="M49" s="233"/>
+      <c r="N49" s="233"/>
+      <c r="O49" s="234"/>
+      <c r="P49" s="235"/>
       <c r="Q49" s="69"/>
       <c r="R49" s="70"/>
     </row>
     <row r="50" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="217"/>
+      <c r="A50" s="272"/>
       <c r="B50" s="66"/>
-      <c r="C50" s="239"/>
-      <c r="D50" s="239"/>
-      <c r="E50" s="239"/>
-      <c r="F50" s="253"/>
-      <c r="G50" s="253"/>
-      <c r="H50" s="244"/>
-      <c r="I50" s="245"/>
-      <c r="J50" s="245"/>
-      <c r="K50" s="246"/>
-      <c r="L50" s="250"/>
-      <c r="M50" s="250"/>
-      <c r="N50" s="250"/>
-      <c r="O50" s="251"/>
-      <c r="P50" s="252"/>
+      <c r="C50" s="223"/>
+      <c r="D50" s="223"/>
+      <c r="E50" s="223"/>
+      <c r="F50" s="236"/>
+      <c r="G50" s="236"/>
+      <c r="H50" s="242"/>
+      <c r="I50" s="243"/>
+      <c r="J50" s="243"/>
+      <c r="K50" s="244"/>
+      <c r="L50" s="237"/>
+      <c r="M50" s="237"/>
+      <c r="N50" s="237"/>
+      <c r="O50" s="234"/>
+      <c r="P50" s="235"/>
       <c r="Q50" s="63"/>
       <c r="R50" s="67"/>
     </row>
     <row r="51" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="217"/>
+      <c r="A51" s="272"/>
       <c r="B51" s="66"/>
-      <c r="C51" s="239"/>
-      <c r="D51" s="239"/>
-      <c r="E51" s="239"/>
-      <c r="F51" s="253"/>
-      <c r="G51" s="253"/>
-      <c r="H51" s="244"/>
-      <c r="I51" s="245"/>
-      <c r="J51" s="245"/>
-      <c r="K51" s="246"/>
-      <c r="L51" s="250"/>
-      <c r="M51" s="250"/>
-      <c r="N51" s="250"/>
-      <c r="O51" s="251"/>
-      <c r="P51" s="252"/>
+      <c r="C51" s="223"/>
+      <c r="D51" s="223"/>
+      <c r="E51" s="223"/>
+      <c r="F51" s="236"/>
+      <c r="G51" s="236"/>
+      <c r="H51" s="242"/>
+      <c r="I51" s="243"/>
+      <c r="J51" s="243"/>
+      <c r="K51" s="244"/>
+      <c r="L51" s="237"/>
+      <c r="M51" s="237"/>
+      <c r="N51" s="237"/>
+      <c r="O51" s="234"/>
+      <c r="P51" s="235"/>
       <c r="Q51" s="63"/>
       <c r="R51" s="67"/>
     </row>
     <row r="52" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="217"/>
+      <c r="A52" s="272"/>
       <c r="B52" s="71"/>
-      <c r="C52" s="239"/>
-      <c r="D52" s="239"/>
-      <c r="E52" s="239"/>
-      <c r="F52" s="256"/>
-      <c r="G52" s="256"/>
-      <c r="H52" s="247"/>
-      <c r="I52" s="248"/>
-      <c r="J52" s="248"/>
-      <c r="K52" s="249"/>
-      <c r="L52" s="257"/>
-      <c r="M52" s="257"/>
-      <c r="N52" s="257"/>
-      <c r="O52" s="258"/>
-      <c r="P52" s="259"/>
+      <c r="C52" s="223"/>
+      <c r="D52" s="223"/>
+      <c r="E52" s="223"/>
+      <c r="F52" s="224"/>
+      <c r="G52" s="224"/>
+      <c r="H52" s="245"/>
+      <c r="I52" s="246"/>
+      <c r="J52" s="246"/>
+      <c r="K52" s="247"/>
+      <c r="L52" s="225"/>
+      <c r="M52" s="225"/>
+      <c r="N52" s="225"/>
+      <c r="O52" s="226"/>
+      <c r="P52" s="227"/>
       <c r="Q52" s="72"/>
       <c r="R52" s="73"/>
     </row>
     <row r="53" spans="1:18" s="61" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="217"/>
+      <c r="A53" s="272"/>
       <c r="B53" s="74"/>
-      <c r="C53" s="260" t="s">
-        <v>87</v>
-      </c>
-      <c r="D53" s="260"/>
-      <c r="E53" s="260"/>
+      <c r="C53" s="228" t="s">
+        <v>80</v>
+      </c>
+      <c r="D53" s="228"/>
+      <c r="E53" s="228"/>
       <c r="F53" s="75"/>
-      <c r="G53" s="261"/>
-      <c r="H53" s="261"/>
-      <c r="I53" s="261"/>
+      <c r="G53" s="229"/>
+      <c r="H53" s="229"/>
+      <c r="I53" s="229"/>
       <c r="J53" s="76"/>
       <c r="K53" s="77"/>
       <c r="L53" s="77"/>
@@ -5914,14 +5916,14 @@
       <c r="R53" s="79"/>
     </row>
     <row r="54" spans="1:18" s="61" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="218"/>
+      <c r="A54" s="273"/>
       <c r="B54" s="80"/>
-      <c r="C54" s="262"/>
-      <c r="D54" s="262"/>
-      <c r="E54" s="262"/>
-      <c r="F54" s="262"/>
-      <c r="G54" s="263"/>
-      <c r="H54" s="263"/>
+      <c r="C54" s="230"/>
+      <c r="D54" s="230"/>
+      <c r="E54" s="230"/>
+      <c r="F54" s="230"/>
+      <c r="G54" s="231"/>
+      <c r="H54" s="231"/>
       <c r="I54" s="82"/>
       <c r="J54" s="82"/>
       <c r="K54" s="81"/>
@@ -5935,177 +5937,177 @@
     </row>
     <row r="55" spans="1:18" s="4" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="R55" s="84" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
     </row>
     <row r="56" spans="1:18" s="4" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="264" t="s">
-        <v>89</v>
-      </c>
-      <c r="C57" s="265"/>
-      <c r="D57" s="266"/>
-      <c r="E57" s="264" t="s">
-        <v>90</v>
-      </c>
-      <c r="F57" s="265"/>
-      <c r="G57" s="266"/>
-      <c r="H57" s="264" t="s">
-        <v>91</v>
-      </c>
-      <c r="I57" s="265"/>
-      <c r="J57" s="266"/>
-      <c r="K57" s="264" t="s">
-        <v>92</v>
-      </c>
-      <c r="L57" s="265"/>
-      <c r="M57" s="266"/>
-      <c r="N57" s="264" t="s">
-        <v>93</v>
-      </c>
-      <c r="O57" s="265"/>
-      <c r="P57" s="266"/>
+      <c r="B57" s="214" t="s">
+        <v>82</v>
+      </c>
+      <c r="C57" s="215"/>
+      <c r="D57" s="216"/>
+      <c r="E57" s="214" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" s="215"/>
+      <c r="G57" s="216"/>
+      <c r="H57" s="214" t="s">
+        <v>84</v>
+      </c>
+      <c r="I57" s="215"/>
+      <c r="J57" s="216"/>
+      <c r="K57" s="214" t="s">
+        <v>85</v>
+      </c>
+      <c r="L57" s="215"/>
+      <c r="M57" s="216"/>
+      <c r="N57" s="214" t="s">
+        <v>86</v>
+      </c>
+      <c r="O57" s="215"/>
+      <c r="P57" s="216"/>
     </row>
     <row r="58" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="267"/>
-      <c r="C58" s="268"/>
-      <c r="D58" s="269"/>
-      <c r="E58" s="267"/>
-      <c r="F58" s="268"/>
-      <c r="G58" s="269"/>
-      <c r="H58" s="267"/>
-      <c r="I58" s="268"/>
-      <c r="J58" s="269"/>
-      <c r="K58" s="267"/>
-      <c r="L58" s="268"/>
-      <c r="M58" s="269"/>
-      <c r="N58" s="267"/>
-      <c r="O58" s="268"/>
-      <c r="P58" s="269"/>
+      <c r="B58" s="217"/>
+      <c r="C58" s="218"/>
+      <c r="D58" s="219"/>
+      <c r="E58" s="217"/>
+      <c r="F58" s="218"/>
+      <c r="G58" s="219"/>
+      <c r="H58" s="217"/>
+      <c r="I58" s="218"/>
+      <c r="J58" s="219"/>
+      <c r="K58" s="217"/>
+      <c r="L58" s="218"/>
+      <c r="M58" s="219"/>
+      <c r="N58" s="217"/>
+      <c r="O58" s="218"/>
+      <c r="P58" s="219"/>
     </row>
     <row r="59" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="270"/>
-      <c r="C59" s="271"/>
-      <c r="D59" s="272"/>
-      <c r="E59" s="270"/>
-      <c r="F59" s="271"/>
-      <c r="G59" s="272"/>
-      <c r="H59" s="270"/>
-      <c r="I59" s="271"/>
-      <c r="J59" s="272"/>
-      <c r="K59" s="270"/>
-      <c r="L59" s="271"/>
-      <c r="M59" s="272"/>
-      <c r="N59" s="270"/>
-      <c r="O59" s="271"/>
-      <c r="P59" s="272"/>
+      <c r="B59" s="220"/>
+      <c r="C59" s="221"/>
+      <c r="D59" s="222"/>
+      <c r="E59" s="220"/>
+      <c r="F59" s="221"/>
+      <c r="G59" s="222"/>
+      <c r="H59" s="220"/>
+      <c r="I59" s="221"/>
+      <c r="J59" s="222"/>
+      <c r="K59" s="220"/>
+      <c r="L59" s="221"/>
+      <c r="M59" s="222"/>
+      <c r="N59" s="220"/>
+      <c r="O59" s="221"/>
+      <c r="P59" s="222"/>
     </row>
     <row r="60" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="85" t="s">
-        <v>94</v>
-      </c>
-      <c r="C60" s="273"/>
-      <c r="D60" s="274"/>
+        <v>87</v>
+      </c>
+      <c r="C60" s="212"/>
+      <c r="D60" s="213"/>
       <c r="E60" s="85" t="s">
-        <v>94</v>
-      </c>
-      <c r="F60" s="273"/>
-      <c r="G60" s="274"/>
+        <v>87</v>
+      </c>
+      <c r="F60" s="212"/>
+      <c r="G60" s="213"/>
       <c r="H60" s="85" t="s">
-        <v>94</v>
-      </c>
-      <c r="I60" s="273"/>
-      <c r="J60" s="274"/>
+        <v>87</v>
+      </c>
+      <c r="I60" s="212"/>
+      <c r="J60" s="213"/>
       <c r="K60" s="85" t="s">
-        <v>94</v>
-      </c>
-      <c r="L60" s="273"/>
-      <c r="M60" s="274"/>
+        <v>87</v>
+      </c>
+      <c r="L60" s="212"/>
+      <c r="M60" s="213"/>
       <c r="N60" s="85" t="s">
-        <v>94</v>
-      </c>
-      <c r="O60" s="273"/>
-      <c r="P60" s="274"/>
+        <v>87</v>
+      </c>
+      <c r="O60" s="212"/>
+      <c r="P60" s="213"/>
     </row>
     <row r="61" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="264" t="s">
-        <v>95</v>
-      </c>
-      <c r="C61" s="265"/>
-      <c r="D61" s="266"/>
-      <c r="E61" s="264" t="s">
-        <v>96</v>
-      </c>
-      <c r="F61" s="265"/>
-      <c r="G61" s="266"/>
-      <c r="H61" s="264" t="s">
-        <v>95</v>
-      </c>
-      <c r="I61" s="265"/>
-      <c r="J61" s="266"/>
-      <c r="K61" s="264" t="s">
-        <v>96</v>
-      </c>
-      <c r="L61" s="265"/>
-      <c r="M61" s="266"/>
-      <c r="N61" s="264" t="s">
-        <v>96</v>
-      </c>
-      <c r="O61" s="265"/>
-      <c r="P61" s="266"/>
+      <c r="B61" s="214" t="s">
+        <v>88</v>
+      </c>
+      <c r="C61" s="215"/>
+      <c r="D61" s="216"/>
+      <c r="E61" s="214" t="s">
+        <v>89</v>
+      </c>
+      <c r="F61" s="215"/>
+      <c r="G61" s="216"/>
+      <c r="H61" s="214" t="s">
+        <v>88</v>
+      </c>
+      <c r="I61" s="215"/>
+      <c r="J61" s="216"/>
+      <c r="K61" s="214" t="s">
+        <v>89</v>
+      </c>
+      <c r="L61" s="215"/>
+      <c r="M61" s="216"/>
+      <c r="N61" s="214" t="s">
+        <v>89</v>
+      </c>
+      <c r="O61" s="215"/>
+      <c r="P61" s="216"/>
     </row>
     <row r="62" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="63" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="264" t="s">
-        <v>97</v>
-      </c>
-      <c r="C63" s="265"/>
-      <c r="D63" s="266"/>
-      <c r="E63" s="264" t="s">
-        <v>98</v>
-      </c>
-      <c r="F63" s="265"/>
-      <c r="G63" s="266"/>
+      <c r="B63" s="214" t="s">
+        <v>90</v>
+      </c>
+      <c r="C63" s="215"/>
+      <c r="D63" s="216"/>
+      <c r="E63" s="214" t="s">
+        <v>91</v>
+      </c>
+      <c r="F63" s="215"/>
+      <c r="G63" s="216"/>
     </row>
     <row r="64" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="267"/>
-      <c r="C64" s="268"/>
-      <c r="D64" s="269"/>
-      <c r="E64" s="267"/>
-      <c r="F64" s="268"/>
-      <c r="G64" s="269"/>
+      <c r="B64" s="217"/>
+      <c r="C64" s="218"/>
+      <c r="D64" s="219"/>
+      <c r="E64" s="217"/>
+      <c r="F64" s="218"/>
+      <c r="G64" s="219"/>
     </row>
     <row r="65" spans="2:7" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="270"/>
-      <c r="C65" s="271"/>
-      <c r="D65" s="272"/>
-      <c r="E65" s="270"/>
-      <c r="F65" s="271"/>
-      <c r="G65" s="272"/>
+      <c r="B65" s="220"/>
+      <c r="C65" s="221"/>
+      <c r="D65" s="222"/>
+      <c r="E65" s="220"/>
+      <c r="F65" s="221"/>
+      <c r="G65" s="222"/>
     </row>
     <row r="66" spans="2:7" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="85" t="s">
-        <v>94</v>
-      </c>
-      <c r="C66" s="273"/>
-      <c r="D66" s="274"/>
+        <v>87</v>
+      </c>
+      <c r="C66" s="212"/>
+      <c r="D66" s="213"/>
       <c r="E66" s="85" t="s">
-        <v>94</v>
-      </c>
-      <c r="F66" s="273"/>
-      <c r="G66" s="274"/>
+        <v>87</v>
+      </c>
+      <c r="F66" s="212"/>
+      <c r="G66" s="213"/>
     </row>
     <row r="67" spans="2:7" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="264" t="s">
-        <v>96</v>
-      </c>
-      <c r="C67" s="265"/>
-      <c r="D67" s="266"/>
-      <c r="E67" s="264" t="s">
-        <v>96</v>
-      </c>
-      <c r="F67" s="265"/>
-      <c r="G67" s="266"/>
+      <c r="B67" s="214" t="s">
+        <v>89</v>
+      </c>
+      <c r="C67" s="215"/>
+      <c r="D67" s="216"/>
+      <c r="E67" s="214" t="s">
+        <v>89</v>
+      </c>
+      <c r="F67" s="215"/>
+      <c r="G67" s="216"/>
     </row>
     <row r="68" spans="2:7" s="4" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="69" spans="2:7" s="4" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6602,63 +6604,46 @@
     <row r="560" s="86" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="121">
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="B67:D67"/>
-    <mergeCell ref="E67:G67"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="N61:P61"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="E63:G63"/>
-    <mergeCell ref="B64:D65"/>
-    <mergeCell ref="E64:G65"/>
-    <mergeCell ref="B58:D59"/>
-    <mergeCell ref="E58:G59"/>
-    <mergeCell ref="H58:J59"/>
-    <mergeCell ref="K58:M59"/>
-    <mergeCell ref="N58:P59"/>
-    <mergeCell ref="C60:D60"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="L60:M60"/>
-    <mergeCell ref="O60:P60"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="L52:N52"/>
-    <mergeCell ref="O52:P52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="G53:I53"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="G54:H54"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="H57:J57"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="N57:P57"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="L49:N49"/>
-    <mergeCell ref="O49:P49"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="L50:N50"/>
-    <mergeCell ref="O50:P50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="L51:N51"/>
-    <mergeCell ref="O51:P51"/>
-    <mergeCell ref="O46:P46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="O47:P47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="L48:N48"/>
-    <mergeCell ref="O48:P48"/>
+    <mergeCell ref="L1:R1"/>
+    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="A3:A54"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="C21:Q21"/>
+    <mergeCell ref="C22:Q22"/>
+    <mergeCell ref="C23:Q23"/>
+    <mergeCell ref="C24:Q24"/>
+    <mergeCell ref="C25:Q25"/>
+    <mergeCell ref="C26:Q26"/>
+    <mergeCell ref="C27:Q27"/>
+    <mergeCell ref="C28:Q28"/>
+    <mergeCell ref="C32:Q32"/>
+    <mergeCell ref="C33:Q33"/>
+    <mergeCell ref="C34:Q34"/>
+    <mergeCell ref="C35:Q35"/>
+    <mergeCell ref="C36:Q36"/>
+    <mergeCell ref="B38:R38"/>
+    <mergeCell ref="C39:E40"/>
+    <mergeCell ref="F39:G40"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="L39:N40"/>
+    <mergeCell ref="O39:P40"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="H40:K40"/>
+    <mergeCell ref="Q39:Q40"/>
+    <mergeCell ref="R39:R40"/>
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="F41:G41"/>
     <mergeCell ref="H41:K52"/>
@@ -6683,46 +6668,63 @@
     <mergeCell ref="C46:E46"/>
     <mergeCell ref="F46:G46"/>
     <mergeCell ref="L46:N46"/>
-    <mergeCell ref="C28:Q28"/>
-    <mergeCell ref="C32:Q32"/>
-    <mergeCell ref="C33:Q33"/>
-    <mergeCell ref="C34:Q34"/>
-    <mergeCell ref="C35:Q35"/>
-    <mergeCell ref="C36:Q36"/>
-    <mergeCell ref="B38:R38"/>
-    <mergeCell ref="C39:E40"/>
-    <mergeCell ref="F39:G40"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="L39:N40"/>
-    <mergeCell ref="O39:P40"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="H40:K40"/>
-    <mergeCell ref="Q39:Q40"/>
-    <mergeCell ref="R39:R40"/>
-    <mergeCell ref="L1:R1"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="A3:A54"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="G7:J7"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="G9:J9"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="G11:J11"/>
-    <mergeCell ref="G12:J12"/>
-    <mergeCell ref="G13:J13"/>
-    <mergeCell ref="G14:J14"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="C21:Q21"/>
-    <mergeCell ref="C22:Q22"/>
-    <mergeCell ref="C23:Q23"/>
-    <mergeCell ref="C24:Q24"/>
-    <mergeCell ref="C25:Q25"/>
-    <mergeCell ref="C26:Q26"/>
-    <mergeCell ref="C27:Q27"/>
+    <mergeCell ref="O46:P46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="L47:N47"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="L48:N48"/>
+    <mergeCell ref="O48:P48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="L49:N49"/>
+    <mergeCell ref="O49:P49"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="L50:N50"/>
+    <mergeCell ref="O50:P50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="L51:N51"/>
+    <mergeCell ref="O51:P51"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="L52:N52"/>
+    <mergeCell ref="O52:P52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="G53:I53"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="G54:H54"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="H57:J57"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="N57:P57"/>
+    <mergeCell ref="B58:D59"/>
+    <mergeCell ref="E58:G59"/>
+    <mergeCell ref="H58:J59"/>
+    <mergeCell ref="K58:M59"/>
+    <mergeCell ref="N58:P59"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="L60:M60"/>
+    <mergeCell ref="O60:P60"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="B67:D67"/>
+    <mergeCell ref="E67:G67"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="N61:P61"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="E63:G63"/>
+    <mergeCell ref="B64:D65"/>
+    <mergeCell ref="E64:G65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>

<commit_message>
Update report.xlsx with new data
</commit_message>
<xml_diff>
--- a/src/assets/excel/report.xlsx
+++ b/src/assets/excel/report.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEEADF01-824D-4BCA-942C-660C87189E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE299FB4-0FEF-4C76-9137-1074EE0CAB38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4890" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="4" r:id="rId1"/>
@@ -282,9 +282,6 @@
     <t xml:space="preserve">After test disposition : </t>
   </si>
   <si>
-    <t>QEF4200.I7.Relia.11.1-19</t>
-  </si>
-  <si>
     <t>REQUEST</t>
   </si>
   <si>
@@ -350,6 +347,9 @@
     <t>Ms.Khachinrat D.
 Ms.Sumitra S.
 Mr.Watcharapan P.</t>
+  </si>
+  <si>
+    <t>QEF4200.I7.Relia.11.4-10</t>
   </si>
 </sst>
 </file>
@@ -1595,132 +1595,6 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="16" fontId="23" fillId="2" borderId="23" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1738,6 +1612,63 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1789,72 +1720,237 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="11" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="11" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -1879,134 +1975,38 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="11" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="11" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2441,9 +2441,9 @@
       <c r="AB1" s="89"/>
     </row>
     <row r="2" spans="1:28" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="150"/>
-      <c r="B2" s="151"/>
-      <c r="C2" s="151"/>
+      <c r="A2" s="148"/>
+      <c r="B2" s="149"/>
+      <c r="C2" s="149"/>
       <c r="D2" s="91"/>
       <c r="E2" s="91"/>
       <c r="F2" s="91"/>
@@ -2452,12 +2452,12 @@
       <c r="I2" s="91"/>
       <c r="J2" s="91"/>
       <c r="K2" s="91"/>
-      <c r="L2" s="151"/>
-      <c r="M2" s="151"/>
-      <c r="N2" s="151"/>
-      <c r="O2" s="151"/>
-      <c r="P2" s="151"/>
-      <c r="Q2" s="151"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
+      <c r="N2" s="149"/>
+      <c r="O2" s="149"/>
+      <c r="P2" s="149"/>
+      <c r="Q2" s="149"/>
       <c r="R2" s="90"/>
       <c r="S2" s="90"/>
       <c r="T2" s="90"/>
@@ -2471,9 +2471,9 @@
       <c r="AB2" s="92"/>
     </row>
     <row r="3" spans="1:28" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="153"/>
-      <c r="B3" s="154"/>
-      <c r="C3" s="154"/>
+      <c r="A3" s="150"/>
+      <c r="B3" s="151"/>
+      <c r="C3" s="151"/>
       <c r="D3" s="93"/>
       <c r="E3" s="93"/>
       <c r="F3" s="94"/>
@@ -2482,12 +2482,12 @@
       <c r="I3" s="94"/>
       <c r="J3" s="94"/>
       <c r="K3" s="94"/>
-      <c r="L3" s="157"/>
-      <c r="M3" s="157"/>
-      <c r="N3" s="157"/>
-      <c r="O3" s="157"/>
-      <c r="P3" s="157"/>
-      <c r="Q3" s="157"/>
+      <c r="L3" s="153"/>
+      <c r="M3" s="153"/>
+      <c r="N3" s="153"/>
+      <c r="O3" s="153"/>
+      <c r="P3" s="153"/>
+      <c r="Q3" s="153"/>
       <c r="R3" s="95"/>
       <c r="S3" s="95"/>
       <c r="T3" s="95"/>
@@ -2497,93 +2497,93 @@
       <c r="AB3" s="96"/>
     </row>
     <row r="4" spans="1:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="153"/>
-      <c r="B4" s="154"/>
-      <c r="C4" s="154"/>
+      <c r="A4" s="150"/>
+      <c r="B4" s="151"/>
+      <c r="C4" s="151"/>
       <c r="E4" s="97"/>
-      <c r="F4" s="151" t="s">
+      <c r="F4" s="149" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="151"/>
-      <c r="H4" s="151"/>
-      <c r="I4" s="151"/>
-      <c r="J4" s="151"/>
-      <c r="K4" s="151"/>
-      <c r="L4" s="151"/>
-      <c r="M4" s="151"/>
-      <c r="N4" s="151"/>
-      <c r="O4" s="151"/>
-      <c r="P4" s="151"/>
-      <c r="Q4" s="151"/>
-      <c r="R4" s="151"/>
-      <c r="S4" s="151"/>
-      <c r="T4" s="151"/>
-      <c r="U4" s="151"/>
-      <c r="V4" s="151"/>
-      <c r="W4" s="151"/>
+      <c r="G4" s="149"/>
+      <c r="H4" s="149"/>
+      <c r="I4" s="149"/>
+      <c r="J4" s="149"/>
+      <c r="K4" s="149"/>
+      <c r="L4" s="149"/>
+      <c r="M4" s="149"/>
+      <c r="N4" s="149"/>
+      <c r="O4" s="149"/>
+      <c r="P4" s="149"/>
+      <c r="Q4" s="149"/>
+      <c r="R4" s="149"/>
+      <c r="S4" s="149"/>
+      <c r="T4" s="149"/>
+      <c r="U4" s="149"/>
+      <c r="V4" s="149"/>
+      <c r="W4" s="149"/>
       <c r="AB4" s="96"/>
     </row>
     <row r="5" spans="1:28" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="156"/>
-      <c r="B5" s="157"/>
-      <c r="C5" s="157"/>
-      <c r="D5" s="206"/>
-      <c r="E5" s="206"/>
-      <c r="F5" s="206"/>
-      <c r="G5" s="206"/>
-      <c r="H5" s="206"/>
-      <c r="I5" s="206"/>
-      <c r="J5" s="206"/>
-      <c r="K5" s="206"/>
-      <c r="L5" s="206"/>
-      <c r="M5" s="206"/>
-      <c r="N5" s="206"/>
-      <c r="O5" s="206"/>
-      <c r="P5" s="206"/>
-      <c r="Q5" s="206"/>
-      <c r="R5" s="206"/>
-      <c r="S5" s="206"/>
-      <c r="T5" s="206"/>
-      <c r="U5" s="206"/>
-      <c r="V5" s="206"/>
-      <c r="W5" s="206"/>
-      <c r="X5" s="206"/>
-      <c r="Y5" s="206"/>
-      <c r="Z5" s="206"/>
-      <c r="AA5" s="206"/>
-      <c r="AB5" s="207"/>
+      <c r="A5" s="152"/>
+      <c r="B5" s="153"/>
+      <c r="C5" s="153"/>
+      <c r="D5" s="154"/>
+      <c r="E5" s="154"/>
+      <c r="F5" s="154"/>
+      <c r="G5" s="154"/>
+      <c r="H5" s="154"/>
+      <c r="I5" s="154"/>
+      <c r="J5" s="154"/>
+      <c r="K5" s="154"/>
+      <c r="L5" s="154"/>
+      <c r="M5" s="154"/>
+      <c r="N5" s="154"/>
+      <c r="O5" s="154"/>
+      <c r="P5" s="154"/>
+      <c r="Q5" s="154"/>
+      <c r="R5" s="154"/>
+      <c r="S5" s="154"/>
+      <c r="T5" s="154"/>
+      <c r="U5" s="154"/>
+      <c r="V5" s="154"/>
+      <c r="W5" s="154"/>
+      <c r="X5" s="154"/>
+      <c r="Y5" s="154"/>
+      <c r="Z5" s="154"/>
+      <c r="AA5" s="154"/>
+      <c r="AB5" s="155"/>
     </row>
     <row r="6" spans="1:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="208" t="s">
+      <c r="A6" s="156" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="209"/>
-      <c r="C6" s="209"/>
-      <c r="D6" s="209"/>
-      <c r="E6" s="209"/>
-      <c r="F6" s="209"/>
-      <c r="G6" s="210"/>
-      <c r="H6" s="209"/>
-      <c r="I6" s="209"/>
-      <c r="J6" s="209"/>
-      <c r="K6" s="209"/>
-      <c r="L6" s="209"/>
-      <c r="M6" s="209"/>
-      <c r="N6" s="209"/>
-      <c r="O6" s="209"/>
-      <c r="P6" s="209"/>
-      <c r="Q6" s="209"/>
-      <c r="R6" s="209"/>
-      <c r="S6" s="209"/>
-      <c r="T6" s="209"/>
-      <c r="U6" s="209"/>
-      <c r="V6" s="209"/>
-      <c r="W6" s="209"/>
-      <c r="X6" s="209"/>
-      <c r="Y6" s="209"/>
-      <c r="Z6" s="209"/>
-      <c r="AA6" s="209"/>
-      <c r="AB6" s="211"/>
+      <c r="B6" s="157"/>
+      <c r="C6" s="157"/>
+      <c r="D6" s="157"/>
+      <c r="E6" s="157"/>
+      <c r="F6" s="157"/>
+      <c r="G6" s="158"/>
+      <c r="H6" s="157"/>
+      <c r="I6" s="157"/>
+      <c r="J6" s="157"/>
+      <c r="K6" s="157"/>
+      <c r="L6" s="157"/>
+      <c r="M6" s="157"/>
+      <c r="N6" s="157"/>
+      <c r="O6" s="157"/>
+      <c r="P6" s="157"/>
+      <c r="Q6" s="157"/>
+      <c r="R6" s="157"/>
+      <c r="S6" s="157"/>
+      <c r="T6" s="157"/>
+      <c r="U6" s="157"/>
+      <c r="V6" s="157"/>
+      <c r="W6" s="157"/>
+      <c r="X6" s="157"/>
+      <c r="Y6" s="157"/>
+      <c r="Z6" s="157"/>
+      <c r="AA6" s="157"/>
+      <c r="AB6" s="159"/>
     </row>
     <row r="7" spans="1:28" ht="6.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="99"/>
@@ -3243,97 +3243,97 @@
     </row>
     <row r="33" spans="1:28" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="105"/>
-      <c r="B33" s="187" t="s">
+      <c r="B33" s="164" t="s">
         <v>17</v>
       </c>
-      <c r="C33" s="188"/>
-      <c r="D33" s="193" t="s">
+      <c r="C33" s="165"/>
+      <c r="D33" s="170" t="s">
         <v>18</v>
       </c>
-      <c r="E33" s="194"/>
-      <c r="F33" s="194"/>
-      <c r="G33" s="194"/>
-      <c r="H33" s="194"/>
-      <c r="I33" s="194"/>
-      <c r="J33" s="194"/>
-      <c r="K33" s="195"/>
-      <c r="L33" s="193" t="s">
+      <c r="E33" s="171"/>
+      <c r="F33" s="171"/>
+      <c r="G33" s="171"/>
+      <c r="H33" s="171"/>
+      <c r="I33" s="171"/>
+      <c r="J33" s="171"/>
+      <c r="K33" s="172"/>
+      <c r="L33" s="170" t="s">
         <v>19</v>
       </c>
-      <c r="M33" s="194"/>
-      <c r="N33" s="195"/>
-      <c r="O33" s="202" t="s">
+      <c r="M33" s="171"/>
+      <c r="N33" s="172"/>
+      <c r="O33" s="160" t="s">
         <v>20</v>
       </c>
-      <c r="P33" s="203"/>
-      <c r="Q33" s="203"/>
-      <c r="R33" s="203"/>
-      <c r="S33" s="203"/>
-      <c r="T33" s="203"/>
-      <c r="U33" s="203"/>
-      <c r="V33" s="204"/>
-      <c r="W33" s="205" t="s">
+      <c r="P33" s="161"/>
+      <c r="Q33" s="161"/>
+      <c r="R33" s="161"/>
+      <c r="S33" s="161"/>
+      <c r="T33" s="161"/>
+      <c r="U33" s="161"/>
+      <c r="V33" s="162"/>
+      <c r="W33" s="163" t="s">
         <v>21</v>
       </c>
-      <c r="X33" s="205"/>
-      <c r="Y33" s="205"/>
-      <c r="Z33" s="205"/>
+      <c r="X33" s="163"/>
+      <c r="Y33" s="163"/>
+      <c r="Z33" s="163"/>
       <c r="AA33" s="106"/>
       <c r="AB33" s="96"/>
     </row>
     <row r="34" spans="1:28" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="105"/>
-      <c r="B34" s="189"/>
-      <c r="C34" s="190"/>
-      <c r="D34" s="196"/>
-      <c r="E34" s="197"/>
-      <c r="F34" s="197"/>
-      <c r="G34" s="197"/>
-      <c r="H34" s="197"/>
-      <c r="I34" s="197"/>
-      <c r="J34" s="197"/>
-      <c r="K34" s="198"/>
-      <c r="L34" s="196"/>
-      <c r="M34" s="197"/>
-      <c r="N34" s="198"/>
-      <c r="O34" s="202" t="s">
+      <c r="B34" s="166"/>
+      <c r="C34" s="167"/>
+      <c r="D34" s="173"/>
+      <c r="E34" s="174"/>
+      <c r="F34" s="174"/>
+      <c r="G34" s="174"/>
+      <c r="H34" s="174"/>
+      <c r="I34" s="174"/>
+      <c r="J34" s="174"/>
+      <c r="K34" s="175"/>
+      <c r="L34" s="173"/>
+      <c r="M34" s="174"/>
+      <c r="N34" s="175"/>
+      <c r="O34" s="160" t="s">
         <v>22</v>
       </c>
-      <c r="P34" s="204"/>
-      <c r="Q34" s="202" t="s">
+      <c r="P34" s="162"/>
+      <c r="Q34" s="160" t="s">
         <v>23</v>
       </c>
-      <c r="R34" s="204"/>
-      <c r="S34" s="202" t="s">
+      <c r="R34" s="162"/>
+      <c r="S34" s="160" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="204"/>
-      <c r="U34" s="202" t="s">
+      <c r="T34" s="162"/>
+      <c r="U34" s="160" t="s">
         <v>25</v>
       </c>
-      <c r="V34" s="204"/>
-      <c r="W34" s="205"/>
-      <c r="X34" s="205"/>
-      <c r="Y34" s="205"/>
-      <c r="Z34" s="205"/>
+      <c r="V34" s="162"/>
+      <c r="W34" s="163"/>
+      <c r="X34" s="163"/>
+      <c r="Y34" s="163"/>
+      <c r="Z34" s="163"/>
       <c r="AA34" s="106"/>
       <c r="AB34" s="96"/>
     </row>
     <row r="35" spans="1:28" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="105"/>
-      <c r="B35" s="191"/>
-      <c r="C35" s="192"/>
-      <c r="D35" s="199"/>
-      <c r="E35" s="200"/>
-      <c r="F35" s="200"/>
-      <c r="G35" s="200"/>
-      <c r="H35" s="200"/>
-      <c r="I35" s="200"/>
-      <c r="J35" s="200"/>
-      <c r="K35" s="201"/>
-      <c r="L35" s="199"/>
-      <c r="M35" s="200"/>
-      <c r="N35" s="201"/>
+      <c r="B35" s="168"/>
+      <c r="C35" s="169"/>
+      <c r="D35" s="176"/>
+      <c r="E35" s="177"/>
+      <c r="F35" s="177"/>
+      <c r="G35" s="177"/>
+      <c r="H35" s="177"/>
+      <c r="I35" s="177"/>
+      <c r="J35" s="177"/>
+      <c r="K35" s="178"/>
+      <c r="L35" s="176"/>
+      <c r="M35" s="177"/>
+      <c r="N35" s="178"/>
       <c r="O35" s="137" t="s">
         <v>26</v>
       </c>
@@ -3358,34 +3358,34 @@
       <c r="V35" s="139" t="s">
         <v>27</v>
       </c>
-      <c r="W35" s="205"/>
-      <c r="X35" s="205"/>
-      <c r="Y35" s="205"/>
-      <c r="Z35" s="205"/>
+      <c r="W35" s="163"/>
+      <c r="X35" s="163"/>
+      <c r="Y35" s="163"/>
+      <c r="Z35" s="163"/>
       <c r="AA35" s="106"/>
       <c r="AB35" s="96"/>
     </row>
     <row r="36" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="105"/>
-      <c r="B36" s="182" t="s">
+      <c r="B36" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" s="141"/>
+      <c r="D36" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C36" s="183"/>
-      <c r="D36" s="184" t="s">
+      <c r="E36" s="143"/>
+      <c r="F36" s="143"/>
+      <c r="G36" s="143"/>
+      <c r="H36" s="143"/>
+      <c r="I36" s="143"/>
+      <c r="J36" s="143"/>
+      <c r="K36" s="144"/>
+      <c r="L36" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E36" s="185"/>
-      <c r="F36" s="185"/>
-      <c r="G36" s="185"/>
-      <c r="H36" s="185"/>
-      <c r="I36" s="185"/>
-      <c r="J36" s="185"/>
-      <c r="K36" s="186"/>
-      <c r="L36" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M36" s="185"/>
-      <c r="N36" s="186"/>
+      <c r="M36" s="143"/>
+      <c r="N36" s="144"/>
       <c r="O36" s="136">
         <v>1</v>
       </c>
@@ -3410,36 +3410,36 @@
       <c r="V36" s="136">
         <v>8</v>
       </c>
-      <c r="W36" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X36" s="180"/>
-      <c r="Y36" s="180"/>
-      <c r="Z36" s="181"/>
+      <c r="W36" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X36" s="146"/>
+      <c r="Y36" s="146"/>
+      <c r="Z36" s="147"/>
       <c r="AA36" s="88"/>
       <c r="AB36" s="96"/>
     </row>
     <row r="37" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="105"/>
-      <c r="B37" s="182" t="s">
+      <c r="B37" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" s="141"/>
+      <c r="D37" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C37" s="183"/>
-      <c r="D37" s="184" t="s">
+      <c r="E37" s="143"/>
+      <c r="F37" s="143"/>
+      <c r="G37" s="143"/>
+      <c r="H37" s="143"/>
+      <c r="I37" s="143"/>
+      <c r="J37" s="143"/>
+      <c r="K37" s="144"/>
+      <c r="L37" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E37" s="185"/>
-      <c r="F37" s="185"/>
-      <c r="G37" s="185"/>
-      <c r="H37" s="185"/>
-      <c r="I37" s="185"/>
-      <c r="J37" s="185"/>
-      <c r="K37" s="186"/>
-      <c r="L37" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M37" s="185"/>
-      <c r="N37" s="186"/>
+      <c r="M37" s="143"/>
+      <c r="N37" s="144"/>
       <c r="O37" s="136">
         <v>1</v>
       </c>
@@ -3464,36 +3464,36 @@
       <c r="V37" s="136">
         <v>8</v>
       </c>
-      <c r="W37" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X37" s="180"/>
-      <c r="Y37" s="180"/>
-      <c r="Z37" s="181"/>
+      <c r="W37" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X37" s="146"/>
+      <c r="Y37" s="146"/>
+      <c r="Z37" s="147"/>
       <c r="AA37" s="88"/>
       <c r="AB37" s="96"/>
     </row>
     <row r="38" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="105"/>
-      <c r="B38" s="182" t="s">
+      <c r="B38" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" s="141"/>
+      <c r="D38" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C38" s="183"/>
-      <c r="D38" s="184" t="s">
+      <c r="E38" s="143"/>
+      <c r="F38" s="143"/>
+      <c r="G38" s="143"/>
+      <c r="H38" s="143"/>
+      <c r="I38" s="143"/>
+      <c r="J38" s="143"/>
+      <c r="K38" s="144"/>
+      <c r="L38" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E38" s="185"/>
-      <c r="F38" s="185"/>
-      <c r="G38" s="185"/>
-      <c r="H38" s="185"/>
-      <c r="I38" s="185"/>
-      <c r="J38" s="185"/>
-      <c r="K38" s="186"/>
-      <c r="L38" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M38" s="185"/>
-      <c r="N38" s="186"/>
+      <c r="M38" s="143"/>
+      <c r="N38" s="144"/>
       <c r="O38" s="136">
         <v>1</v>
       </c>
@@ -3518,35 +3518,35 @@
       <c r="V38" s="136">
         <v>8</v>
       </c>
-      <c r="W38" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X38" s="180"/>
-      <c r="Y38" s="180"/>
-      <c r="Z38" s="181"/>
+      <c r="W38" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X38" s="146"/>
+      <c r="Y38" s="146"/>
+      <c r="Z38" s="147"/>
       <c r="AA38" s="88"/>
       <c r="AB38" s="96"/>
     </row>
     <row r="39" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="182" t="s">
+      <c r="B39" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39" s="141"/>
+      <c r="D39" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="183"/>
-      <c r="D39" s="184" t="s">
+      <c r="E39" s="143"/>
+      <c r="F39" s="143"/>
+      <c r="G39" s="143"/>
+      <c r="H39" s="143"/>
+      <c r="I39" s="143"/>
+      <c r="J39" s="143"/>
+      <c r="K39" s="144"/>
+      <c r="L39" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E39" s="185"/>
-      <c r="F39" s="185"/>
-      <c r="G39" s="185"/>
-      <c r="H39" s="185"/>
-      <c r="I39" s="185"/>
-      <c r="J39" s="185"/>
-      <c r="K39" s="186"/>
-      <c r="L39" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M39" s="185"/>
-      <c r="N39" s="186"/>
+      <c r="M39" s="143"/>
+      <c r="N39" s="144"/>
       <c r="O39" s="136">
         <v>1</v>
       </c>
@@ -3571,33 +3571,33 @@
       <c r="V39" s="136">
         <v>8</v>
       </c>
-      <c r="W39" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X39" s="180"/>
-      <c r="Y39" s="180"/>
-      <c r="Z39" s="181"/>
+      <c r="W39" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X39" s="146"/>
+      <c r="Y39" s="146"/>
+      <c r="Z39" s="147"/>
     </row>
     <row r="40" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="182" t="s">
+      <c r="B40" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" s="141"/>
+      <c r="D40" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C40" s="183"/>
-      <c r="D40" s="184" t="s">
+      <c r="E40" s="143"/>
+      <c r="F40" s="143"/>
+      <c r="G40" s="143"/>
+      <c r="H40" s="143"/>
+      <c r="I40" s="143"/>
+      <c r="J40" s="143"/>
+      <c r="K40" s="144"/>
+      <c r="L40" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E40" s="185"/>
-      <c r="F40" s="185"/>
-      <c r="G40" s="185"/>
-      <c r="H40" s="185"/>
-      <c r="I40" s="185"/>
-      <c r="J40" s="185"/>
-      <c r="K40" s="186"/>
-      <c r="L40" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M40" s="185"/>
-      <c r="N40" s="186"/>
+      <c r="M40" s="143"/>
+      <c r="N40" s="144"/>
       <c r="O40" s="136">
         <v>1</v>
       </c>
@@ -3622,33 +3622,33 @@
       <c r="V40" s="136">
         <v>8</v>
       </c>
-      <c r="W40" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X40" s="180"/>
-      <c r="Y40" s="180"/>
-      <c r="Z40" s="181"/>
+      <c r="W40" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X40" s="146"/>
+      <c r="Y40" s="146"/>
+      <c r="Z40" s="147"/>
     </row>
     <row r="41" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="182" t="s">
+      <c r="B41" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41" s="141"/>
+      <c r="D41" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C41" s="183"/>
-      <c r="D41" s="184" t="s">
+      <c r="E41" s="143"/>
+      <c r="F41" s="143"/>
+      <c r="G41" s="143"/>
+      <c r="H41" s="143"/>
+      <c r="I41" s="143"/>
+      <c r="J41" s="143"/>
+      <c r="K41" s="144"/>
+      <c r="L41" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E41" s="185"/>
-      <c r="F41" s="185"/>
-      <c r="G41" s="185"/>
-      <c r="H41" s="185"/>
-      <c r="I41" s="185"/>
-      <c r="J41" s="185"/>
-      <c r="K41" s="186"/>
-      <c r="L41" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M41" s="185"/>
-      <c r="N41" s="186"/>
+      <c r="M41" s="143"/>
+      <c r="N41" s="144"/>
       <c r="O41" s="136">
         <v>1</v>
       </c>
@@ -3673,33 +3673,33 @@
       <c r="V41" s="136">
         <v>8</v>
       </c>
-      <c r="W41" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X41" s="180"/>
-      <c r="Y41" s="180"/>
-      <c r="Z41" s="181"/>
+      <c r="W41" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X41" s="146"/>
+      <c r="Y41" s="146"/>
+      <c r="Z41" s="147"/>
     </row>
     <row r="42" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="182" t="s">
+      <c r="B42" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C42" s="141"/>
+      <c r="D42" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C42" s="183"/>
-      <c r="D42" s="184" t="s">
+      <c r="E42" s="143"/>
+      <c r="F42" s="143"/>
+      <c r="G42" s="143"/>
+      <c r="H42" s="143"/>
+      <c r="I42" s="143"/>
+      <c r="J42" s="143"/>
+      <c r="K42" s="144"/>
+      <c r="L42" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E42" s="185"/>
-      <c r="F42" s="185"/>
-      <c r="G42" s="185"/>
-      <c r="H42" s="185"/>
-      <c r="I42" s="185"/>
-      <c r="J42" s="185"/>
-      <c r="K42" s="186"/>
-      <c r="L42" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M42" s="185"/>
-      <c r="N42" s="186"/>
+      <c r="M42" s="143"/>
+      <c r="N42" s="144"/>
       <c r="O42" s="136">
         <v>1</v>
       </c>
@@ -3724,33 +3724,33 @@
       <c r="V42" s="136">
         <v>8</v>
       </c>
-      <c r="W42" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X42" s="180"/>
-      <c r="Y42" s="180"/>
-      <c r="Z42" s="181"/>
+      <c r="W42" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X42" s="146"/>
+      <c r="Y42" s="146"/>
+      <c r="Z42" s="147"/>
     </row>
     <row r="43" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="182" t="s">
+      <c r="B43" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C43" s="141"/>
+      <c r="D43" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C43" s="183"/>
-      <c r="D43" s="184" t="s">
+      <c r="E43" s="143"/>
+      <c r="F43" s="143"/>
+      <c r="G43" s="143"/>
+      <c r="H43" s="143"/>
+      <c r="I43" s="143"/>
+      <c r="J43" s="143"/>
+      <c r="K43" s="144"/>
+      <c r="L43" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E43" s="185"/>
-      <c r="F43" s="185"/>
-      <c r="G43" s="185"/>
-      <c r="H43" s="185"/>
-      <c r="I43" s="185"/>
-      <c r="J43" s="185"/>
-      <c r="K43" s="186"/>
-      <c r="L43" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M43" s="185"/>
-      <c r="N43" s="186"/>
+      <c r="M43" s="143"/>
+      <c r="N43" s="144"/>
       <c r="O43" s="136">
         <v>1</v>
       </c>
@@ -3775,33 +3775,33 @@
       <c r="V43" s="136">
         <v>8</v>
       </c>
-      <c r="W43" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X43" s="180"/>
-      <c r="Y43" s="180"/>
-      <c r="Z43" s="181"/>
+      <c r="W43" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X43" s="146"/>
+      <c r="Y43" s="146"/>
+      <c r="Z43" s="147"/>
     </row>
     <row r="44" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="182" t="s">
+      <c r="B44" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="141"/>
+      <c r="D44" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C44" s="183"/>
-      <c r="D44" s="184" t="s">
+      <c r="E44" s="143"/>
+      <c r="F44" s="143"/>
+      <c r="G44" s="143"/>
+      <c r="H44" s="143"/>
+      <c r="I44" s="143"/>
+      <c r="J44" s="143"/>
+      <c r="K44" s="144"/>
+      <c r="L44" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E44" s="185"/>
-      <c r="F44" s="185"/>
-      <c r="G44" s="185"/>
-      <c r="H44" s="185"/>
-      <c r="I44" s="185"/>
-      <c r="J44" s="185"/>
-      <c r="K44" s="186"/>
-      <c r="L44" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M44" s="185"/>
-      <c r="N44" s="186"/>
+      <c r="M44" s="143"/>
+      <c r="N44" s="144"/>
       <c r="O44" s="136">
         <v>1</v>
       </c>
@@ -3826,33 +3826,33 @@
       <c r="V44" s="136">
         <v>8</v>
       </c>
-      <c r="W44" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X44" s="180"/>
-      <c r="Y44" s="180"/>
-      <c r="Z44" s="181"/>
+      <c r="W44" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X44" s="146"/>
+      <c r="Y44" s="146"/>
+      <c r="Z44" s="147"/>
     </row>
     <row r="45" spans="1:28" s="120" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="182" t="s">
+      <c r="B45" s="140" t="s">
+        <v>91</v>
+      </c>
+      <c r="C45" s="141"/>
+      <c r="D45" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="C45" s="183"/>
-      <c r="D45" s="184" t="s">
+      <c r="E45" s="143"/>
+      <c r="F45" s="143"/>
+      <c r="G45" s="143"/>
+      <c r="H45" s="143"/>
+      <c r="I45" s="143"/>
+      <c r="J45" s="143"/>
+      <c r="K45" s="144"/>
+      <c r="L45" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="E45" s="185"/>
-      <c r="F45" s="185"/>
-      <c r="G45" s="185"/>
-      <c r="H45" s="185"/>
-      <c r="I45" s="185"/>
-      <c r="J45" s="185"/>
-      <c r="K45" s="186"/>
-      <c r="L45" s="184" t="s">
-        <v>94</v>
-      </c>
-      <c r="M45" s="185"/>
-      <c r="N45" s="186"/>
+      <c r="M45" s="143"/>
+      <c r="N45" s="144"/>
       <c r="O45" s="136">
         <v>1</v>
       </c>
@@ -3877,12 +3877,12 @@
       <c r="V45" s="136">
         <v>8</v>
       </c>
-      <c r="W45" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="X45" s="180"/>
-      <c r="Y45" s="180"/>
-      <c r="Z45" s="181"/>
+      <c r="W45" s="145" t="s">
+        <v>94</v>
+      </c>
+      <c r="X45" s="146"/>
+      <c r="Y45" s="146"/>
+      <c r="Z45" s="147"/>
     </row>
     <row r="46" spans="1:28" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="105"/>
@@ -4073,34 +4073,34 @@
       <c r="AB51" s="125"/>
     </row>
     <row r="52" spans="1:32" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="153"/>
-      <c r="B52" s="154"/>
-      <c r="C52" s="154"/>
-      <c r="D52" s="154"/>
-      <c r="E52" s="154"/>
-      <c r="F52" s="154"/>
-      <c r="G52" s="154"/>
-      <c r="H52" s="154"/>
-      <c r="I52" s="154"/>
-      <c r="J52" s="154"/>
-      <c r="K52" s="154"/>
-      <c r="L52" s="154"/>
-      <c r="M52" s="154"/>
-      <c r="N52" s="154"/>
-      <c r="O52" s="154"/>
-      <c r="P52" s="154"/>
-      <c r="Q52" s="154"/>
+      <c r="A52" s="150"/>
+      <c r="B52" s="151"/>
+      <c r="C52" s="151"/>
+      <c r="D52" s="151"/>
+      <c r="E52" s="151"/>
+      <c r="F52" s="151"/>
+      <c r="G52" s="151"/>
+      <c r="H52" s="151"/>
+      <c r="I52" s="151"/>
+      <c r="J52" s="151"/>
+      <c r="K52" s="151"/>
+      <c r="L52" s="151"/>
+      <c r="M52" s="151"/>
+      <c r="N52" s="151"/>
+      <c r="O52" s="151"/>
+      <c r="P52" s="151"/>
+      <c r="Q52" s="151"/>
       <c r="R52" s="88"/>
       <c r="S52" s="88"/>
       <c r="T52" s="88"/>
-      <c r="U52" s="154"/>
-      <c r="V52" s="154"/>
-      <c r="W52" s="154"/>
+      <c r="U52" s="151"/>
+      <c r="V52" s="151"/>
+      <c r="W52" s="151"/>
       <c r="X52" s="88"/>
-      <c r="Y52" s="154"/>
-      <c r="Z52" s="154"/>
-      <c r="AA52" s="154"/>
-      <c r="AB52" s="155"/>
+      <c r="Y52" s="151"/>
+      <c r="Z52" s="151"/>
+      <c r="AA52" s="151"/>
+      <c r="AB52" s="179"/>
     </row>
     <row r="53" spans="1:32" s="120" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="105"/>
@@ -4147,162 +4147,162 @@
       <c r="AB54" s="96"/>
     </row>
     <row r="55" spans="1:32" s="119" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="149" t="s">
+      <c r="A55" s="180" t="s">
         <v>31</v>
       </c>
-      <c r="B55" s="149"/>
-      <c r="C55" s="149"/>
-      <c r="D55" s="175" t="s">
-        <v>96</v>
-      </c>
-      <c r="E55" s="176"/>
-      <c r="F55" s="176"/>
-      <c r="G55" s="177"/>
-      <c r="H55" s="178" t="s">
+      <c r="B55" s="180"/>
+      <c r="C55" s="180"/>
+      <c r="D55" s="181" t="s">
+        <v>95</v>
+      </c>
+      <c r="E55" s="182"/>
+      <c r="F55" s="182"/>
+      <c r="G55" s="183"/>
+      <c r="H55" s="184" t="s">
         <v>32</v>
       </c>
-      <c r="I55" s="178"/>
-      <c r="J55" s="178"/>
-      <c r="K55" s="175" t="s">
+      <c r="I55" s="184"/>
+      <c r="J55" s="184"/>
+      <c r="K55" s="181" t="s">
         <v>33</v>
       </c>
-      <c r="L55" s="176"/>
-      <c r="M55" s="177"/>
-      <c r="N55" s="178" t="s">
+      <c r="L55" s="182"/>
+      <c r="M55" s="183"/>
+      <c r="N55" s="184" t="s">
         <v>34</v>
       </c>
-      <c r="O55" s="178"/>
-      <c r="P55" s="178"/>
-      <c r="Q55" s="178" t="s">
+      <c r="O55" s="184"/>
+      <c r="P55" s="184"/>
+      <c r="Q55" s="184" t="s">
         <v>35</v>
       </c>
-      <c r="R55" s="178"/>
-      <c r="S55" s="178"/>
-      <c r="T55" s="175" t="s">
+      <c r="R55" s="184"/>
+      <c r="S55" s="184"/>
+      <c r="T55" s="181" t="s">
         <v>36</v>
       </c>
-      <c r="U55" s="176"/>
-      <c r="V55" s="177"/>
-      <c r="W55" s="175" t="s">
+      <c r="U55" s="182"/>
+      <c r="V55" s="183"/>
+      <c r="W55" s="181" t="s">
         <v>37</v>
       </c>
-      <c r="X55" s="176"/>
-      <c r="Y55" s="177"/>
-      <c r="Z55" s="175" t="s">
+      <c r="X55" s="182"/>
+      <c r="Y55" s="183"/>
+      <c r="Z55" s="181" t="s">
         <v>38</v>
       </c>
-      <c r="AA55" s="176"/>
-      <c r="AB55" s="177"/>
+      <c r="AA55" s="182"/>
+      <c r="AB55" s="183"/>
       <c r="AC55" s="87"/>
       <c r="AF55" s="128"/>
     </row>
     <row r="56" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="166"/>
-      <c r="B56" s="167"/>
-      <c r="C56" s="168"/>
-      <c r="D56" s="140" t="s">
+      <c r="A56" s="185"/>
+      <c r="B56" s="186"/>
+      <c r="C56" s="187"/>
+      <c r="D56" s="194" t="s">
+        <v>97</v>
+      </c>
+      <c r="E56" s="195"/>
+      <c r="F56" s="195"/>
+      <c r="G56" s="196"/>
+      <c r="H56" s="194" t="s">
+        <v>96</v>
+      </c>
+      <c r="I56" s="195"/>
+      <c r="J56" s="196"/>
+      <c r="K56" s="148" t="s">
+        <v>39</v>
+      </c>
+      <c r="L56" s="149"/>
+      <c r="M56" s="203"/>
+      <c r="N56" s="148" t="s">
         <v>98</v>
       </c>
-      <c r="E56" s="141"/>
-      <c r="F56" s="141"/>
-      <c r="G56" s="142"/>
-      <c r="H56" s="140" t="s">
-        <v>97</v>
-      </c>
-      <c r="I56" s="141"/>
-      <c r="J56" s="142"/>
-      <c r="K56" s="150" t="s">
-        <v>39</v>
-      </c>
-      <c r="L56" s="151"/>
-      <c r="M56" s="152"/>
-      <c r="N56" s="150" t="s">
+      <c r="O56" s="149"/>
+      <c r="P56" s="203"/>
+      <c r="Q56" s="148" t="s">
         <v>99</v>
       </c>
-      <c r="O56" s="151"/>
-      <c r="P56" s="152"/>
-      <c r="Q56" s="150" t="s">
+      <c r="R56" s="149"/>
+      <c r="S56" s="203"/>
+      <c r="T56" s="148" t="s">
         <v>100</v>
       </c>
-      <c r="R56" s="151"/>
-      <c r="S56" s="152"/>
-      <c r="T56" s="150" t="s">
+      <c r="U56" s="149"/>
+      <c r="V56" s="203"/>
+      <c r="W56" s="194" t="s">
         <v>101</v>
       </c>
-      <c r="U56" s="151"/>
-      <c r="V56" s="152"/>
-      <c r="W56" s="140" t="s">
-        <v>102</v>
-      </c>
-      <c r="X56" s="141"/>
-      <c r="Y56" s="142"/>
-      <c r="Z56" s="150" t="s">
+      <c r="X56" s="195"/>
+      <c r="Y56" s="196"/>
+      <c r="Z56" s="148" t="s">
         <v>40</v>
       </c>
-      <c r="AA56" s="151"/>
-      <c r="AB56" s="152"/>
+      <c r="AA56" s="149"/>
+      <c r="AB56" s="203"/>
       <c r="AF56" s="128"/>
     </row>
     <row r="57" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="169"/>
-      <c r="B57" s="170"/>
-      <c r="C57" s="171"/>
-      <c r="D57" s="143"/>
-      <c r="E57" s="144"/>
-      <c r="F57" s="144"/>
-      <c r="G57" s="145"/>
-      <c r="H57" s="143"/>
-      <c r="I57" s="144"/>
-      <c r="J57" s="145"/>
-      <c r="K57" s="153"/>
-      <c r="L57" s="154"/>
-      <c r="M57" s="155"/>
-      <c r="N57" s="153"/>
-      <c r="O57" s="154"/>
-      <c r="P57" s="155"/>
-      <c r="Q57" s="153"/>
-      <c r="R57" s="154"/>
-      <c r="S57" s="155"/>
-      <c r="T57" s="153"/>
-      <c r="U57" s="154"/>
-      <c r="V57" s="155"/>
-      <c r="W57" s="143"/>
-      <c r="X57" s="144"/>
-      <c r="Y57" s="145"/>
-      <c r="Z57" s="153"/>
-      <c r="AA57" s="154"/>
-      <c r="AB57" s="155"/>
+      <c r="A57" s="188"/>
+      <c r="B57" s="189"/>
+      <c r="C57" s="190"/>
+      <c r="D57" s="197"/>
+      <c r="E57" s="198"/>
+      <c r="F57" s="198"/>
+      <c r="G57" s="199"/>
+      <c r="H57" s="197"/>
+      <c r="I57" s="198"/>
+      <c r="J57" s="199"/>
+      <c r="K57" s="150"/>
+      <c r="L57" s="151"/>
+      <c r="M57" s="179"/>
+      <c r="N57" s="150"/>
+      <c r="O57" s="151"/>
+      <c r="P57" s="179"/>
+      <c r="Q57" s="150"/>
+      <c r="R57" s="151"/>
+      <c r="S57" s="179"/>
+      <c r="T57" s="150"/>
+      <c r="U57" s="151"/>
+      <c r="V57" s="179"/>
+      <c r="W57" s="197"/>
+      <c r="X57" s="198"/>
+      <c r="Y57" s="199"/>
+      <c r="Z57" s="150"/>
+      <c r="AA57" s="151"/>
+      <c r="AB57" s="179"/>
       <c r="AF57" s="128"/>
     </row>
     <row r="58" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="172"/>
-      <c r="B58" s="173"/>
-      <c r="C58" s="174"/>
-      <c r="D58" s="146"/>
-      <c r="E58" s="147"/>
-      <c r="F58" s="147"/>
-      <c r="G58" s="148"/>
-      <c r="H58" s="146"/>
-      <c r="I58" s="147"/>
-      <c r="J58" s="148"/>
-      <c r="K58" s="156"/>
-      <c r="L58" s="157"/>
-      <c r="M58" s="158"/>
-      <c r="N58" s="156"/>
-      <c r="O58" s="157"/>
-      <c r="P58" s="158"/>
-      <c r="Q58" s="156"/>
-      <c r="R58" s="157"/>
-      <c r="S58" s="158"/>
-      <c r="T58" s="156"/>
-      <c r="U58" s="157"/>
-      <c r="V58" s="158"/>
-      <c r="W58" s="146"/>
-      <c r="X58" s="147"/>
-      <c r="Y58" s="148"/>
-      <c r="Z58" s="156"/>
-      <c r="AA58" s="157"/>
-      <c r="AB58" s="158"/>
+      <c r="A58" s="191"/>
+      <c r="B58" s="192"/>
+      <c r="C58" s="193"/>
+      <c r="D58" s="200"/>
+      <c r="E58" s="201"/>
+      <c r="F58" s="201"/>
+      <c r="G58" s="202"/>
+      <c r="H58" s="200"/>
+      <c r="I58" s="201"/>
+      <c r="J58" s="202"/>
+      <c r="K58" s="152"/>
+      <c r="L58" s="153"/>
+      <c r="M58" s="204"/>
+      <c r="N58" s="152"/>
+      <c r="O58" s="153"/>
+      <c r="P58" s="204"/>
+      <c r="Q58" s="152"/>
+      <c r="R58" s="153"/>
+      <c r="S58" s="204"/>
+      <c r="T58" s="152"/>
+      <c r="U58" s="153"/>
+      <c r="V58" s="204"/>
+      <c r="W58" s="200"/>
+      <c r="X58" s="201"/>
+      <c r="Y58" s="202"/>
+      <c r="Z58" s="152"/>
+      <c r="AA58" s="153"/>
+      <c r="AB58" s="204"/>
       <c r="AF58" s="128"/>
     </row>
     <row r="59" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4350,9 +4350,9 @@
       <c r="C60" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="D60" s="165"/>
-      <c r="E60" s="165"/>
-      <c r="F60" s="165"/>
+      <c r="D60" s="205"/>
+      <c r="E60" s="205"/>
+      <c r="F60" s="205"/>
       <c r="G60" s="130"/>
       <c r="H60" s="130"/>
       <c r="I60" s="130"/>
@@ -4393,203 +4393,203 @@
       <c r="AF61" s="128"/>
     </row>
     <row r="62" spans="1:32" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="159" t="s">
+      <c r="A62" s="206" t="s">
         <v>43</v>
       </c>
-      <c r="B62" s="160"/>
-      <c r="C62" s="160"/>
-      <c r="D62" s="160"/>
-      <c r="E62" s="160"/>
-      <c r="F62" s="160"/>
-      <c r="G62" s="160"/>
-      <c r="H62" s="160"/>
-      <c r="I62" s="160"/>
-      <c r="J62" s="160"/>
-      <c r="K62" s="160"/>
-      <c r="L62" s="160"/>
-      <c r="M62" s="160"/>
-      <c r="N62" s="160"/>
-      <c r="O62" s="160"/>
-      <c r="P62" s="160"/>
-      <c r="Q62" s="160"/>
-      <c r="R62" s="160"/>
-      <c r="S62" s="160"/>
-      <c r="T62" s="160"/>
-      <c r="U62" s="160"/>
-      <c r="V62" s="160"/>
-      <c r="W62" s="160"/>
-      <c r="X62" s="160"/>
-      <c r="Y62" s="160"/>
-      <c r="Z62" s="160"/>
-      <c r="AA62" s="160"/>
-      <c r="AB62" s="161"/>
+      <c r="B62" s="207"/>
+      <c r="C62" s="207"/>
+      <c r="D62" s="207"/>
+      <c r="E62" s="207"/>
+      <c r="F62" s="207"/>
+      <c r="G62" s="207"/>
+      <c r="H62" s="207"/>
+      <c r="I62" s="207"/>
+      <c r="J62" s="207"/>
+      <c r="K62" s="207"/>
+      <c r="L62" s="207"/>
+      <c r="M62" s="207"/>
+      <c r="N62" s="207"/>
+      <c r="O62" s="207"/>
+      <c r="P62" s="207"/>
+      <c r="Q62" s="207"/>
+      <c r="R62" s="207"/>
+      <c r="S62" s="207"/>
+      <c r="T62" s="207"/>
+      <c r="U62" s="207"/>
+      <c r="V62" s="207"/>
+      <c r="W62" s="207"/>
+      <c r="X62" s="207"/>
+      <c r="Y62" s="207"/>
+      <c r="Z62" s="207"/>
+      <c r="AA62" s="207"/>
+      <c r="AB62" s="208"/>
       <c r="AF62" s="128" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="63" spans="1:32" s="119" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="162" t="s">
+      <c r="A63" s="209" t="s">
         <v>45</v>
       </c>
-      <c r="B63" s="163"/>
-      <c r="C63" s="163"/>
-      <c r="D63" s="163"/>
-      <c r="E63" s="164"/>
-      <c r="F63" s="162" t="s">
+      <c r="B63" s="210"/>
+      <c r="C63" s="210"/>
+      <c r="D63" s="210"/>
+      <c r="E63" s="211"/>
+      <c r="F63" s="209" t="s">
         <v>46</v>
       </c>
-      <c r="G63" s="163"/>
-      <c r="H63" s="163"/>
-      <c r="I63" s="163"/>
-      <c r="J63" s="163"/>
-      <c r="K63" s="164"/>
-      <c r="L63" s="162" t="s">
+      <c r="G63" s="210"/>
+      <c r="H63" s="210"/>
+      <c r="I63" s="210"/>
+      <c r="J63" s="210"/>
+      <c r="K63" s="211"/>
+      <c r="L63" s="209" t="s">
         <v>47</v>
       </c>
-      <c r="M63" s="163"/>
-      <c r="N63" s="163"/>
-      <c r="O63" s="163"/>
-      <c r="P63" s="164"/>
-      <c r="Q63" s="150" t="s">
+      <c r="M63" s="210"/>
+      <c r="N63" s="210"/>
+      <c r="O63" s="210"/>
+      <c r="P63" s="211"/>
+      <c r="Q63" s="148" t="s">
         <v>48</v>
       </c>
-      <c r="R63" s="151"/>
-      <c r="S63" s="151"/>
-      <c r="T63" s="151"/>
-      <c r="U63" s="152"/>
-      <c r="V63" s="162" t="s">
+      <c r="R63" s="149"/>
+      <c r="S63" s="149"/>
+      <c r="T63" s="149"/>
+      <c r="U63" s="203"/>
+      <c r="V63" s="209" t="s">
         <v>49</v>
       </c>
-      <c r="W63" s="163"/>
-      <c r="X63" s="163"/>
-      <c r="Y63" s="163"/>
-      <c r="Z63" s="163"/>
-      <c r="AA63" s="163"/>
-      <c r="AB63" s="164"/>
+      <c r="W63" s="210"/>
+      <c r="X63" s="210"/>
+      <c r="Y63" s="210"/>
+      <c r="Z63" s="210"/>
+      <c r="AA63" s="210"/>
+      <c r="AB63" s="211"/>
       <c r="AF63" s="128"/>
     </row>
     <row r="64" spans="1:32" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="140"/>
-      <c r="B64" s="141"/>
-      <c r="C64" s="141"/>
-      <c r="D64" s="141"/>
-      <c r="E64" s="142"/>
-      <c r="F64" s="140"/>
-      <c r="G64" s="141"/>
-      <c r="H64" s="141"/>
-      <c r="I64" s="141"/>
-      <c r="J64" s="141"/>
-      <c r="K64" s="142"/>
-      <c r="L64" s="141"/>
-      <c r="M64" s="141"/>
-      <c r="N64" s="141"/>
-      <c r="O64" s="141"/>
-      <c r="P64" s="142"/>
-      <c r="Q64" s="149"/>
-      <c r="R64" s="149"/>
-      <c r="S64" s="149"/>
-      <c r="T64" s="149"/>
-      <c r="U64" s="149"/>
-      <c r="V64" s="150"/>
-      <c r="W64" s="151"/>
-      <c r="X64" s="151"/>
-      <c r="Y64" s="151"/>
-      <c r="Z64" s="151"/>
-      <c r="AA64" s="151"/>
-      <c r="AB64" s="152"/>
+      <c r="A64" s="194"/>
+      <c r="B64" s="195"/>
+      <c r="C64" s="195"/>
+      <c r="D64" s="195"/>
+      <c r="E64" s="196"/>
+      <c r="F64" s="194"/>
+      <c r="G64" s="195"/>
+      <c r="H64" s="195"/>
+      <c r="I64" s="195"/>
+      <c r="J64" s="195"/>
+      <c r="K64" s="196"/>
+      <c r="L64" s="195"/>
+      <c r="M64" s="195"/>
+      <c r="N64" s="195"/>
+      <c r="O64" s="195"/>
+      <c r="P64" s="196"/>
+      <c r="Q64" s="180"/>
+      <c r="R64" s="180"/>
+      <c r="S64" s="180"/>
+      <c r="T64" s="180"/>
+      <c r="U64" s="180"/>
+      <c r="V64" s="148"/>
+      <c r="W64" s="149"/>
+      <c r="X64" s="149"/>
+      <c r="Y64" s="149"/>
+      <c r="Z64" s="149"/>
+      <c r="AA64" s="149"/>
+      <c r="AB64" s="203"/>
       <c r="AF64" s="128"/>
     </row>
     <row r="65" spans="1:32" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="143"/>
-      <c r="B65" s="144"/>
-      <c r="C65" s="144"/>
-      <c r="D65" s="144"/>
-      <c r="E65" s="145"/>
-      <c r="F65" s="143"/>
-      <c r="G65" s="144"/>
-      <c r="H65" s="144"/>
-      <c r="I65" s="144"/>
-      <c r="J65" s="144"/>
-      <c r="K65" s="145"/>
-      <c r="L65" s="144"/>
-      <c r="M65" s="144"/>
-      <c r="N65" s="144"/>
-      <c r="O65" s="144"/>
-      <c r="P65" s="145"/>
-      <c r="Q65" s="149"/>
-      <c r="R65" s="149"/>
-      <c r="S65" s="149"/>
-      <c r="T65" s="149"/>
-      <c r="U65" s="149"/>
-      <c r="V65" s="153"/>
-      <c r="W65" s="154"/>
-      <c r="X65" s="154"/>
-      <c r="Y65" s="154"/>
-      <c r="Z65" s="154"/>
-      <c r="AA65" s="154"/>
-      <c r="AB65" s="155"/>
+      <c r="A65" s="197"/>
+      <c r="B65" s="198"/>
+      <c r="C65" s="198"/>
+      <c r="D65" s="198"/>
+      <c r="E65" s="199"/>
+      <c r="F65" s="197"/>
+      <c r="G65" s="198"/>
+      <c r="H65" s="198"/>
+      <c r="I65" s="198"/>
+      <c r="J65" s="198"/>
+      <c r="K65" s="199"/>
+      <c r="L65" s="198"/>
+      <c r="M65" s="198"/>
+      <c r="N65" s="198"/>
+      <c r="O65" s="198"/>
+      <c r="P65" s="199"/>
+      <c r="Q65" s="180"/>
+      <c r="R65" s="180"/>
+      <c r="S65" s="180"/>
+      <c r="T65" s="180"/>
+      <c r="U65" s="180"/>
+      <c r="V65" s="150"/>
+      <c r="W65" s="151"/>
+      <c r="X65" s="151"/>
+      <c r="Y65" s="151"/>
+      <c r="Z65" s="151"/>
+      <c r="AA65" s="151"/>
+      <c r="AB65" s="179"/>
       <c r="AF65" s="128"/>
     </row>
     <row r="66" spans="1:32" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="143"/>
-      <c r="B66" s="144"/>
-      <c r="C66" s="144"/>
-      <c r="D66" s="144"/>
-      <c r="E66" s="145"/>
-      <c r="F66" s="143"/>
-      <c r="G66" s="144"/>
-      <c r="H66" s="144"/>
-      <c r="I66" s="144"/>
-      <c r="J66" s="144"/>
-      <c r="K66" s="145"/>
-      <c r="L66" s="144"/>
-      <c r="M66" s="144"/>
-      <c r="N66" s="144"/>
-      <c r="O66" s="144"/>
-      <c r="P66" s="145"/>
-      <c r="Q66" s="149"/>
-      <c r="R66" s="149"/>
-      <c r="S66" s="149"/>
-      <c r="T66" s="149"/>
-      <c r="U66" s="149"/>
-      <c r="V66" s="153"/>
-      <c r="W66" s="154"/>
-      <c r="X66" s="154"/>
-      <c r="Y66" s="154"/>
-      <c r="Z66" s="154"/>
-      <c r="AA66" s="154"/>
-      <c r="AB66" s="155"/>
+      <c r="A66" s="197"/>
+      <c r="B66" s="198"/>
+      <c r="C66" s="198"/>
+      <c r="D66" s="198"/>
+      <c r="E66" s="199"/>
+      <c r="F66" s="197"/>
+      <c r="G66" s="198"/>
+      <c r="H66" s="198"/>
+      <c r="I66" s="198"/>
+      <c r="J66" s="198"/>
+      <c r="K66" s="199"/>
+      <c r="L66" s="198"/>
+      <c r="M66" s="198"/>
+      <c r="N66" s="198"/>
+      <c r="O66" s="198"/>
+      <c r="P66" s="199"/>
+      <c r="Q66" s="180"/>
+      <c r="R66" s="180"/>
+      <c r="S66" s="180"/>
+      <c r="T66" s="180"/>
+      <c r="U66" s="180"/>
+      <c r="V66" s="150"/>
+      <c r="W66" s="151"/>
+      <c r="X66" s="151"/>
+      <c r="Y66" s="151"/>
+      <c r="Z66" s="151"/>
+      <c r="AA66" s="151"/>
+      <c r="AB66" s="179"/>
       <c r="AF66" s="128"/>
     </row>
     <row r="67" spans="1:32" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="146"/>
-      <c r="B67" s="147"/>
-      <c r="C67" s="147"/>
-      <c r="D67" s="147"/>
-      <c r="E67" s="148"/>
-      <c r="F67" s="146"/>
-      <c r="G67" s="147"/>
-      <c r="H67" s="147"/>
-      <c r="I67" s="147"/>
-      <c r="J67" s="147"/>
-      <c r="K67" s="148"/>
-      <c r="L67" s="147"/>
-      <c r="M67" s="147"/>
-      <c r="N67" s="147"/>
-      <c r="O67" s="147"/>
-      <c r="P67" s="148"/>
-      <c r="Q67" s="149"/>
-      <c r="R67" s="149"/>
-      <c r="S67" s="149"/>
-      <c r="T67" s="149"/>
-      <c r="U67" s="149"/>
-      <c r="V67" s="156"/>
-      <c r="W67" s="157"/>
-      <c r="X67" s="157"/>
-      <c r="Y67" s="157"/>
-      <c r="Z67" s="157"/>
-      <c r="AA67" s="157"/>
-      <c r="AB67" s="158"/>
+      <c r="A67" s="200"/>
+      <c r="B67" s="201"/>
+      <c r="C67" s="201"/>
+      <c r="D67" s="201"/>
+      <c r="E67" s="202"/>
+      <c r="F67" s="200"/>
+      <c r="G67" s="201"/>
+      <c r="H67" s="201"/>
+      <c r="I67" s="201"/>
+      <c r="J67" s="201"/>
+      <c r="K67" s="202"/>
+      <c r="L67" s="201"/>
+      <c r="M67" s="201"/>
+      <c r="N67" s="201"/>
+      <c r="O67" s="201"/>
+      <c r="P67" s="202"/>
+      <c r="Q67" s="180"/>
+      <c r="R67" s="180"/>
+      <c r="S67" s="180"/>
+      <c r="T67" s="180"/>
+      <c r="U67" s="180"/>
+      <c r="V67" s="152"/>
+      <c r="W67" s="153"/>
+      <c r="X67" s="153"/>
+      <c r="Y67" s="153"/>
+      <c r="Z67" s="153"/>
+      <c r="AA67" s="153"/>
+      <c r="AB67" s="204"/>
       <c r="AF67" s="128"/>
     </row>
     <row r="68" spans="1:32" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4630,64 +4630,27 @@
     </row>
   </sheetData>
   <mergeCells count="95">
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="D45:K45"/>
-    <mergeCell ref="L45:N45"/>
-    <mergeCell ref="W45:Z45"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="D43:K43"/>
-    <mergeCell ref="L43:N43"/>
-    <mergeCell ref="W43:Z43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="D44:K44"/>
-    <mergeCell ref="L44:N44"/>
-    <mergeCell ref="W44:Z44"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="D41:K41"/>
-    <mergeCell ref="L41:N41"/>
-    <mergeCell ref="W41:Z41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="D42:K42"/>
-    <mergeCell ref="L42:N42"/>
-    <mergeCell ref="W42:Z42"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D39:K39"/>
-    <mergeCell ref="L39:N39"/>
-    <mergeCell ref="W39:Z39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D40:K40"/>
-    <mergeCell ref="L40:N40"/>
-    <mergeCell ref="W40:Z40"/>
-    <mergeCell ref="A2:C5"/>
-    <mergeCell ref="L2:Q3"/>
-    <mergeCell ref="F4:W4"/>
-    <mergeCell ref="D5:AB5"/>
-    <mergeCell ref="A6:AB6"/>
-    <mergeCell ref="O33:V33"/>
-    <mergeCell ref="W33:Z35"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:R34"/>
-    <mergeCell ref="S34:T34"/>
-    <mergeCell ref="U34:V34"/>
-    <mergeCell ref="B33:C35"/>
-    <mergeCell ref="D33:K35"/>
-    <mergeCell ref="L33:N35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="D36:K36"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="D37:K37"/>
-    <mergeCell ref="L37:N37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:K38"/>
-    <mergeCell ref="L38:N38"/>
-    <mergeCell ref="M52:O52"/>
-    <mergeCell ref="P52:Q52"/>
-    <mergeCell ref="U52:W52"/>
-    <mergeCell ref="Y52:Z52"/>
-    <mergeCell ref="W36:Z36"/>
-    <mergeCell ref="W37:Z37"/>
-    <mergeCell ref="W38:Z38"/>
+    <mergeCell ref="A64:E67"/>
+    <mergeCell ref="F64:K67"/>
+    <mergeCell ref="L64:P67"/>
+    <mergeCell ref="Q64:U67"/>
+    <mergeCell ref="V64:AB67"/>
+    <mergeCell ref="A62:AB62"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="F63:K63"/>
+    <mergeCell ref="L63:P63"/>
+    <mergeCell ref="Q63:U63"/>
+    <mergeCell ref="V63:AB63"/>
+    <mergeCell ref="Q56:S58"/>
+    <mergeCell ref="T56:V58"/>
+    <mergeCell ref="W56:Y58"/>
+    <mergeCell ref="Z56:AB58"/>
+    <mergeCell ref="D60:F60"/>
+    <mergeCell ref="A56:C58"/>
+    <mergeCell ref="D56:G58"/>
+    <mergeCell ref="H56:J58"/>
+    <mergeCell ref="K56:M58"/>
+    <mergeCell ref="N56:P58"/>
     <mergeCell ref="AA52:AB52"/>
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="D55:G55"/>
@@ -4704,27 +4667,64 @@
     <mergeCell ref="G52:H52"/>
     <mergeCell ref="I52:J52"/>
     <mergeCell ref="K52:L52"/>
-    <mergeCell ref="A56:C58"/>
-    <mergeCell ref="D56:G58"/>
-    <mergeCell ref="H56:J58"/>
-    <mergeCell ref="K56:M58"/>
-    <mergeCell ref="N56:P58"/>
-    <mergeCell ref="Q56:S58"/>
-    <mergeCell ref="T56:V58"/>
-    <mergeCell ref="W56:Y58"/>
-    <mergeCell ref="Z56:AB58"/>
-    <mergeCell ref="D60:F60"/>
-    <mergeCell ref="A62:AB62"/>
-    <mergeCell ref="A63:E63"/>
-    <mergeCell ref="F63:K63"/>
-    <mergeCell ref="L63:P63"/>
-    <mergeCell ref="Q63:U63"/>
-    <mergeCell ref="V63:AB63"/>
-    <mergeCell ref="A64:E67"/>
-    <mergeCell ref="F64:K67"/>
-    <mergeCell ref="L64:P67"/>
-    <mergeCell ref="Q64:U67"/>
-    <mergeCell ref="V64:AB67"/>
+    <mergeCell ref="M52:O52"/>
+    <mergeCell ref="P52:Q52"/>
+    <mergeCell ref="U52:W52"/>
+    <mergeCell ref="Y52:Z52"/>
+    <mergeCell ref="W36:Z36"/>
+    <mergeCell ref="W37:Z37"/>
+    <mergeCell ref="W38:Z38"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D37:K37"/>
+    <mergeCell ref="L37:N37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D38:K38"/>
+    <mergeCell ref="L38:N38"/>
+    <mergeCell ref="B33:C35"/>
+    <mergeCell ref="D33:K35"/>
+    <mergeCell ref="L33:N35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="D36:K36"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="O33:V33"/>
+    <mergeCell ref="W33:Z35"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="U34:V34"/>
+    <mergeCell ref="A2:C5"/>
+    <mergeCell ref="L2:Q3"/>
+    <mergeCell ref="F4:W4"/>
+    <mergeCell ref="D5:AB5"/>
+    <mergeCell ref="A6:AB6"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D39:K39"/>
+    <mergeCell ref="L39:N39"/>
+    <mergeCell ref="W39:Z39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="D40:K40"/>
+    <mergeCell ref="L40:N40"/>
+    <mergeCell ref="W40:Z40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D41:K41"/>
+    <mergeCell ref="L41:N41"/>
+    <mergeCell ref="W41:Z41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D42:K42"/>
+    <mergeCell ref="L42:N42"/>
+    <mergeCell ref="W42:Z42"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="D45:K45"/>
+    <mergeCell ref="L45:N45"/>
+    <mergeCell ref="W45:Z45"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="D43:K43"/>
+    <mergeCell ref="L43:N43"/>
+    <mergeCell ref="W43:Z43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="D44:K44"/>
+    <mergeCell ref="L44:N44"/>
+    <mergeCell ref="W44:Z44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="24" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -4755,32 +4755,32 @@
       </c>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
-      <c r="L1" s="267"/>
-      <c r="M1" s="267"/>
-      <c r="N1" s="267"/>
-      <c r="O1" s="267"/>
-      <c r="P1" s="267"/>
-      <c r="Q1" s="267"/>
-      <c r="R1" s="267"/>
+      <c r="L1" s="212"/>
+      <c r="M1" s="212"/>
+      <c r="N1" s="212"/>
+      <c r="O1" s="212"/>
+      <c r="P1" s="212"/>
+      <c r="Q1" s="212"/>
+      <c r="R1" s="212"/>
     </row>
     <row r="2" spans="1:21" s="4" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="213" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="269"/>
-      <c r="C2" s="269"/>
-      <c r="D2" s="269"/>
-      <c r="E2" s="269"/>
-      <c r="F2" s="269"/>
-      <c r="G2" s="269"/>
-      <c r="H2" s="269"/>
-      <c r="I2" s="269"/>
-      <c r="J2" s="269"/>
-      <c r="K2" s="269"/>
-      <c r="L2" s="269"/>
-      <c r="M2" s="269"/>
-      <c r="N2" s="269"/>
-      <c r="O2" s="269"/>
+      <c r="B2" s="214"/>
+      <c r="C2" s="214"/>
+      <c r="D2" s="214"/>
+      <c r="E2" s="214"/>
+      <c r="F2" s="214"/>
+      <c r="G2" s="214"/>
+      <c r="H2" s="214"/>
+      <c r="I2" s="214"/>
+      <c r="J2" s="214"/>
+      <c r="K2" s="214"/>
+      <c r="L2" s="214"/>
+      <c r="M2" s="214"/>
+      <c r="N2" s="214"/>
+      <c r="O2" s="214"/>
       <c r="P2" s="5" t="s">
         <v>52</v>
       </c>
@@ -4788,7 +4788,7 @@
       <c r="R2" s="7"/>
     </row>
     <row r="3" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="271" t="s">
+      <c r="A3" s="216" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="9" t="s">
@@ -4800,10 +4800,10 @@
       <c r="F3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="270"/>
-      <c r="H3" s="270"/>
-      <c r="I3" s="270"/>
-      <c r="J3" s="270"/>
+      <c r="G3" s="215"/>
+      <c r="H3" s="215"/>
+      <c r="I3" s="215"/>
+      <c r="J3" s="215"/>
       <c r="K3" s="13"/>
       <c r="R3" s="14"/>
       <c r="S3" s="15"/>
@@ -4811,7 +4811,7 @@
       <c r="U3" s="15"/>
     </row>
     <row r="4" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="272"/>
+      <c r="A4" s="217"/>
       <c r="B4" s="16" t="s">
         <v>55</v>
       </c>
@@ -4821,10 +4821,10 @@
       <c r="F4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="270"/>
-      <c r="H4" s="270"/>
-      <c r="I4" s="270"/>
-      <c r="J4" s="270"/>
+      <c r="G4" s="215"/>
+      <c r="H4" s="215"/>
+      <c r="I4" s="215"/>
+      <c r="J4" s="215"/>
       <c r="K4" s="18"/>
       <c r="R4" s="14"/>
       <c r="S4" s="15"/>
@@ -4832,7 +4832,7 @@
       <c r="U4" s="15"/>
     </row>
     <row r="5" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="272"/>
+      <c r="A5" s="217"/>
       <c r="B5" s="16" t="s">
         <v>56</v>
       </c>
@@ -4842,10 +4842,10 @@
       <c r="F5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="270"/>
-      <c r="H5" s="270"/>
-      <c r="I5" s="270"/>
-      <c r="J5" s="270"/>
+      <c r="G5" s="215"/>
+      <c r="H5" s="215"/>
+      <c r="I5" s="215"/>
+      <c r="J5" s="215"/>
       <c r="K5" s="18"/>
       <c r="R5" s="14"/>
       <c r="S5" s="15"/>
@@ -4853,7 +4853,7 @@
       <c r="U5" s="15"/>
     </row>
     <row r="6" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="272"/>
+      <c r="A6" s="217"/>
       <c r="B6" s="16" t="s">
         <v>57</v>
       </c>
@@ -4863,10 +4863,10 @@
       <c r="F6" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="274"/>
-      <c r="H6" s="274"/>
-      <c r="I6" s="274"/>
-      <c r="J6" s="274"/>
+      <c r="G6" s="219"/>
+      <c r="H6" s="219"/>
+      <c r="I6" s="219"/>
+      <c r="J6" s="219"/>
       <c r="K6" s="20"/>
       <c r="R6" s="14"/>
       <c r="S6" s="15"/>
@@ -4874,7 +4874,7 @@
       <c r="U6" s="15"/>
     </row>
     <row r="7" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="272"/>
+      <c r="A7" s="217"/>
       <c r="B7" s="21" t="s">
         <v>58</v>
       </c>
@@ -4884,10 +4884,10 @@
       <c r="F7" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="274"/>
-      <c r="H7" s="274"/>
-      <c r="I7" s="274"/>
-      <c r="J7" s="274"/>
+      <c r="G7" s="219"/>
+      <c r="H7" s="219"/>
+      <c r="I7" s="219"/>
+      <c r="J7" s="219"/>
       <c r="K7" s="20"/>
       <c r="R7" s="14"/>
       <c r="S7" s="15"/>
@@ -4895,7 +4895,7 @@
       <c r="U7" s="15"/>
     </row>
     <row r="8" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="272"/>
+      <c r="A8" s="217"/>
       <c r="B8" s="16" t="s">
         <v>59</v>
       </c>
@@ -4905,10 +4905,10 @@
       <c r="F8" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G8" s="270"/>
-      <c r="H8" s="270"/>
-      <c r="I8" s="270"/>
-      <c r="J8" s="270"/>
+      <c r="G8" s="215"/>
+      <c r="H8" s="215"/>
+      <c r="I8" s="215"/>
+      <c r="J8" s="215"/>
       <c r="K8" s="20"/>
       <c r="R8" s="14"/>
       <c r="S8" s="15"/>
@@ -4916,7 +4916,7 @@
       <c r="U8" s="15"/>
     </row>
     <row r="9" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="272"/>
+      <c r="A9" s="217"/>
       <c r="B9" s="16" t="s">
         <v>60</v>
       </c>
@@ -4926,10 +4926,10 @@
       <c r="F9" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G9" s="270"/>
-      <c r="H9" s="270"/>
-      <c r="I9" s="270"/>
-      <c r="J9" s="270"/>
+      <c r="G9" s="215"/>
+      <c r="H9" s="215"/>
+      <c r="I9" s="215"/>
+      <c r="J9" s="215"/>
       <c r="K9" s="18"/>
       <c r="R9" s="14"/>
       <c r="S9" s="15"/>
@@ -4937,7 +4937,7 @@
       <c r="U9" s="15"/>
     </row>
     <row r="10" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="272"/>
+      <c r="A10" s="217"/>
       <c r="B10" s="16" t="s">
         <v>61</v>
       </c>
@@ -4947,10 +4947,10 @@
       <c r="F10" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G10" s="270"/>
-      <c r="H10" s="270"/>
-      <c r="I10" s="270"/>
-      <c r="J10" s="270"/>
+      <c r="G10" s="215"/>
+      <c r="H10" s="215"/>
+      <c r="I10" s="215"/>
+      <c r="J10" s="215"/>
       <c r="K10" s="18"/>
       <c r="R10" s="14"/>
       <c r="S10" s="15"/>
@@ -4958,7 +4958,7 @@
       <c r="U10" s="15"/>
     </row>
     <row r="11" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="272"/>
+      <c r="A11" s="217"/>
       <c r="B11" s="22" t="s">
         <v>62</v>
       </c>
@@ -4968,10 +4968,10 @@
       <c r="F11" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="270"/>
-      <c r="H11" s="270"/>
-      <c r="I11" s="270"/>
-      <c r="J11" s="270"/>
+      <c r="G11" s="215"/>
+      <c r="H11" s="215"/>
+      <c r="I11" s="215"/>
+      <c r="J11" s="215"/>
       <c r="K11" s="18"/>
       <c r="L11" s="18"/>
       <c r="M11" s="18"/>
@@ -4985,7 +4985,7 @@
       <c r="U11" s="15"/>
     </row>
     <row r="12" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="272"/>
+      <c r="A12" s="217"/>
       <c r="B12" s="22" t="s">
         <v>63</v>
       </c>
@@ -4995,10 +4995,10 @@
       <c r="F12" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G12" s="270"/>
-      <c r="H12" s="270"/>
-      <c r="I12" s="270"/>
-      <c r="J12" s="270"/>
+      <c r="G12" s="215"/>
+      <c r="H12" s="215"/>
+      <c r="I12" s="215"/>
+      <c r="J12" s="215"/>
       <c r="K12" s="18"/>
       <c r="L12" s="24"/>
       <c r="M12" s="24"/>
@@ -5009,7 +5009,7 @@
       <c r="R12" s="25"/>
     </row>
     <row r="13" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="272"/>
+      <c r="A13" s="217"/>
       <c r="B13" s="26" t="s">
         <v>64</v>
       </c>
@@ -5019,10 +5019,10 @@
       <c r="F13" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G13" s="274"/>
-      <c r="H13" s="274"/>
-      <c r="I13" s="274"/>
-      <c r="J13" s="274"/>
+      <c r="G13" s="219"/>
+      <c r="H13" s="219"/>
+      <c r="I13" s="219"/>
+      <c r="J13" s="219"/>
       <c r="K13" s="24"/>
       <c r="L13" s="18"/>
       <c r="M13" s="24"/>
@@ -5033,7 +5033,7 @@
       <c r="R13" s="25"/>
     </row>
     <row r="14" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="272"/>
+      <c r="A14" s="217"/>
       <c r="B14" s="22" t="s">
         <v>65</v>
       </c>
@@ -5043,10 +5043,10 @@
       <c r="F14" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G14" s="274"/>
-      <c r="H14" s="274"/>
-      <c r="I14" s="274"/>
-      <c r="J14" s="274"/>
+      <c r="G14" s="219"/>
+      <c r="H14" s="219"/>
+      <c r="I14" s="219"/>
+      <c r="J14" s="219"/>
       <c r="K14" s="24"/>
       <c r="L14" s="18"/>
       <c r="M14" s="24"/>
@@ -5057,7 +5057,7 @@
       <c r="R14" s="25"/>
     </row>
     <row r="15" spans="1:21" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="272"/>
+      <c r="A15" s="217"/>
       <c r="B15" s="22" t="s">
         <v>66</v>
       </c>
@@ -5067,10 +5067,10 @@
       <c r="F15" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G15" s="270"/>
-      <c r="H15" s="270"/>
-      <c r="I15" s="270"/>
-      <c r="J15" s="270"/>
+      <c r="G15" s="215"/>
+      <c r="H15" s="215"/>
+      <c r="I15" s="215"/>
+      <c r="J15" s="215"/>
       <c r="K15" s="24"/>
       <c r="L15" s="18"/>
       <c r="M15" s="24"/>
@@ -5081,7 +5081,7 @@
       <c r="R15" s="25"/>
     </row>
     <row r="16" spans="1:21" s="8" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="272"/>
+      <c r="A16" s="217"/>
       <c r="B16" s="22" t="s">
         <v>67</v>
       </c>
@@ -5091,10 +5091,10 @@
       <c r="F16" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G16" s="270"/>
-      <c r="H16" s="270"/>
-      <c r="I16" s="270"/>
-      <c r="J16" s="270"/>
+      <c r="G16" s="215"/>
+      <c r="H16" s="215"/>
+      <c r="I16" s="215"/>
+      <c r="J16" s="215"/>
       <c r="K16" s="24"/>
       <c r="L16" s="18"/>
       <c r="M16" s="24"/>
@@ -5105,7 +5105,7 @@
       <c r="R16" s="25"/>
     </row>
     <row r="17" spans="1:23" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="272"/>
+      <c r="A17" s="217"/>
       <c r="B17" s="22"/>
       <c r="C17" s="28"/>
       <c r="D17" s="28"/>
@@ -5125,7 +5125,7 @@
       <c r="R17" s="25"/>
     </row>
     <row r="18" spans="1:23" s="8" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="272"/>
+      <c r="A18" s="217"/>
       <c r="B18" s="22"/>
       <c r="C18" s="28"/>
       <c r="D18" s="28"/>
@@ -5145,7 +5145,7 @@
       <c r="R18" s="25"/>
     </row>
     <row r="19" spans="1:23" s="8" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="272"/>
+      <c r="A19" s="217"/>
       <c r="B19" s="22"/>
       <c r="C19" s="24"/>
       <c r="D19" s="24"/>
@@ -5165,7 +5165,7 @@
       <c r="R19" s="25"/>
     </row>
     <row r="20" spans="1:23" s="8" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="272"/>
+      <c r="A20" s="217"/>
       <c r="B20" s="33" t="s">
         <v>68</v>
       </c>
@@ -5187,23 +5187,23 @@
       <c r="R20" s="36"/>
     </row>
     <row r="21" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="272"/>
+      <c r="A21" s="217"/>
       <c r="B21" s="38"/>
-      <c r="C21" s="248"/>
-      <c r="D21" s="248"/>
-      <c r="E21" s="248"/>
-      <c r="F21" s="248"/>
-      <c r="G21" s="248"/>
-      <c r="H21" s="248"/>
-      <c r="I21" s="248"/>
-      <c r="J21" s="248"/>
-      <c r="K21" s="248"/>
-      <c r="L21" s="248"/>
-      <c r="M21" s="248"/>
-      <c r="N21" s="248"/>
-      <c r="O21" s="248"/>
-      <c r="P21" s="248"/>
-      <c r="Q21" s="248"/>
+      <c r="C21" s="220"/>
+      <c r="D21" s="220"/>
+      <c r="E21" s="220"/>
+      <c r="F21" s="220"/>
+      <c r="G21" s="220"/>
+      <c r="H21" s="220"/>
+      <c r="I21" s="220"/>
+      <c r="J21" s="220"/>
+      <c r="K21" s="220"/>
+      <c r="L21" s="220"/>
+      <c r="M21" s="220"/>
+      <c r="N21" s="220"/>
+      <c r="O21" s="220"/>
+      <c r="P21" s="220"/>
+      <c r="Q21" s="220"/>
       <c r="R21" s="39"/>
       <c r="S21" s="40"/>
       <c r="T21" s="41"/>
@@ -5212,23 +5212,23 @@
       <c r="W21" s="41"/>
     </row>
     <row r="22" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="272"/>
+      <c r="A22" s="217"/>
       <c r="B22" s="38"/>
-      <c r="C22" s="248"/>
-      <c r="D22" s="248"/>
-      <c r="E22" s="248"/>
-      <c r="F22" s="248"/>
-      <c r="G22" s="248"/>
-      <c r="H22" s="248"/>
-      <c r="I22" s="248"/>
-      <c r="J22" s="248"/>
-      <c r="K22" s="248"/>
-      <c r="L22" s="248"/>
-      <c r="M22" s="248"/>
-      <c r="N22" s="248"/>
-      <c r="O22" s="248"/>
-      <c r="P22" s="248"/>
-      <c r="Q22" s="248"/>
+      <c r="C22" s="220"/>
+      <c r="D22" s="220"/>
+      <c r="E22" s="220"/>
+      <c r="F22" s="220"/>
+      <c r="G22" s="220"/>
+      <c r="H22" s="220"/>
+      <c r="I22" s="220"/>
+      <c r="J22" s="220"/>
+      <c r="K22" s="220"/>
+      <c r="L22" s="220"/>
+      <c r="M22" s="220"/>
+      <c r="N22" s="220"/>
+      <c r="O22" s="220"/>
+      <c r="P22" s="220"/>
+      <c r="Q22" s="220"/>
       <c r="R22" s="39"/>
       <c r="S22" s="40"/>
       <c r="T22" s="41"/>
@@ -5237,23 +5237,23 @@
       <c r="W22" s="41"/>
     </row>
     <row r="23" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="272"/>
+      <c r="A23" s="217"/>
       <c r="B23" s="38"/>
-      <c r="C23" s="248"/>
-      <c r="D23" s="248"/>
-      <c r="E23" s="248"/>
-      <c r="F23" s="248"/>
-      <c r="G23" s="248"/>
-      <c r="H23" s="248"/>
-      <c r="I23" s="248"/>
-      <c r="J23" s="248"/>
-      <c r="K23" s="248"/>
-      <c r="L23" s="248"/>
-      <c r="M23" s="248"/>
-      <c r="N23" s="248"/>
-      <c r="O23" s="248"/>
-      <c r="P23" s="248"/>
-      <c r="Q23" s="248"/>
+      <c r="C23" s="220"/>
+      <c r="D23" s="220"/>
+      <c r="E23" s="220"/>
+      <c r="F23" s="220"/>
+      <c r="G23" s="220"/>
+      <c r="H23" s="220"/>
+      <c r="I23" s="220"/>
+      <c r="J23" s="220"/>
+      <c r="K23" s="220"/>
+      <c r="L23" s="220"/>
+      <c r="M23" s="220"/>
+      <c r="N23" s="220"/>
+      <c r="O23" s="220"/>
+      <c r="P23" s="220"/>
+      <c r="Q23" s="220"/>
       <c r="R23" s="39"/>
       <c r="S23" s="40"/>
       <c r="T23" s="41"/>
@@ -5262,23 +5262,23 @@
       <c r="W23" s="41"/>
     </row>
     <row r="24" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="272"/>
+      <c r="A24" s="217"/>
       <c r="B24" s="38"/>
-      <c r="C24" s="248"/>
-      <c r="D24" s="248"/>
-      <c r="E24" s="248"/>
-      <c r="F24" s="248"/>
-      <c r="G24" s="248"/>
-      <c r="H24" s="248"/>
-      <c r="I24" s="248"/>
-      <c r="J24" s="248"/>
-      <c r="K24" s="248"/>
-      <c r="L24" s="248"/>
-      <c r="M24" s="248"/>
-      <c r="N24" s="248"/>
-      <c r="O24" s="248"/>
-      <c r="P24" s="248"/>
-      <c r="Q24" s="248"/>
+      <c r="C24" s="220"/>
+      <c r="D24" s="220"/>
+      <c r="E24" s="220"/>
+      <c r="F24" s="220"/>
+      <c r="G24" s="220"/>
+      <c r="H24" s="220"/>
+      <c r="I24" s="220"/>
+      <c r="J24" s="220"/>
+      <c r="K24" s="220"/>
+      <c r="L24" s="220"/>
+      <c r="M24" s="220"/>
+      <c r="N24" s="220"/>
+      <c r="O24" s="220"/>
+      <c r="P24" s="220"/>
+      <c r="Q24" s="220"/>
       <c r="R24" s="39"/>
       <c r="S24" s="40"/>
       <c r="T24" s="41"/>
@@ -5287,23 +5287,23 @@
       <c r="W24" s="41"/>
     </row>
     <row r="25" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="272"/>
+      <c r="A25" s="217"/>
       <c r="B25" s="38"/>
-      <c r="C25" s="248"/>
-      <c r="D25" s="248"/>
-      <c r="E25" s="248"/>
-      <c r="F25" s="248"/>
-      <c r="G25" s="248"/>
-      <c r="H25" s="248"/>
-      <c r="I25" s="248"/>
-      <c r="J25" s="248"/>
-      <c r="K25" s="248"/>
-      <c r="L25" s="248"/>
-      <c r="M25" s="248"/>
-      <c r="N25" s="248"/>
-      <c r="O25" s="248"/>
-      <c r="P25" s="248"/>
-      <c r="Q25" s="248"/>
+      <c r="C25" s="220"/>
+      <c r="D25" s="220"/>
+      <c r="E25" s="220"/>
+      <c r="F25" s="220"/>
+      <c r="G25" s="220"/>
+      <c r="H25" s="220"/>
+      <c r="I25" s="220"/>
+      <c r="J25" s="220"/>
+      <c r="K25" s="220"/>
+      <c r="L25" s="220"/>
+      <c r="M25" s="220"/>
+      <c r="N25" s="220"/>
+      <c r="O25" s="220"/>
+      <c r="P25" s="220"/>
+      <c r="Q25" s="220"/>
       <c r="R25" s="42"/>
       <c r="S25" s="40"/>
       <c r="T25" s="41"/>
@@ -5312,23 +5312,23 @@
       <c r="W25" s="41"/>
     </row>
     <row r="26" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="272"/>
+      <c r="A26" s="217"/>
       <c r="B26" s="38"/>
-      <c r="C26" s="248"/>
-      <c r="D26" s="248"/>
-      <c r="E26" s="248"/>
-      <c r="F26" s="248"/>
-      <c r="G26" s="248"/>
-      <c r="H26" s="248"/>
-      <c r="I26" s="248"/>
-      <c r="J26" s="248"/>
-      <c r="K26" s="248"/>
-      <c r="L26" s="248"/>
-      <c r="M26" s="248"/>
-      <c r="N26" s="248"/>
-      <c r="O26" s="248"/>
-      <c r="P26" s="248"/>
-      <c r="Q26" s="248"/>
+      <c r="C26" s="220"/>
+      <c r="D26" s="220"/>
+      <c r="E26" s="220"/>
+      <c r="F26" s="220"/>
+      <c r="G26" s="220"/>
+      <c r="H26" s="220"/>
+      <c r="I26" s="220"/>
+      <c r="J26" s="220"/>
+      <c r="K26" s="220"/>
+      <c r="L26" s="220"/>
+      <c r="M26" s="220"/>
+      <c r="N26" s="220"/>
+      <c r="O26" s="220"/>
+      <c r="P26" s="220"/>
+      <c r="Q26" s="220"/>
       <c r="R26" s="39"/>
       <c r="S26" s="40"/>
       <c r="T26" s="41"/>
@@ -5337,23 +5337,23 @@
       <c r="W26" s="41"/>
     </row>
     <row r="27" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="272"/>
+      <c r="A27" s="217"/>
       <c r="B27" s="38"/>
-      <c r="C27" s="248"/>
-      <c r="D27" s="248"/>
-      <c r="E27" s="248"/>
-      <c r="F27" s="248"/>
-      <c r="G27" s="248"/>
-      <c r="H27" s="248"/>
-      <c r="I27" s="248"/>
-      <c r="J27" s="248"/>
-      <c r="K27" s="248"/>
-      <c r="L27" s="248"/>
-      <c r="M27" s="248"/>
-      <c r="N27" s="248"/>
-      <c r="O27" s="248"/>
-      <c r="P27" s="248"/>
-      <c r="Q27" s="248"/>
+      <c r="C27" s="220"/>
+      <c r="D27" s="220"/>
+      <c r="E27" s="220"/>
+      <c r="F27" s="220"/>
+      <c r="G27" s="220"/>
+      <c r="H27" s="220"/>
+      <c r="I27" s="220"/>
+      <c r="J27" s="220"/>
+      <c r="K27" s="220"/>
+      <c r="L27" s="220"/>
+      <c r="M27" s="220"/>
+      <c r="N27" s="220"/>
+      <c r="O27" s="220"/>
+      <c r="P27" s="220"/>
+      <c r="Q27" s="220"/>
       <c r="R27" s="39"/>
       <c r="S27" s="40"/>
       <c r="T27" s="41"/>
@@ -5362,23 +5362,23 @@
       <c r="W27" s="41"/>
     </row>
     <row r="28" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="272"/>
+      <c r="A28" s="217"/>
       <c r="B28" s="38"/>
-      <c r="C28" s="248"/>
-      <c r="D28" s="248"/>
-      <c r="E28" s="248"/>
-      <c r="F28" s="248"/>
-      <c r="G28" s="248"/>
-      <c r="H28" s="248"/>
-      <c r="I28" s="248"/>
-      <c r="J28" s="248"/>
-      <c r="K28" s="248"/>
-      <c r="L28" s="248"/>
-      <c r="M28" s="248"/>
-      <c r="N28" s="248"/>
-      <c r="O28" s="248"/>
-      <c r="P28" s="248"/>
-      <c r="Q28" s="248"/>
+      <c r="C28" s="220"/>
+      <c r="D28" s="220"/>
+      <c r="E28" s="220"/>
+      <c r="F28" s="220"/>
+      <c r="G28" s="220"/>
+      <c r="H28" s="220"/>
+      <c r="I28" s="220"/>
+      <c r="J28" s="220"/>
+      <c r="K28" s="220"/>
+      <c r="L28" s="220"/>
+      <c r="M28" s="220"/>
+      <c r="N28" s="220"/>
+      <c r="O28" s="220"/>
+      <c r="P28" s="220"/>
+      <c r="Q28" s="220"/>
       <c r="R28" s="39"/>
       <c r="S28" s="40"/>
       <c r="T28" s="41"/>
@@ -5387,7 +5387,7 @@
       <c r="W28" s="41"/>
     </row>
     <row r="29" spans="1:23" s="37" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="272"/>
+      <c r="A29" s="217"/>
       <c r="B29" s="38"/>
       <c r="C29" s="43"/>
       <c r="D29" s="43"/>
@@ -5412,7 +5412,7 @@
       <c r="W29" s="41"/>
     </row>
     <row r="30" spans="1:23" s="8" customFormat="1" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="272"/>
+      <c r="A30" s="217"/>
       <c r="B30" s="46"/>
       <c r="C30" s="47"/>
       <c r="D30" s="47"/>
@@ -5432,7 +5432,7 @@
       <c r="R30" s="50"/>
     </row>
     <row r="31" spans="1:23" s="8" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="272"/>
+      <c r="A31" s="217"/>
       <c r="B31" s="51" t="s">
         <v>69</v>
       </c>
@@ -5454,107 +5454,107 @@
       <c r="R31" s="55"/>
     </row>
     <row r="32" spans="1:23" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="272"/>
+      <c r="A32" s="217"/>
       <c r="B32" s="57"/>
-      <c r="C32" s="248"/>
-      <c r="D32" s="248"/>
-      <c r="E32" s="248"/>
-      <c r="F32" s="248"/>
-      <c r="G32" s="248"/>
-      <c r="H32" s="248"/>
-      <c r="I32" s="248"/>
-      <c r="J32" s="248"/>
-      <c r="K32" s="248"/>
-      <c r="L32" s="248"/>
-      <c r="M32" s="248"/>
-      <c r="N32" s="248"/>
-      <c r="O32" s="248"/>
-      <c r="P32" s="248"/>
-      <c r="Q32" s="248"/>
+      <c r="C32" s="220"/>
+      <c r="D32" s="220"/>
+      <c r="E32" s="220"/>
+      <c r="F32" s="220"/>
+      <c r="G32" s="220"/>
+      <c r="H32" s="220"/>
+      <c r="I32" s="220"/>
+      <c r="J32" s="220"/>
+      <c r="K32" s="220"/>
+      <c r="L32" s="220"/>
+      <c r="M32" s="220"/>
+      <c r="N32" s="220"/>
+      <c r="O32" s="220"/>
+      <c r="P32" s="220"/>
+      <c r="Q32" s="220"/>
       <c r="R32" s="58"/>
     </row>
     <row r="33" spans="1:18" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="272"/>
+      <c r="A33" s="217"/>
       <c r="B33" s="57"/>
-      <c r="C33" s="248"/>
-      <c r="D33" s="248"/>
-      <c r="E33" s="248"/>
-      <c r="F33" s="248"/>
-      <c r="G33" s="248"/>
-      <c r="H33" s="248"/>
-      <c r="I33" s="248"/>
-      <c r="J33" s="248"/>
-      <c r="K33" s="248"/>
-      <c r="L33" s="248"/>
-      <c r="M33" s="248"/>
-      <c r="N33" s="248"/>
-      <c r="O33" s="248"/>
-      <c r="P33" s="248"/>
-      <c r="Q33" s="248"/>
+      <c r="C33" s="220"/>
+      <c r="D33" s="220"/>
+      <c r="E33" s="220"/>
+      <c r="F33" s="220"/>
+      <c r="G33" s="220"/>
+      <c r="H33" s="220"/>
+      <c r="I33" s="220"/>
+      <c r="J33" s="220"/>
+      <c r="K33" s="220"/>
+      <c r="L33" s="220"/>
+      <c r="M33" s="220"/>
+      <c r="N33" s="220"/>
+      <c r="O33" s="220"/>
+      <c r="P33" s="220"/>
+      <c r="Q33" s="220"/>
       <c r="R33" s="58"/>
     </row>
     <row r="34" spans="1:18" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="272"/>
+      <c r="A34" s="217"/>
       <c r="B34" s="57"/>
-      <c r="C34" s="248"/>
-      <c r="D34" s="248"/>
-      <c r="E34" s="248"/>
-      <c r="F34" s="248"/>
-      <c r="G34" s="248"/>
-      <c r="H34" s="248"/>
-      <c r="I34" s="248"/>
-      <c r="J34" s="248"/>
-      <c r="K34" s="248"/>
-      <c r="L34" s="248"/>
-      <c r="M34" s="248"/>
-      <c r="N34" s="248"/>
-      <c r="O34" s="248"/>
-      <c r="P34" s="248"/>
-      <c r="Q34" s="248"/>
+      <c r="C34" s="220"/>
+      <c r="D34" s="220"/>
+      <c r="E34" s="220"/>
+      <c r="F34" s="220"/>
+      <c r="G34" s="220"/>
+      <c r="H34" s="220"/>
+      <c r="I34" s="220"/>
+      <c r="J34" s="220"/>
+      <c r="K34" s="220"/>
+      <c r="L34" s="220"/>
+      <c r="M34" s="220"/>
+      <c r="N34" s="220"/>
+      <c r="O34" s="220"/>
+      <c r="P34" s="220"/>
+      <c r="Q34" s="220"/>
       <c r="R34" s="58"/>
     </row>
     <row r="35" spans="1:18" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="272"/>
+      <c r="A35" s="217"/>
       <c r="B35" s="57"/>
-      <c r="C35" s="248"/>
-      <c r="D35" s="248"/>
-      <c r="E35" s="248"/>
-      <c r="F35" s="248"/>
-      <c r="G35" s="248"/>
-      <c r="H35" s="248"/>
-      <c r="I35" s="248"/>
-      <c r="J35" s="248"/>
-      <c r="K35" s="248"/>
-      <c r="L35" s="248"/>
-      <c r="M35" s="248"/>
-      <c r="N35" s="248"/>
-      <c r="O35" s="248"/>
-      <c r="P35" s="248"/>
-      <c r="Q35" s="248"/>
+      <c r="C35" s="220"/>
+      <c r="D35" s="220"/>
+      <c r="E35" s="220"/>
+      <c r="F35" s="220"/>
+      <c r="G35" s="220"/>
+      <c r="H35" s="220"/>
+      <c r="I35" s="220"/>
+      <c r="J35" s="220"/>
+      <c r="K35" s="220"/>
+      <c r="L35" s="220"/>
+      <c r="M35" s="220"/>
+      <c r="N35" s="220"/>
+      <c r="O35" s="220"/>
+      <c r="P35" s="220"/>
+      <c r="Q35" s="220"/>
       <c r="R35" s="58"/>
     </row>
     <row r="36" spans="1:18" s="56" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="272"/>
+      <c r="A36" s="217"/>
       <c r="B36" s="57"/>
-      <c r="C36" s="248"/>
-      <c r="D36" s="248"/>
-      <c r="E36" s="248"/>
-      <c r="F36" s="248"/>
-      <c r="G36" s="248"/>
-      <c r="H36" s="248"/>
-      <c r="I36" s="248"/>
-      <c r="J36" s="248"/>
-      <c r="K36" s="248"/>
-      <c r="L36" s="248"/>
-      <c r="M36" s="248"/>
-      <c r="N36" s="248"/>
-      <c r="O36" s="248"/>
-      <c r="P36" s="248"/>
-      <c r="Q36" s="248"/>
+      <c r="C36" s="220"/>
+      <c r="D36" s="220"/>
+      <c r="E36" s="220"/>
+      <c r="F36" s="220"/>
+      <c r="G36" s="220"/>
+      <c r="H36" s="220"/>
+      <c r="I36" s="220"/>
+      <c r="J36" s="220"/>
+      <c r="K36" s="220"/>
+      <c r="L36" s="220"/>
+      <c r="M36" s="220"/>
+      <c r="N36" s="220"/>
+      <c r="O36" s="220"/>
+      <c r="P36" s="220"/>
+      <c r="Q36" s="220"/>
       <c r="R36" s="58"/>
     </row>
     <row r="37" spans="1:18" s="8" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="272"/>
+      <c r="A37" s="217"/>
       <c r="B37" s="59"/>
       <c r="C37" s="24"/>
       <c r="D37" s="24"/>
@@ -5574,337 +5574,337 @@
       <c r="R37" s="25"/>
     </row>
     <row r="38" spans="1:18" s="8" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="272"/>
-      <c r="B38" s="249" t="s">
+      <c r="A38" s="217"/>
+      <c r="B38" s="221" t="s">
         <v>70</v>
       </c>
-      <c r="C38" s="250"/>
-      <c r="D38" s="250"/>
-      <c r="E38" s="250"/>
-      <c r="F38" s="250"/>
-      <c r="G38" s="250"/>
-      <c r="H38" s="250"/>
-      <c r="I38" s="250"/>
-      <c r="J38" s="250"/>
-      <c r="K38" s="250"/>
-      <c r="L38" s="250"/>
-      <c r="M38" s="250"/>
-      <c r="N38" s="250"/>
-      <c r="O38" s="250"/>
-      <c r="P38" s="250"/>
-      <c r="Q38" s="250"/>
-      <c r="R38" s="251"/>
+      <c r="C38" s="222"/>
+      <c r="D38" s="222"/>
+      <c r="E38" s="222"/>
+      <c r="F38" s="222"/>
+      <c r="G38" s="222"/>
+      <c r="H38" s="222"/>
+      <c r="I38" s="222"/>
+      <c r="J38" s="222"/>
+      <c r="K38" s="222"/>
+      <c r="L38" s="222"/>
+      <c r="M38" s="222"/>
+      <c r="N38" s="222"/>
+      <c r="O38" s="222"/>
+      <c r="P38" s="222"/>
+      <c r="Q38" s="222"/>
+      <c r="R38" s="223"/>
     </row>
     <row r="39" spans="1:18" s="61" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="272"/>
-      <c r="B39" s="261" t="s">
+      <c r="A39" s="217"/>
+      <c r="B39" s="233" t="s">
         <v>71</v>
       </c>
-      <c r="C39" s="252" t="s">
+      <c r="C39" s="224" t="s">
         <v>72</v>
       </c>
-      <c r="D39" s="253"/>
-      <c r="E39" s="254"/>
-      <c r="F39" s="252" t="s">
+      <c r="D39" s="225"/>
+      <c r="E39" s="226"/>
+      <c r="F39" s="224" t="s">
         <v>73</v>
       </c>
-      <c r="G39" s="254"/>
-      <c r="H39" s="258" t="s">
+      <c r="G39" s="226"/>
+      <c r="H39" s="230" t="s">
         <v>74</v>
       </c>
-      <c r="I39" s="259"/>
-      <c r="J39" s="259"/>
-      <c r="K39" s="260"/>
-      <c r="L39" s="252" t="s">
+      <c r="I39" s="231"/>
+      <c r="J39" s="231"/>
+      <c r="K39" s="232"/>
+      <c r="L39" s="224" t="s">
         <v>75</v>
       </c>
-      <c r="M39" s="253"/>
-      <c r="N39" s="254"/>
-      <c r="O39" s="252" t="s">
+      <c r="M39" s="225"/>
+      <c r="N39" s="226"/>
+      <c r="O39" s="224" t="s">
         <v>76</v>
       </c>
-      <c r="P39" s="254"/>
-      <c r="Q39" s="263" t="s">
+      <c r="P39" s="226"/>
+      <c r="Q39" s="235" t="s">
         <v>77</v>
       </c>
-      <c r="R39" s="265" t="s">
+      <c r="R39" s="237" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:18" s="61" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="272"/>
-      <c r="B40" s="262"/>
-      <c r="C40" s="255"/>
-      <c r="D40" s="256"/>
-      <c r="E40" s="257"/>
-      <c r="F40" s="255"/>
-      <c r="G40" s="257"/>
-      <c r="H40" s="258" t="s">
+      <c r="A40" s="217"/>
+      <c r="B40" s="234"/>
+      <c r="C40" s="227"/>
+      <c r="D40" s="228"/>
+      <c r="E40" s="229"/>
+      <c r="F40" s="227"/>
+      <c r="G40" s="229"/>
+      <c r="H40" s="230" t="s">
         <v>79</v>
       </c>
-      <c r="I40" s="259"/>
-      <c r="J40" s="259"/>
-      <c r="K40" s="260"/>
-      <c r="L40" s="255"/>
-      <c r="M40" s="256"/>
-      <c r="N40" s="257"/>
-      <c r="O40" s="255"/>
-      <c r="P40" s="257"/>
-      <c r="Q40" s="264"/>
-      <c r="R40" s="266"/>
+      <c r="I40" s="231"/>
+      <c r="J40" s="231"/>
+      <c r="K40" s="232"/>
+      <c r="L40" s="227"/>
+      <c r="M40" s="228"/>
+      <c r="N40" s="229"/>
+      <c r="O40" s="227"/>
+      <c r="P40" s="229"/>
+      <c r="Q40" s="236"/>
+      <c r="R40" s="238"/>
     </row>
     <row r="41" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="272"/>
+      <c r="A41" s="217"/>
       <c r="B41" s="62"/>
-      <c r="C41" s="223"/>
-      <c r="D41" s="223"/>
-      <c r="E41" s="223"/>
-      <c r="F41" s="238"/>
-      <c r="G41" s="238"/>
-      <c r="H41" s="239"/>
-      <c r="I41" s="240"/>
-      <c r="J41" s="240"/>
-      <c r="K41" s="241"/>
-      <c r="L41" s="237"/>
-      <c r="M41" s="237"/>
-      <c r="N41" s="237"/>
-      <c r="O41" s="234"/>
-      <c r="P41" s="235"/>
+      <c r="C41" s="239"/>
+      <c r="D41" s="239"/>
+      <c r="E41" s="239"/>
+      <c r="F41" s="240"/>
+      <c r="G41" s="240"/>
+      <c r="H41" s="241"/>
+      <c r="I41" s="242"/>
+      <c r="J41" s="242"/>
+      <c r="K41" s="243"/>
+      <c r="L41" s="250"/>
+      <c r="M41" s="250"/>
+      <c r="N41" s="250"/>
+      <c r="O41" s="251"/>
+      <c r="P41" s="252"/>
       <c r="Q41" s="64"/>
       <c r="R41" s="65"/>
     </row>
     <row r="42" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="272"/>
+      <c r="A42" s="217"/>
       <c r="B42" s="66"/>
-      <c r="C42" s="223"/>
-      <c r="D42" s="223"/>
-      <c r="E42" s="223"/>
-      <c r="F42" s="236"/>
-      <c r="G42" s="236"/>
-      <c r="H42" s="242"/>
-      <c r="I42" s="243"/>
-      <c r="J42" s="243"/>
-      <c r="K42" s="244"/>
-      <c r="L42" s="237"/>
-      <c r="M42" s="237"/>
-      <c r="N42" s="237"/>
-      <c r="O42" s="234"/>
-      <c r="P42" s="235"/>
+      <c r="C42" s="239"/>
+      <c r="D42" s="239"/>
+      <c r="E42" s="239"/>
+      <c r="F42" s="253"/>
+      <c r="G42" s="253"/>
+      <c r="H42" s="244"/>
+      <c r="I42" s="245"/>
+      <c r="J42" s="245"/>
+      <c r="K42" s="246"/>
+      <c r="L42" s="250"/>
+      <c r="M42" s="250"/>
+      <c r="N42" s="250"/>
+      <c r="O42" s="251"/>
+      <c r="P42" s="252"/>
       <c r="Q42" s="63"/>
       <c r="R42" s="67"/>
     </row>
     <row r="43" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="272"/>
+      <c r="A43" s="217"/>
       <c r="B43" s="66"/>
-      <c r="C43" s="223"/>
-      <c r="D43" s="223"/>
-      <c r="E43" s="223"/>
-      <c r="F43" s="236"/>
-      <c r="G43" s="236"/>
-      <c r="H43" s="242"/>
-      <c r="I43" s="243"/>
-      <c r="J43" s="243"/>
-      <c r="K43" s="244"/>
-      <c r="L43" s="237"/>
-      <c r="M43" s="237"/>
-      <c r="N43" s="237"/>
-      <c r="O43" s="234"/>
-      <c r="P43" s="235"/>
+      <c r="C43" s="239"/>
+      <c r="D43" s="239"/>
+      <c r="E43" s="239"/>
+      <c r="F43" s="253"/>
+      <c r="G43" s="253"/>
+      <c r="H43" s="244"/>
+      <c r="I43" s="245"/>
+      <c r="J43" s="245"/>
+      <c r="K43" s="246"/>
+      <c r="L43" s="250"/>
+      <c r="M43" s="250"/>
+      <c r="N43" s="250"/>
+      <c r="O43" s="251"/>
+      <c r="P43" s="252"/>
       <c r="Q43" s="63"/>
       <c r="R43" s="67"/>
     </row>
     <row r="44" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="272"/>
+      <c r="A44" s="217"/>
       <c r="B44" s="66"/>
-      <c r="C44" s="223"/>
-      <c r="D44" s="223"/>
-      <c r="E44" s="223"/>
-      <c r="F44" s="236"/>
-      <c r="G44" s="236"/>
-      <c r="H44" s="242"/>
-      <c r="I44" s="243"/>
-      <c r="J44" s="243"/>
-      <c r="K44" s="244"/>
-      <c r="L44" s="237"/>
-      <c r="M44" s="237"/>
-      <c r="N44" s="237"/>
-      <c r="O44" s="234"/>
-      <c r="P44" s="235"/>
+      <c r="C44" s="239"/>
+      <c r="D44" s="239"/>
+      <c r="E44" s="239"/>
+      <c r="F44" s="253"/>
+      <c r="G44" s="253"/>
+      <c r="H44" s="244"/>
+      <c r="I44" s="245"/>
+      <c r="J44" s="245"/>
+      <c r="K44" s="246"/>
+      <c r="L44" s="250"/>
+      <c r="M44" s="250"/>
+      <c r="N44" s="250"/>
+      <c r="O44" s="251"/>
+      <c r="P44" s="252"/>
       <c r="Q44" s="63"/>
       <c r="R44" s="67"/>
     </row>
     <row r="45" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="272"/>
+      <c r="A45" s="217"/>
       <c r="B45" s="66"/>
-      <c r="C45" s="223"/>
-      <c r="D45" s="223"/>
-      <c r="E45" s="223"/>
-      <c r="F45" s="236"/>
-      <c r="G45" s="236"/>
-      <c r="H45" s="242"/>
-      <c r="I45" s="243"/>
-      <c r="J45" s="243"/>
-      <c r="K45" s="244"/>
-      <c r="L45" s="237"/>
-      <c r="M45" s="237"/>
-      <c r="N45" s="237"/>
-      <c r="O45" s="234"/>
-      <c r="P45" s="235"/>
+      <c r="C45" s="239"/>
+      <c r="D45" s="239"/>
+      <c r="E45" s="239"/>
+      <c r="F45" s="253"/>
+      <c r="G45" s="253"/>
+      <c r="H45" s="244"/>
+      <c r="I45" s="245"/>
+      <c r="J45" s="245"/>
+      <c r="K45" s="246"/>
+      <c r="L45" s="250"/>
+      <c r="M45" s="250"/>
+      <c r="N45" s="250"/>
+      <c r="O45" s="251"/>
+      <c r="P45" s="252"/>
       <c r="Q45" s="63"/>
       <c r="R45" s="67"/>
     </row>
     <row r="46" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="272"/>
+      <c r="A46" s="217"/>
       <c r="B46" s="66"/>
-      <c r="C46" s="223"/>
-      <c r="D46" s="223"/>
-      <c r="E46" s="223"/>
-      <c r="F46" s="236"/>
-      <c r="G46" s="236"/>
-      <c r="H46" s="242"/>
-      <c r="I46" s="243"/>
-      <c r="J46" s="243"/>
-      <c r="K46" s="244"/>
-      <c r="L46" s="237"/>
-      <c r="M46" s="237"/>
-      <c r="N46" s="237"/>
-      <c r="O46" s="234"/>
-      <c r="P46" s="235"/>
+      <c r="C46" s="239"/>
+      <c r="D46" s="239"/>
+      <c r="E46" s="239"/>
+      <c r="F46" s="253"/>
+      <c r="G46" s="253"/>
+      <c r="H46" s="244"/>
+      <c r="I46" s="245"/>
+      <c r="J46" s="245"/>
+      <c r="K46" s="246"/>
+      <c r="L46" s="250"/>
+      <c r="M46" s="250"/>
+      <c r="N46" s="250"/>
+      <c r="O46" s="251"/>
+      <c r="P46" s="252"/>
       <c r="Q46" s="63"/>
       <c r="R46" s="67"/>
     </row>
     <row r="47" spans="1:18" s="61" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="272"/>
+      <c r="A47" s="217"/>
       <c r="B47" s="66"/>
-      <c r="C47" s="223"/>
-      <c r="D47" s="223"/>
-      <c r="E47" s="223"/>
-      <c r="F47" s="236"/>
-      <c r="G47" s="236"/>
-      <c r="H47" s="242"/>
-      <c r="I47" s="243"/>
-      <c r="J47" s="243"/>
-      <c r="K47" s="244"/>
-      <c r="L47" s="237"/>
-      <c r="M47" s="237"/>
-      <c r="N47" s="237"/>
-      <c r="O47" s="234"/>
-      <c r="P47" s="235"/>
+      <c r="C47" s="239"/>
+      <c r="D47" s="239"/>
+      <c r="E47" s="239"/>
+      <c r="F47" s="253"/>
+      <c r="G47" s="253"/>
+      <c r="H47" s="244"/>
+      <c r="I47" s="245"/>
+      <c r="J47" s="245"/>
+      <c r="K47" s="246"/>
+      <c r="L47" s="250"/>
+      <c r="M47" s="250"/>
+      <c r="N47" s="250"/>
+      <c r="O47" s="251"/>
+      <c r="P47" s="252"/>
       <c r="Q47" s="63"/>
       <c r="R47" s="67"/>
     </row>
     <row r="48" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="272"/>
+      <c r="A48" s="217"/>
       <c r="B48" s="68"/>
-      <c r="C48" s="223"/>
-      <c r="D48" s="223"/>
-      <c r="E48" s="223"/>
-      <c r="F48" s="232"/>
-      <c r="G48" s="232"/>
-      <c r="H48" s="242"/>
-      <c r="I48" s="243"/>
-      <c r="J48" s="243"/>
-      <c r="K48" s="244"/>
-      <c r="L48" s="233"/>
-      <c r="M48" s="233"/>
-      <c r="N48" s="233"/>
-      <c r="O48" s="234"/>
-      <c r="P48" s="235"/>
+      <c r="C48" s="239"/>
+      <c r="D48" s="239"/>
+      <c r="E48" s="239"/>
+      <c r="F48" s="254"/>
+      <c r="G48" s="254"/>
+      <c r="H48" s="244"/>
+      <c r="I48" s="245"/>
+      <c r="J48" s="245"/>
+      <c r="K48" s="246"/>
+      <c r="L48" s="255"/>
+      <c r="M48" s="255"/>
+      <c r="N48" s="255"/>
+      <c r="O48" s="251"/>
+      <c r="P48" s="252"/>
       <c r="Q48" s="69"/>
       <c r="R48" s="70"/>
     </row>
     <row r="49" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="272"/>
+      <c r="A49" s="217"/>
       <c r="B49" s="68"/>
-      <c r="C49" s="223"/>
-      <c r="D49" s="223"/>
-      <c r="E49" s="223"/>
-      <c r="F49" s="232"/>
-      <c r="G49" s="232"/>
-      <c r="H49" s="242"/>
-      <c r="I49" s="243"/>
-      <c r="J49" s="243"/>
-      <c r="K49" s="244"/>
-      <c r="L49" s="233"/>
-      <c r="M49" s="233"/>
-      <c r="N49" s="233"/>
-      <c r="O49" s="234"/>
-      <c r="P49" s="235"/>
+      <c r="C49" s="239"/>
+      <c r="D49" s="239"/>
+      <c r="E49" s="239"/>
+      <c r="F49" s="254"/>
+      <c r="G49" s="254"/>
+      <c r="H49" s="244"/>
+      <c r="I49" s="245"/>
+      <c r="J49" s="245"/>
+      <c r="K49" s="246"/>
+      <c r="L49" s="255"/>
+      <c r="M49" s="255"/>
+      <c r="N49" s="255"/>
+      <c r="O49" s="251"/>
+      <c r="P49" s="252"/>
       <c r="Q49" s="69"/>
       <c r="R49" s="70"/>
     </row>
     <row r="50" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="272"/>
+      <c r="A50" s="217"/>
       <c r="B50" s="66"/>
-      <c r="C50" s="223"/>
-      <c r="D50" s="223"/>
-      <c r="E50" s="223"/>
-      <c r="F50" s="236"/>
-      <c r="G50" s="236"/>
-      <c r="H50" s="242"/>
-      <c r="I50" s="243"/>
-      <c r="J50" s="243"/>
-      <c r="K50" s="244"/>
-      <c r="L50" s="237"/>
-      <c r="M50" s="237"/>
-      <c r="N50" s="237"/>
-      <c r="O50" s="234"/>
-      <c r="P50" s="235"/>
+      <c r="C50" s="239"/>
+      <c r="D50" s="239"/>
+      <c r="E50" s="239"/>
+      <c r="F50" s="253"/>
+      <c r="G50" s="253"/>
+      <c r="H50" s="244"/>
+      <c r="I50" s="245"/>
+      <c r="J50" s="245"/>
+      <c r="K50" s="246"/>
+      <c r="L50" s="250"/>
+      <c r="M50" s="250"/>
+      <c r="N50" s="250"/>
+      <c r="O50" s="251"/>
+      <c r="P50" s="252"/>
       <c r="Q50" s="63"/>
       <c r="R50" s="67"/>
     </row>
     <row r="51" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="272"/>
+      <c r="A51" s="217"/>
       <c r="B51" s="66"/>
-      <c r="C51" s="223"/>
-      <c r="D51" s="223"/>
-      <c r="E51" s="223"/>
-      <c r="F51" s="236"/>
-      <c r="G51" s="236"/>
-      <c r="H51" s="242"/>
-      <c r="I51" s="243"/>
-      <c r="J51" s="243"/>
-      <c r="K51" s="244"/>
-      <c r="L51" s="237"/>
-      <c r="M51" s="237"/>
-      <c r="N51" s="237"/>
-      <c r="O51" s="234"/>
-      <c r="P51" s="235"/>
+      <c r="C51" s="239"/>
+      <c r="D51" s="239"/>
+      <c r="E51" s="239"/>
+      <c r="F51" s="253"/>
+      <c r="G51" s="253"/>
+      <c r="H51" s="244"/>
+      <c r="I51" s="245"/>
+      <c r="J51" s="245"/>
+      <c r="K51" s="246"/>
+      <c r="L51" s="250"/>
+      <c r="M51" s="250"/>
+      <c r="N51" s="250"/>
+      <c r="O51" s="251"/>
+      <c r="P51" s="252"/>
       <c r="Q51" s="63"/>
       <c r="R51" s="67"/>
     </row>
     <row r="52" spans="1:18" s="61" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="272"/>
+      <c r="A52" s="217"/>
       <c r="B52" s="71"/>
-      <c r="C52" s="223"/>
-      <c r="D52" s="223"/>
-      <c r="E52" s="223"/>
-      <c r="F52" s="224"/>
-      <c r="G52" s="224"/>
-      <c r="H52" s="245"/>
-      <c r="I52" s="246"/>
-      <c r="J52" s="246"/>
-      <c r="K52" s="247"/>
-      <c r="L52" s="225"/>
-      <c r="M52" s="225"/>
-      <c r="N52" s="225"/>
-      <c r="O52" s="226"/>
-      <c r="P52" s="227"/>
+      <c r="C52" s="239"/>
+      <c r="D52" s="239"/>
+      <c r="E52" s="239"/>
+      <c r="F52" s="256"/>
+      <c r="G52" s="256"/>
+      <c r="H52" s="247"/>
+      <c r="I52" s="248"/>
+      <c r="J52" s="248"/>
+      <c r="K52" s="249"/>
+      <c r="L52" s="257"/>
+      <c r="M52" s="257"/>
+      <c r="N52" s="257"/>
+      <c r="O52" s="258"/>
+      <c r="P52" s="259"/>
       <c r="Q52" s="72"/>
       <c r="R52" s="73"/>
     </row>
     <row r="53" spans="1:18" s="61" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="272"/>
+      <c r="A53" s="217"/>
       <c r="B53" s="74"/>
-      <c r="C53" s="228" t="s">
+      <c r="C53" s="260" t="s">
         <v>80</v>
       </c>
-      <c r="D53" s="228"/>
-      <c r="E53" s="228"/>
+      <c r="D53" s="260"/>
+      <c r="E53" s="260"/>
       <c r="F53" s="75"/>
-      <c r="G53" s="229"/>
-      <c r="H53" s="229"/>
-      <c r="I53" s="229"/>
+      <c r="G53" s="261"/>
+      <c r="H53" s="261"/>
+      <c r="I53" s="261"/>
       <c r="J53" s="76"/>
       <c r="K53" s="77"/>
       <c r="L53" s="77"/>
@@ -5916,14 +5916,14 @@
       <c r="R53" s="79"/>
     </row>
     <row r="54" spans="1:18" s="61" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="273"/>
+      <c r="A54" s="218"/>
       <c r="B54" s="80"/>
-      <c r="C54" s="230"/>
-      <c r="D54" s="230"/>
-      <c r="E54" s="230"/>
-      <c r="F54" s="230"/>
-      <c r="G54" s="231"/>
-      <c r="H54" s="231"/>
+      <c r="C54" s="262"/>
+      <c r="D54" s="262"/>
+      <c r="E54" s="262"/>
+      <c r="F54" s="262"/>
+      <c r="G54" s="263"/>
+      <c r="H54" s="263"/>
       <c r="I54" s="82"/>
       <c r="J54" s="82"/>
       <c r="K54" s="81"/>
@@ -5937,177 +5937,177 @@
     </row>
     <row r="55" spans="1:18" s="4" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="R55" s="84" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:18" s="4" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="214" t="s">
+      <c r="B57" s="264" t="s">
+        <v>81</v>
+      </c>
+      <c r="C57" s="265"/>
+      <c r="D57" s="266"/>
+      <c r="E57" s="264" t="s">
         <v>82</v>
       </c>
-      <c r="C57" s="215"/>
-      <c r="D57" s="216"/>
-      <c r="E57" s="214" t="s">
+      <c r="F57" s="265"/>
+      <c r="G57" s="266"/>
+      <c r="H57" s="264" t="s">
         <v>83</v>
       </c>
-      <c r="F57" s="215"/>
-      <c r="G57" s="216"/>
-      <c r="H57" s="214" t="s">
+      <c r="I57" s="265"/>
+      <c r="J57" s="266"/>
+      <c r="K57" s="264" t="s">
         <v>84</v>
       </c>
-      <c r="I57" s="215"/>
-      <c r="J57" s="216"/>
-      <c r="K57" s="214" t="s">
+      <c r="L57" s="265"/>
+      <c r="M57" s="266"/>
+      <c r="N57" s="264" t="s">
         <v>85</v>
       </c>
-      <c r="L57" s="215"/>
-      <c r="M57" s="216"/>
-      <c r="N57" s="214" t="s">
-        <v>86</v>
-      </c>
-      <c r="O57" s="215"/>
-      <c r="P57" s="216"/>
+      <c r="O57" s="265"/>
+      <c r="P57" s="266"/>
     </row>
     <row r="58" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="217"/>
-      <c r="C58" s="218"/>
-      <c r="D58" s="219"/>
-      <c r="E58" s="217"/>
-      <c r="F58" s="218"/>
-      <c r="G58" s="219"/>
-      <c r="H58" s="217"/>
-      <c r="I58" s="218"/>
-      <c r="J58" s="219"/>
-      <c r="K58" s="217"/>
-      <c r="L58" s="218"/>
-      <c r="M58" s="219"/>
-      <c r="N58" s="217"/>
-      <c r="O58" s="218"/>
-      <c r="P58" s="219"/>
+      <c r="B58" s="267"/>
+      <c r="C58" s="268"/>
+      <c r="D58" s="269"/>
+      <c r="E58" s="267"/>
+      <c r="F58" s="268"/>
+      <c r="G58" s="269"/>
+      <c r="H58" s="267"/>
+      <c r="I58" s="268"/>
+      <c r="J58" s="269"/>
+      <c r="K58" s="267"/>
+      <c r="L58" s="268"/>
+      <c r="M58" s="269"/>
+      <c r="N58" s="267"/>
+      <c r="O58" s="268"/>
+      <c r="P58" s="269"/>
     </row>
     <row r="59" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="220"/>
-      <c r="C59" s="221"/>
-      <c r="D59" s="222"/>
-      <c r="E59" s="220"/>
-      <c r="F59" s="221"/>
-      <c r="G59" s="222"/>
-      <c r="H59" s="220"/>
-      <c r="I59" s="221"/>
-      <c r="J59" s="222"/>
-      <c r="K59" s="220"/>
-      <c r="L59" s="221"/>
-      <c r="M59" s="222"/>
-      <c r="N59" s="220"/>
-      <c r="O59" s="221"/>
-      <c r="P59" s="222"/>
+      <c r="B59" s="270"/>
+      <c r="C59" s="271"/>
+      <c r="D59" s="272"/>
+      <c r="E59" s="270"/>
+      <c r="F59" s="271"/>
+      <c r="G59" s="272"/>
+      <c r="H59" s="270"/>
+      <c r="I59" s="271"/>
+      <c r="J59" s="272"/>
+      <c r="K59" s="270"/>
+      <c r="L59" s="271"/>
+      <c r="M59" s="272"/>
+      <c r="N59" s="270"/>
+      <c r="O59" s="271"/>
+      <c r="P59" s="272"/>
     </row>
     <row r="60" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="85" t="s">
+        <v>86</v>
+      </c>
+      <c r="C60" s="273"/>
+      <c r="D60" s="274"/>
+      <c r="E60" s="85" t="s">
+        <v>86</v>
+      </c>
+      <c r="F60" s="273"/>
+      <c r="G60" s="274"/>
+      <c r="H60" s="85" t="s">
+        <v>86</v>
+      </c>
+      <c r="I60" s="273"/>
+      <c r="J60" s="274"/>
+      <c r="K60" s="85" t="s">
+        <v>86</v>
+      </c>
+      <c r="L60" s="273"/>
+      <c r="M60" s="274"/>
+      <c r="N60" s="85" t="s">
+        <v>86</v>
+      </c>
+      <c r="O60" s="273"/>
+      <c r="P60" s="274"/>
+    </row>
+    <row r="61" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="264" t="s">
         <v>87</v>
       </c>
-      <c r="C60" s="212"/>
-      <c r="D60" s="213"/>
-      <c r="E60" s="85" t="s">
+      <c r="C61" s="265"/>
+      <c r="D61" s="266"/>
+      <c r="E61" s="264" t="s">
+        <v>88</v>
+      </c>
+      <c r="F61" s="265"/>
+      <c r="G61" s="266"/>
+      <c r="H61" s="264" t="s">
         <v>87</v>
       </c>
-      <c r="F60" s="212"/>
-      <c r="G60" s="213"/>
-      <c r="H60" s="85" t="s">
-        <v>87</v>
-      </c>
-      <c r="I60" s="212"/>
-      <c r="J60" s="213"/>
-      <c r="K60" s="85" t="s">
-        <v>87</v>
-      </c>
-      <c r="L60" s="212"/>
-      <c r="M60" s="213"/>
-      <c r="N60" s="85" t="s">
-        <v>87</v>
-      </c>
-      <c r="O60" s="212"/>
-      <c r="P60" s="213"/>
-    </row>
-    <row r="61" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="214" t="s">
+      <c r="I61" s="265"/>
+      <c r="J61" s="266"/>
+      <c r="K61" s="264" t="s">
         <v>88</v>
       </c>
-      <c r="C61" s="215"/>
-      <c r="D61" s="216"/>
-      <c r="E61" s="214" t="s">
-        <v>89</v>
-      </c>
-      <c r="F61" s="215"/>
-      <c r="G61" s="216"/>
-      <c r="H61" s="214" t="s">
+      <c r="L61" s="265"/>
+      <c r="M61" s="266"/>
+      <c r="N61" s="264" t="s">
         <v>88</v>
       </c>
-      <c r="I61" s="215"/>
-      <c r="J61" s="216"/>
-      <c r="K61" s="214" t="s">
-        <v>89</v>
-      </c>
-      <c r="L61" s="215"/>
-      <c r="M61" s="216"/>
-      <c r="N61" s="214" t="s">
-        <v>89</v>
-      </c>
-      <c r="O61" s="215"/>
-      <c r="P61" s="216"/>
+      <c r="O61" s="265"/>
+      <c r="P61" s="266"/>
     </row>
     <row r="62" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="63" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="214" t="s">
+      <c r="B63" s="264" t="s">
+        <v>89</v>
+      </c>
+      <c r="C63" s="265"/>
+      <c r="D63" s="266"/>
+      <c r="E63" s="264" t="s">
         <v>90</v>
       </c>
-      <c r="C63" s="215"/>
-      <c r="D63" s="216"/>
-      <c r="E63" s="214" t="s">
-        <v>91</v>
-      </c>
-      <c r="F63" s="215"/>
-      <c r="G63" s="216"/>
+      <c r="F63" s="265"/>
+      <c r="G63" s="266"/>
     </row>
     <row r="64" spans="1:18" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="217"/>
-      <c r="C64" s="218"/>
-      <c r="D64" s="219"/>
-      <c r="E64" s="217"/>
-      <c r="F64" s="218"/>
-      <c r="G64" s="219"/>
+      <c r="B64" s="267"/>
+      <c r="C64" s="268"/>
+      <c r="D64" s="269"/>
+      <c r="E64" s="267"/>
+      <c r="F64" s="268"/>
+      <c r="G64" s="269"/>
     </row>
     <row r="65" spans="2:7" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="220"/>
-      <c r="C65" s="221"/>
-      <c r="D65" s="222"/>
-      <c r="E65" s="220"/>
-      <c r="F65" s="221"/>
-      <c r="G65" s="222"/>
+      <c r="B65" s="270"/>
+      <c r="C65" s="271"/>
+      <c r="D65" s="272"/>
+      <c r="E65" s="270"/>
+      <c r="F65" s="271"/>
+      <c r="G65" s="272"/>
     </row>
     <row r="66" spans="2:7" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="85" t="s">
-        <v>87</v>
-      </c>
-      <c r="C66" s="212"/>
-      <c r="D66" s="213"/>
+        <v>86</v>
+      </c>
+      <c r="C66" s="273"/>
+      <c r="D66" s="274"/>
       <c r="E66" s="85" t="s">
-        <v>87</v>
-      </c>
-      <c r="F66" s="212"/>
-      <c r="G66" s="213"/>
+        <v>86</v>
+      </c>
+      <c r="F66" s="273"/>
+      <c r="G66" s="274"/>
     </row>
     <row r="67" spans="2:7" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="214" t="s">
-        <v>89</v>
-      </c>
-      <c r="C67" s="215"/>
-      <c r="D67" s="216"/>
-      <c r="E67" s="214" t="s">
-        <v>89</v>
-      </c>
-      <c r="F67" s="215"/>
-      <c r="G67" s="216"/>
+      <c r="B67" s="264" t="s">
+        <v>88</v>
+      </c>
+      <c r="C67" s="265"/>
+      <c r="D67" s="266"/>
+      <c r="E67" s="264" t="s">
+        <v>88</v>
+      </c>
+      <c r="F67" s="265"/>
+      <c r="G67" s="266"/>
     </row>
     <row r="68" spans="2:7" s="4" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="69" spans="2:7" s="4" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6604,6 +6604,103 @@
     <row r="560" s="86" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="121">
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="B67:D67"/>
+    <mergeCell ref="E67:G67"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="N61:P61"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="E63:G63"/>
+    <mergeCell ref="B64:D65"/>
+    <mergeCell ref="E64:G65"/>
+    <mergeCell ref="B58:D59"/>
+    <mergeCell ref="E58:G59"/>
+    <mergeCell ref="H58:J59"/>
+    <mergeCell ref="K58:M59"/>
+    <mergeCell ref="N58:P59"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="L60:M60"/>
+    <mergeCell ref="O60:P60"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="L52:N52"/>
+    <mergeCell ref="O52:P52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="G53:I53"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="G54:H54"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="H57:J57"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="N57:P57"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="L49:N49"/>
+    <mergeCell ref="O49:P49"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="L50:N50"/>
+    <mergeCell ref="O50:P50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="L51:N51"/>
+    <mergeCell ref="O51:P51"/>
+    <mergeCell ref="O46:P46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="L47:N47"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="L48:N48"/>
+    <mergeCell ref="O48:P48"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="H41:K52"/>
+    <mergeCell ref="L41:N41"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="L42:N42"/>
+    <mergeCell ref="O42:P42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="L43:N43"/>
+    <mergeCell ref="O43:P43"/>
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="L44:N44"/>
+    <mergeCell ref="O44:P44"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="L45:N45"/>
+    <mergeCell ref="O45:P45"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="C28:Q28"/>
+    <mergeCell ref="C32:Q32"/>
+    <mergeCell ref="C33:Q33"/>
+    <mergeCell ref="C34:Q34"/>
+    <mergeCell ref="C35:Q35"/>
+    <mergeCell ref="C36:Q36"/>
+    <mergeCell ref="B38:R38"/>
+    <mergeCell ref="C39:E40"/>
+    <mergeCell ref="F39:G40"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="L39:N40"/>
+    <mergeCell ref="O39:P40"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="H40:K40"/>
+    <mergeCell ref="Q39:Q40"/>
+    <mergeCell ref="R39:R40"/>
     <mergeCell ref="L1:R1"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="G3:J3"/>
@@ -6628,103 +6725,6 @@
     <mergeCell ref="C25:Q25"/>
     <mergeCell ref="C26:Q26"/>
     <mergeCell ref="C27:Q27"/>
-    <mergeCell ref="C28:Q28"/>
-    <mergeCell ref="C32:Q32"/>
-    <mergeCell ref="C33:Q33"/>
-    <mergeCell ref="C34:Q34"/>
-    <mergeCell ref="C35:Q35"/>
-    <mergeCell ref="C36:Q36"/>
-    <mergeCell ref="B38:R38"/>
-    <mergeCell ref="C39:E40"/>
-    <mergeCell ref="F39:G40"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="L39:N40"/>
-    <mergeCell ref="O39:P40"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="H40:K40"/>
-    <mergeCell ref="Q39:Q40"/>
-    <mergeCell ref="R39:R40"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="H41:K52"/>
-    <mergeCell ref="L41:N41"/>
-    <mergeCell ref="O41:P41"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="L42:N42"/>
-    <mergeCell ref="O42:P42"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="L43:N43"/>
-    <mergeCell ref="O43:P43"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="L44:N44"/>
-    <mergeCell ref="O44:P44"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="L45:N45"/>
-    <mergeCell ref="O45:P45"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="O46:P46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="O47:P47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="L48:N48"/>
-    <mergeCell ref="O48:P48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="L49:N49"/>
-    <mergeCell ref="O49:P49"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="L50:N50"/>
-    <mergeCell ref="O50:P50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="L51:N51"/>
-    <mergeCell ref="O51:P51"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="L52:N52"/>
-    <mergeCell ref="O52:P52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="G53:I53"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="G54:H54"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="H57:J57"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="N57:P57"/>
-    <mergeCell ref="B58:D59"/>
-    <mergeCell ref="E58:G59"/>
-    <mergeCell ref="H58:J59"/>
-    <mergeCell ref="K58:M59"/>
-    <mergeCell ref="N58:P59"/>
-    <mergeCell ref="C60:D60"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="L60:M60"/>
-    <mergeCell ref="O60:P60"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="B67:D67"/>
-    <mergeCell ref="E67:G67"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="N61:P61"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="E63:G63"/>
-    <mergeCell ref="B64:D65"/>
-    <mergeCell ref="E64:G65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>